<commit_message>
Update soccer trades 2026-07-31 12:03:07 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/EFL Cup/trades.xlsx
+++ b/data/sxbet/ligas/EFL Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:V4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,77 +546,77 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1.46</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>L19298738</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785346230</t>
+          <t>1785497246</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2.173913</t>
+          <t>5.97619</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,110 +643,222 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>1785346230</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>2.173913</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>0xea48d5fe72de69b25067fdb4fdaf1d08ce7262ad75f6855864d3a656da39b313</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>1.46</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>L19298738</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>1785345250</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>1785592800</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>2.173913</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-31 21:02:49 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/EFL Cup/trades.xlsx
+++ b/data/sxbet/ligas/EFL Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:V5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2.51</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.605</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785497246</t>
+          <t>1785512959</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>5.97619</t>
+          <t>1.652893</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,12 +658,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.51</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785346230</t>
+          <t>1785497246</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2.173913</t>
+          <t>5.97619</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,110 +755,222 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1785346230</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>2.173913</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>0xea48d5fe72de69b25067fdb4fdaf1d08ce7262ad75f6855864d3a656da39b313</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>1.46</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>L19298738</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
         <is>
           <t>1785345250</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>1785592800</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>2.173913</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-01 10:02:57 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/EFL Cup/trades.xlsx
+++ b/data/sxbet/ligas/EFL Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
+          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.605</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298738</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785512959</t>
+          <t>1785577998</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1785592800</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.652893</t>
+          <t>59.143969</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,12 +658,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2.51</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -673,32 +673,32 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785497246</t>
+          <t>1785577962</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>5.97619</t>
+          <t>82.758621</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,12 +755,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -770,12 +770,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>1.3225</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -785,32 +785,32 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785346230</t>
+          <t>1785577789</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2.173913</t>
+          <t>3.534884</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,110 +867,2118 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>18.99909</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.3213</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>1785577788</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>59.141136</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1.96</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.3213</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>1785576753</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>6.101167</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2.81824</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1785576753</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>8.807</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>20.06</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1785576072</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>62.6875</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>22.07</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>1785575036</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>68.96875</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1.16</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>1785574569</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>3.625</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>19.25059</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1785574187</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>60.158094</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>20.96</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>1785574186</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>65.5</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2.69</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>1785574186</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>8.40625</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2.21</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>1785574073</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>6.90625</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>1785573852</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>6.25</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2.01</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1.3213</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>1785570690</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>6.256809</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>1785570471</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>31.25</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>19.72999</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1.6062</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>1785569792</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>32.544313</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>1785569076</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>6.59375</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1.605</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>York City</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>York City vs Crawley Town</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>York City</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Crawley Town</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>L19299060</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>1785512959</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>1785781800</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>1.652893</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>1785497246</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>5.97619</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>1785346230</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>2.173913</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>0xea48d5fe72de69b25067fdb4fdaf1d08ce7262ad75f6855864d3a656da39b313</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>1.46</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>L19298738</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
         <is>
           <t>1785345250</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="S23" t="inlineStr">
         <is>
           <t>1785592800</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="T23" t="inlineStr">
         <is>
           <t>2.173913</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="U23" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="V23" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-01 17:02:47 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/EFL Cup/trades.xlsx
+++ b/data/sxbet/ligas/EFL Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:V41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
+          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>23.26</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785577998</t>
+          <t>1785597225</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>59.143969</t>
+          <t>53.62536</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
+          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,12 +658,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785577962</t>
+          <t>1785595661</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>82.758621</t>
+          <t>3.11284</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,7 +755,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
+          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -770,12 +770,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.3225</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785577789</t>
+          <t>1785594340</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>3.534884</t>
+          <t>27.777778</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,7 +867,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
+          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -882,12 +882,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>18.99909</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785577788</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>59.141136</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,7 +979,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
+          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -994,12 +994,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>6.101167</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1091,7 +1091,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
+          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1106,12 +1106,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.81824</t>
+          <t>25.04</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.385</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785593611</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>8.807</t>
+          <t>65.038961</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1203,7 +1203,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
+          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1218,12 +1218,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>20.06</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.2375</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785576072</t>
+          <t>1785593186</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>62.6875</t>
+          <t>49.263158</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1315,7 +1315,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
+          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1330,12 +1330,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>22.07</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785575036</t>
+          <t>1785592744</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>68.96875</t>
+          <t>7.088608</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
+          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1442,12 +1442,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>3.59</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785574569</t>
+          <t>1785592658</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>3.625</t>
+          <t>9.088608</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1539,7 +1539,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
+          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1554,12 +1554,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>19.25059</t>
+          <t>22.05</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785574187</t>
+          <t>1785592637</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>60.158094</t>
+          <t>55.822785</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1651,7 +1651,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
+          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1659,19 +1659,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>20.96</t>
+          <t>36.31948</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1679,11 +1675,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1706,7 +1698,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1736,7 +1728,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785589857</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1746,7 +1738,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>65.5</t>
+          <t>58.816972</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1763,7 +1755,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
+          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1771,19 +1763,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2.69</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1791,11 +1779,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1818,7 +1802,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1848,7 +1832,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785589600</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1858,7 +1842,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>8.40625</t>
+          <t>6.54251</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1875,7 +1859,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
+          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1883,19 +1867,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>18.36999</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.615</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1903,11 +1883,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1930,7 +1906,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1960,7 +1936,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785574073</t>
+          <t>1785589491</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1970,7 +1946,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>6.90625</t>
+          <t>29.869902</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1987,7 +1963,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
+          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1995,19 +1971,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>18.54999</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2015,11 +1987,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2042,7 +2010,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2072,7 +2040,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785573852</t>
+          <t>1785588508</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2082,7 +2050,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>6.25</t>
+          <t>30.597922</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2099,12 +2067,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
+          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2114,12 +2082,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>15.21</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.2812</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2129,7 +2097,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2154,7 +2122,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2184,7 +2152,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785570690</t>
+          <t>1785587700</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2194,7 +2162,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>6.256809</t>
+          <t>54.08</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2211,7 +2179,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
+          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2219,19 +2187,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>6.44999</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.7237</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2239,11 +2203,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2266,7 +2226,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2296,7 +2256,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785570471</t>
+          <t>1785585922</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2306,7 +2266,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>31.25</t>
+          <t>8.911903</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2323,7 +2283,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
+          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2334,12 +2294,12 @@
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>19.72999</t>
+          <t>3.26</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2370,7 +2330,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2400,7 +2360,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785569792</t>
+          <t>1785579524</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2410,7 +2370,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>32.544313</t>
+          <t>4.519931</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2427,7 +2387,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
+          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2435,19 +2395,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>3.61999</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2455,11 +2411,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2482,7 +2434,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2512,7 +2464,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785569076</t>
+          <t>1785579365</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2522,7 +2474,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>6.59375</t>
+          <t>5.01905</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2539,12 +2491,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
+          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2554,12 +2506,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.605</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2569,7 +2521,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2579,27 +2531,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298738</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2624,17 +2576,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785512959</t>
+          <t>1785577998</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1785592800</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1.652893</t>
+          <t>59.143969</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2651,12 +2603,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2666,12 +2618,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2.51</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2681,32 +2633,32 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2736,7 +2688,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785497246</t>
+          <t>1785577962</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2746,7 +2698,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>5.97619</t>
+          <t>82.758621</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2763,12 +2715,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2778,12 +2730,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>1.3225</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2793,32 +2745,32 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2848,7 +2800,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785346230</t>
+          <t>1785577789</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2858,7 +2810,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2.173913</t>
+          <t>3.534884</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2875,110 +2827,2118 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>18.99909</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1.3213</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>1785577788</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>59.141136</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>1.96</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1.3213</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>1785576753</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>6.101167</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2.81824</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>1785576753</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>8.807</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>20.06</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>1785576072</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>62.6875</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>22.07</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>1785575036</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>68.96875</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>1.16</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>1785574569</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>3.625</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>19.25059</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>1785574187</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>60.158094</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>20.96</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>1785574186</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>65.5</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2.69</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>1785574186</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>8.40625</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2.21</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>1785574073</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>6.90625</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>1785573852</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>6.25</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2.01</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>1.3213</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>1785570690</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>6.256809</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>1785570471</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>31.25</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>19.72999</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1.6062</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>1785569792</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>32.544313</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>1785569076</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>6.59375</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>1.605</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>York City</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>York City vs Crawley Town</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>York City</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Crawley Town</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>L19299060</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>1785512959</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>1785781800</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>1.652893</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>1785497246</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>5.97619</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>1785346230</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>2.173913</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>0xea48d5fe72de69b25067fdb4fdaf1d08ce7262ad75f6855864d3a656da39b313</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>1.46</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="M41" t="inlineStr">
         <is>
           <t>L19298738</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
         <is>
           <t>1785345250</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr">
+      <c r="S41" t="inlineStr">
         <is>
           <t>1785592800</t>
         </is>
       </c>
-      <c r="T23" t="inlineStr">
+      <c r="T41" t="inlineStr">
         <is>
           <t>2.173913</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="U41" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr">
+      <c r="V41" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-03 04:02:08 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/EFL Cup/trades.xlsx
+++ b/data/sxbet/ligas/EFL Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V41"/>
+  <dimension ref="A1:V42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
+          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>23.26</t>
+          <t>3.99987</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.4338</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785597225</t>
+          <t>1785729635</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>53.62536</t>
+          <t>16.079879</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
+          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -658,12 +658,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>23.26</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -673,32 +673,32 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785595661</t>
+          <t>1785597225</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>3.11284</t>
+          <t>53.62536</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,7 +755,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
+          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -770,12 +770,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785594340</t>
+          <t>1785595661</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>27.777778</t>
+          <t>3.11284</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,7 +867,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
+          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785593884</t>
+          <t>1785594340</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>27.777778</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,7 +979,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
+          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1091,7 +1091,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
+          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1106,12 +1106,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>25.04</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.385</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785593611</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>65.038961</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1203,7 +1203,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
+          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1218,12 +1218,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>25.04</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.2375</t>
+          <t>1.385</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785593186</t>
+          <t>1785593611</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>49.263158</t>
+          <t>65.038961</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1315,7 +1315,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
+          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1330,12 +1330,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.2375</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1345,32 +1345,32 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785592744</t>
+          <t>1785593186</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>7.088608</t>
+          <t>49.263158</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
+          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.59</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785592658</t>
+          <t>1785592744</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>9.088608</t>
+          <t>7.088608</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1539,7 +1539,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
+          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>22.05</t>
+          <t>3.59</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785592637</t>
+          <t>1785592658</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>55.822785</t>
+          <t>9.088608</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1651,7 +1651,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
+          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1659,15 +1659,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>36.31948</t>
+          <t>22.05</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1675,7 +1679,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1728,7 +1736,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785589857</t>
+          <t>1785592637</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1738,7 +1746,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>58.816972</t>
+          <t>55.822785</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1755,7 +1763,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
+          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1766,7 +1774,7 @@
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>36.31948</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1832,7 +1840,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785589600</t>
+          <t>1785589857</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1842,7 +1850,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>6.54251</t>
+          <t>58.816972</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1859,7 +1867,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
+          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1870,12 +1878,12 @@
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>18.36999</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.615</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1936,7 +1944,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785589491</t>
+          <t>1785589600</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1946,7 +1954,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>29.869902</t>
+          <t>6.54251</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1963,7 +1971,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
+          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1974,12 +1982,12 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>18.54999</t>
+          <t>18.36999</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.615</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2040,7 +2048,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785588508</t>
+          <t>1785589491</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2050,7 +2058,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>30.597922</t>
+          <t>29.869902</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2067,27 +2075,23 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
+          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>15.21</t>
+          <t>18.54999</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2095,11 +2099,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2122,7 +2122,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785587700</t>
+          <t>1785588508</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>54.08</t>
+          <t>30.597922</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2179,23 +2179,27 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
+          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>6.44999</t>
+          <t>15.21</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.7237</t>
+          <t>1.2812</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2203,7 +2207,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2256,7 +2264,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785585922</t>
+          <t>1785587700</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2266,7 +2274,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>8.911903</t>
+          <t>54.08</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2283,7 +2291,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
+          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2294,12 +2302,12 @@
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.26</t>
+          <t>6.44999</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.7212</t>
+          <t>1.7237</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2360,7 +2368,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785579524</t>
+          <t>1785585922</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2370,7 +2378,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>4.519931</t>
+          <t>8.911903</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2387,7 +2395,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
+          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2398,7 +2406,7 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.61999</t>
+          <t>3.26</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2464,7 +2472,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785579365</t>
+          <t>1785579524</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2474,7 +2482,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>5.01905</t>
+          <t>4.519931</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2491,27 +2499,23 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
+          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>3.61999</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2519,11 +2523,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785577998</t>
+          <t>1785579365</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>59.143969</t>
+          <t>5.01905</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2603,7 +2603,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
+          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2618,12 +2618,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2658,7 +2658,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2688,7 +2688,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785577962</t>
+          <t>1785577998</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2698,7 +2698,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>82.758621</t>
+          <t>59.143969</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2715,12 +2715,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
+          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2730,12 +2730,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.3225</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2770,7 +2770,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785577789</t>
+          <t>1785577962</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>3.534884</t>
+          <t>82.758621</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2827,7 +2827,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
+          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2842,12 +2842,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>18.99909</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.3225</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785577788</t>
+          <t>1785577789</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>59.141136</t>
+          <t>3.534884</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2939,7 +2939,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
+          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>18.99909</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785577788</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>6.101167</t>
+          <t>59.141136</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3051,7 +3051,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
+          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3066,12 +3066,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2.81824</t>
+          <t>1.96</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>8.807</t>
+          <t>6.101167</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3163,7 +3163,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
+          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3178,7 +3178,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>20.06</t>
+          <t>2.81824</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785576072</t>
+          <t>1785576753</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>62.6875</t>
+          <t>8.807</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3275,7 +3275,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
+          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>22.07</t>
+          <t>20.06</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785575036</t>
+          <t>1785576072</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>68.96875</t>
+          <t>62.6875</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3387,7 +3387,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
+          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>22.07</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785574569</t>
+          <t>1785575036</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>3.625</t>
+          <t>68.96875</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3499,7 +3499,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
+          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>19.25059</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -3584,7 +3584,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785574187</t>
+          <t>1785574569</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>60.158094</t>
+          <t>3.625</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3611,7 +3611,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
+          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>20.96</t>
+          <t>19.25059</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785574187</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>65.5</t>
+          <t>60.158094</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3723,7 +3723,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
+          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3738,7 +3738,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2.69</t>
+          <t>20.96</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>8.40625</t>
+          <t>65.5</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3835,7 +3835,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
+          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3850,7 +3850,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>2.69</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785574073</t>
+          <t>1785574186</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3930,7 +3930,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>6.90625</t>
+          <t>8.40625</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
+          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -4032,7 +4032,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785573852</t>
+          <t>1785574073</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -4042,7 +4042,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>6.25</t>
+          <t>6.90625</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4059,7 +4059,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
+          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4074,12 +4074,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4144,7 +4144,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785570690</t>
+          <t>1785573852</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4154,7 +4154,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>6.256809</t>
+          <t>6.25</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4171,7 +4171,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
+          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4186,12 +4186,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2.01</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4256,7 +4256,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785570471</t>
+          <t>1785570690</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>31.25</t>
+          <t>6.256809</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4283,7 +4283,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
+          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4291,15 +4291,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>19.72999</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4307,7 +4311,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4330,7 +4338,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4360,7 +4368,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785569792</t>
+          <t>1785570471</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4370,7 +4378,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>32.544313</t>
+          <t>31.25</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4387,7 +4395,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
+          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4395,19 +4403,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>19.72999</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4415,11 +4419,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4442,7 +4442,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4472,7 +4472,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1785569076</t>
+          <t>1785569792</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>6.59375</t>
+          <t>32.544313</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4499,12 +4499,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
+          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4514,12 +4514,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.11</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.605</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4529,7 +4529,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -4539,27 +4539,27 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298738</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -4584,17 +4584,17 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785512959</t>
+          <t>1785569076</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1785592800</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>1.652893</t>
+          <t>6.59375</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4611,12 +4611,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4626,12 +4626,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2.51</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.605</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4641,7 +4641,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -4651,27 +4651,27 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -4696,17 +4696,17 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1785497246</t>
+          <t>1785512959</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>5.97619</t>
+          <t>1.652893</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4723,12 +4723,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -4738,12 +4738,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.51</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4808,7 +4808,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1785346230</t>
+          <t>1785497246</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4818,7 +4818,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>2.173913</t>
+          <t>5.97619</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4835,110 +4835,222 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>1785346230</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>2.173913</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>0xea48d5fe72de69b25067fdb4fdaf1d08ce7262ad75f6855864d3a656da39b313</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>1.46</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H42" t="inlineStr">
         <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="M42" t="inlineStr">
         <is>
           <t>L19298738</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P41" t="inlineStr">
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R41" t="inlineStr">
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
         <is>
           <t>1785345250</t>
         </is>
       </c>
-      <c r="S41" t="inlineStr">
+      <c r="S42" t="inlineStr">
         <is>
           <t>1785592800</t>
         </is>
       </c>
-      <c r="T41" t="inlineStr">
+      <c r="T42" t="inlineStr">
         <is>
           <t>2.173913</t>
         </is>
       </c>
-      <c r="U41" t="inlineStr">
+      <c r="U42" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V41" t="inlineStr">
+      <c r="V42" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-03 05:02:31 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/EFL Cup/trades.xlsx
+++ b/data/sxbet/ligas/EFL Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V42"/>
+  <dimension ref="A1:V43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
+          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3.99987</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.2475</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785729635</t>
+          <t>1785729810</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>16.079879</t>
+          <t>4.040404</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
+          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -658,12 +658,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>23.26</t>
+          <t>3.99987</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.4338</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -683,27 +683,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -728,17 +728,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785597225</t>
+          <t>1785729635</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>53.62536</t>
+          <t>16.079879</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,7 +755,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
+          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -770,12 +770,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>23.26</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -785,32 +785,32 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785595661</t>
+          <t>1785597225</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>3.11284</t>
+          <t>53.62536</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,7 +867,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
+          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -882,12 +882,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785594340</t>
+          <t>1785595661</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>27.777778</t>
+          <t>3.11284</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,7 +979,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
+          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785593884</t>
+          <t>1785594340</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>27.777778</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1091,7 +1091,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
+          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1203,7 +1203,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
+          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1218,12 +1218,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>25.04</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.385</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785593611</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>65.038961</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1315,7 +1315,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
+          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1330,12 +1330,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>25.04</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.2375</t>
+          <t>1.385</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785593186</t>
+          <t>1785593611</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>49.263158</t>
+          <t>65.038961</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
+          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1442,12 +1442,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.2375</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1457,32 +1457,32 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785592744</t>
+          <t>1785593186</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>7.088608</t>
+          <t>49.263158</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1539,7 +1539,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
+          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3.59</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785592658</t>
+          <t>1785592744</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>9.088608</t>
+          <t>7.088608</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1651,7 +1651,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
+          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>22.05</t>
+          <t>3.59</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1736,7 +1736,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785592637</t>
+          <t>1785592658</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>55.822785</t>
+          <t>9.088608</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1763,7 +1763,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
+          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1771,15 +1771,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>36.31948</t>
+          <t>22.05</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1787,7 +1791,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1840,7 +1848,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785589857</t>
+          <t>1785592637</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1850,7 +1858,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>58.816972</t>
+          <t>55.822785</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1867,7 +1875,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
+          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1878,7 +1886,7 @@
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>36.31948</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1944,7 +1952,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785589600</t>
+          <t>1785589857</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1954,7 +1962,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>6.54251</t>
+          <t>58.816972</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1971,7 +1979,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
+          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1982,12 +1990,12 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>18.36999</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.615</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2048,7 +2056,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785589491</t>
+          <t>1785589600</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2058,7 +2066,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>29.869902</t>
+          <t>6.54251</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2075,7 +2083,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
+          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2086,12 +2094,12 @@
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>18.54999</t>
+          <t>18.36999</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.615</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2152,7 +2160,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785588508</t>
+          <t>1785589491</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2162,7 +2170,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>30.597922</t>
+          <t>29.869902</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2179,27 +2187,23 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
+          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>15.21</t>
+          <t>18.54999</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2207,11 +2211,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785587700</t>
+          <t>1785588508</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>54.08</t>
+          <t>30.597922</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2291,23 +2291,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
+          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6.44999</t>
+          <t>15.21</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.7237</t>
+          <t>1.2812</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2315,7 +2319,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2368,7 +2376,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785585922</t>
+          <t>1785587700</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2378,7 +2386,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>8.911903</t>
+          <t>54.08</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2395,7 +2403,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
+          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2406,12 +2414,12 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.26</t>
+          <t>6.44999</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.7212</t>
+          <t>1.7237</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2472,7 +2480,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785579524</t>
+          <t>1785585922</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2482,7 +2490,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>4.519931</t>
+          <t>8.911903</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2499,7 +2507,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
+          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2510,7 +2518,7 @@
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>3.61999</t>
+          <t>3.26</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2576,7 +2584,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785579365</t>
+          <t>1785579524</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2586,7 +2594,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>5.01905</t>
+          <t>4.519931</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2603,27 +2611,23 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
+          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>3.61999</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2631,11 +2635,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2658,7 +2658,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2688,7 +2688,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785577998</t>
+          <t>1785579365</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2698,7 +2698,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>59.143969</t>
+          <t>5.01905</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2715,7 +2715,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
+          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2730,12 +2730,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2770,7 +2770,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785577962</t>
+          <t>1785577998</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>82.758621</t>
+          <t>59.143969</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2827,12 +2827,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
+          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2842,12 +2842,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.3225</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2882,7 +2882,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785577789</t>
+          <t>1785577962</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>3.534884</t>
+          <t>82.758621</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2939,7 +2939,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
+          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2954,12 +2954,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>18.99909</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.3225</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785577788</t>
+          <t>1785577789</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>59.141136</t>
+          <t>3.534884</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3051,7 +3051,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
+          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3066,7 +3066,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>18.99909</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785577788</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>6.101167</t>
+          <t>59.141136</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3163,7 +3163,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
+          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3178,12 +3178,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2.81824</t>
+          <t>1.96</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>8.807</t>
+          <t>6.101167</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3275,7 +3275,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
+          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>20.06</t>
+          <t>2.81824</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785576072</t>
+          <t>1785576753</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>62.6875</t>
+          <t>8.807</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3387,7 +3387,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
+          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>22.07</t>
+          <t>20.06</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785575036</t>
+          <t>1785576072</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>68.96875</t>
+          <t>62.6875</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3499,7 +3499,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
+          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>22.07</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -3584,7 +3584,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785574569</t>
+          <t>1785575036</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>3.625</t>
+          <t>68.96875</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3611,7 +3611,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
+          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>19.25059</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785574187</t>
+          <t>1785574569</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>60.158094</t>
+          <t>3.625</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3723,7 +3723,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
+          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3738,7 +3738,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>20.96</t>
+          <t>19.25059</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785574187</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>65.5</t>
+          <t>60.158094</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3835,7 +3835,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
+          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3850,7 +3850,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2.69</t>
+          <t>20.96</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3930,7 +3930,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>8.40625</t>
+          <t>65.5</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
+          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>2.69</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -4032,7 +4032,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785574073</t>
+          <t>1785574186</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -4042,7 +4042,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>6.90625</t>
+          <t>8.40625</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4059,7 +4059,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
+          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4074,7 +4074,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -4144,7 +4144,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785573852</t>
+          <t>1785574073</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4154,7 +4154,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>6.25</t>
+          <t>6.90625</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4171,7 +4171,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
+          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4186,12 +4186,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4256,7 +4256,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785570690</t>
+          <t>1785573852</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>6.256809</t>
+          <t>6.25</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4283,7 +4283,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
+          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4298,12 +4298,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2.01</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785570471</t>
+          <t>1785570690</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4378,7 +4378,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>31.25</t>
+          <t>6.256809</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4395,7 +4395,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
+          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4403,15 +4403,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>19.72999</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4419,7 +4423,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4442,7 +4450,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4472,7 +4480,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1785569792</t>
+          <t>1785570471</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4482,7 +4490,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>32.544313</t>
+          <t>31.25</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4499,7 +4507,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
+          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4507,19 +4515,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>19.72999</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4527,11 +4531,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4554,7 +4554,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4584,7 +4584,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785569076</t>
+          <t>1785569792</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>6.59375</t>
+          <t>32.544313</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4611,12 +4611,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
+          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4626,12 +4626,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.11</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.605</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4641,7 +4641,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -4651,27 +4651,27 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298738</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -4696,17 +4696,17 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1785512959</t>
+          <t>1785569076</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1785592800</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1.652893</t>
+          <t>6.59375</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4723,12 +4723,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -4738,12 +4738,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2.51</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.605</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4753,7 +4753,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -4763,27 +4763,27 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -4808,17 +4808,17 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1785497246</t>
+          <t>1785512959</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>5.97619</t>
+          <t>1.652893</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4835,12 +4835,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -4850,12 +4850,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.51</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4920,7 +4920,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1785346230</t>
+          <t>1785497246</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4930,7 +4930,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>2.173913</t>
+          <t>5.97619</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4947,110 +4947,222 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>1785346230</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>2.173913</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>0xea48d5fe72de69b25067fdb4fdaf1d08ce7262ad75f6855864d3a656da39b313</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>1.46</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="M43" t="inlineStr">
         <is>
           <t>L19298738</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P42" t="inlineStr">
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R42" t="inlineStr">
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
         <is>
           <t>1785345250</t>
         </is>
       </c>
-      <c r="S42" t="inlineStr">
+      <c r="S43" t="inlineStr">
         <is>
           <t>1785592800</t>
         </is>
       </c>
-      <c r="T42" t="inlineStr">
+      <c r="T43" t="inlineStr">
         <is>
           <t>2.173913</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="U43" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V42" t="inlineStr">
+      <c r="V43" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-03 18:02:58 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/EFL Cup/trades.xlsx
+++ b/data/sxbet/ligas/EFL Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V56"/>
+  <dimension ref="A1:V57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x9b63fb9bdb0939e4fa277441c5160ae767a06c0723ae1697f56722a32c1dbbf4</t>
+          <t>0xfcba109b300bea480abe542eaa7725c7fec13f0fedc18d9991df424ad450dc90</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x095B1B11E9C470934404Ba7F04da5F79930b2504</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,39 +546,39 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.47999</t>
+          <t>14.58</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5762</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>York City vs Crawley Town</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>York City</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>York City vs Crawley Town</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>York City</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>Crawley Town</t>
@@ -586,7 +586,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0x30711e53de1ac1c4a025d48c70e4859ee55e52e5e57d10ed46259cc01bb5d46e</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785751617</t>
+          <t>1785778500</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2.568312</t>
+          <t>18.0</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x34fd96c52ca66603743b136c029d1196926b8ea965b35ad916e9e624891a3c31</t>
+          <t>0x9b63fb9bdb0939e4fa277441c5160ae767a06c0723ae1697f56722a32c1dbbf4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -651,23 +651,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2.59999</t>
+          <t>1.47999</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.6887</t>
+          <t>1.5762</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>York City</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -690,7 +698,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xb943c3d4cb1b4aebd6296b959eb4168b4f43df52a8043a9e84d184a931ac076c</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -720,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785751591</t>
+          <t>1785751617</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>3.77494</t>
+          <t>2.568312</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,39 +755,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x92e4361325da8adb7d2c64339dc80666c0b8e0d69bcdd503c9dcdc859b32e858</t>
+          <t>0x34fd96c52ca66603743b136c029d1196926b8ea965b35ad916e9e624891a3c31</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>288.19</t>
+          <t>2.59999</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.555</t>
+          <t>1.6887</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -802,7 +802,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
+          <t>0xb943c3d4cb1b4aebd6296b959eb4168b4f43df52a8043a9e84d184a931ac076c</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785746436</t>
+          <t>1785751591</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>519.261261</t>
+          <t>3.77494</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,31 +859,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x2f280a5348c67d22f499a879111a6cd14ba32c30651f4b235087504d75fcb720</t>
+          <t>0x92e4361325da8adb7d2c64339dc80666c0b8e0d69bcdd503c9dcdc859b32e858</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>288.19</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.5263</t>
+          <t>1.555</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -906,7 +914,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
+          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -936,7 +944,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785743240</t>
+          <t>1785746436</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -946,7 +954,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>9.501188</t>
+          <t>519.261261</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,7 +971,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xe649643b38b6c14acf9bbbd3214bd63ce98d37feffda0c872c3665293f137b9c</t>
+          <t>0x2f280a5348c67d22f499a879111a6cd14ba32c30651f4b235087504d75fcb720</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -979,12 +987,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.3862</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>EFL Cup</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -1010,7 +1018,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x75d0d882d84fabe75ec0ebfdf953c3267c7e17303f40762904f5aabc9353a5f5</t>
+          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1040,7 +1048,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785743239</t>
+          <t>1785743240</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1050,7 +1058,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>12.944984</t>
+          <t>9.501188</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1067,7 +1075,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x6da358c7d3a4cfc684658518c8cb0424ee2d0662e048d78a024625d5b4747aed</t>
+          <t>0xe649643b38b6c14acf9bbbd3214bd63ce98d37feffda0c872c3665293f137b9c</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1083,12 +1091,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.5263</t>
+          <t>1.3862</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>EFL Cup</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -1114,7 +1122,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0x75d0d882d84fabe75ec0ebfdf953c3267c7e17303f40762904f5aabc9353a5f5</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1154,7 +1162,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>9.501188</t>
+          <t>12.944984</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1171,7 +1179,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x22ee20a74b7feafe1f674ddfe8f64eb18b48a4aa83ee151db7142c920e3c6990</t>
+          <t>0x6da358c7d3a4cfc684658518c8cb0424ee2d0662e048d78a024625d5b4747aed</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1187,7 +1195,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.3862</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1258,7 +1266,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>12.944984</t>
+          <t>9.501188</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1275,7 +1283,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xe3c6c58c8dab85d1b37033a7121e1d3f4c42a16c31fe969f436aa82e973fe331</t>
+          <t>0x22ee20a74b7feafe1f674ddfe8f64eb18b48a4aa83ee151db7142c920e3c6990</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1286,17 +1294,17 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.3862</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1322,7 +1330,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1352,7 +1360,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785743238</t>
+          <t>1785743239</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1362,7 +1370,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>17.130621</t>
+          <t>12.944984</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1379,7 +1387,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x67892d913ba613f3f4808f12a89e3a4415421d7988b81f5c03035cac2e9e85b1</t>
+          <t>0xe3c6c58c8dab85d1b37033a7121e1d3f4c42a16c31fe969f436aa82e973fe331</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1395,12 +1403,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.445</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1426,7 +1434,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1466,7 +1474,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>22.47191</t>
+          <t>17.130621</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1483,7 +1491,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x51e83e15ab97eefc2ccce2074368f96e4d6b2bc474d60fd48cec81194acc78e8</t>
+          <t>0x67892d913ba613f3f4808f12a89e3a4415421d7988b81f5c03035cac2e9e85b1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1491,11 +1499,7 @@
           <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>10</t>
@@ -1503,19 +1507,15 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.335</t>
+          <t>1.445</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1538,7 +1538,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x1b7328b49fa63aee1bd67882f5cac5a5686aebcb538af0959dcdd4181c5e2f57</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785742250</t>
+          <t>1785743238</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>29.850746</t>
+          <t>22.47191</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1595,7 +1595,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x0e0cffe2676af4f324fc06dde5b8beaeded42b973c319bbf3fb70687f8887f41</t>
+          <t>0x51e83e15ab97eefc2ccce2074368f96e4d6b2bc474d60fd48cec81194acc78e8</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1615,17 +1615,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.5587</t>
+          <t>1.335</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
+          <t>0x1b7328b49fa63aee1bd67882f5cac5a5686aebcb538af0959dcdd4181c5e2f57</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>17.897092</t>
+          <t>29.850746</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1707,12 +1707,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xb28bdee5a5bd24b5937965869b7830544160fac83e2df3848790121d4082d3d0</t>
+          <t>0x0e0cffe2676af4f324fc06dde5b8beaeded42b973c319bbf3fb70687f8887f41</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1722,22 +1722,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.5587</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1792,7 +1792,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785741714</t>
+          <t>1785742250</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>4.020101</t>
+          <t>17.897092</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1819,12 +1819,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xf27c17a15bfe9521fe22971af3d8cd2a8b3c9955888a401e463346a949eb3345</t>
+          <t>0xb28bdee5a5bd24b5937965869b7830544160fac83e2df3848790121d4082d3d0</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1834,22 +1834,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.4438</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x7c21a171d3ea8b89b468e5886d9b7cec062e0e10cc0a3ad080d701f2e478e0d8</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785740160</t>
+          <t>1785741714</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>22.535211</t>
+          <t>4.020101</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1931,12 +1931,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
+          <t>0xf27c17a15bfe9521fe22971af3d8cd2a8b3c9955888a401e463346a949eb3345</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1946,22 +1946,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.2475</t>
+          <t>1.4438</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0x7c21a171d3ea8b89b468e5886d9b7cec062e0e10cc0a3ad080d701f2e478e0d8</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785729810</t>
+          <t>1785740160</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>4.040404</t>
+          <t>22.535211</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2043,7 +2043,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
+          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2058,12 +2058,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>3.99987</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.2475</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785729635</t>
+          <t>1785729810</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>16.079879</t>
+          <t>4.040404</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2155,7 +2155,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
+          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2170,12 +2170,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>23.26</t>
+          <t>3.99987</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.4338</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2195,27 +2195,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2240,17 +2240,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785597225</t>
+          <t>1785729635</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>53.62536</t>
+          <t>16.079879</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
+          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2282,12 +2282,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>23.26</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2297,32 +2297,32 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785595661</t>
+          <t>1785597225</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>3.11284</t>
+          <t>53.62536</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2379,7 +2379,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
+          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2394,12 +2394,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785594340</t>
+          <t>1785595661</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>27.777778</t>
+          <t>3.11284</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2491,7 +2491,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
+          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785593884</t>
+          <t>1785594340</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>27.777778</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2603,7 +2603,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
+          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2715,7 +2715,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
+          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2730,12 +2730,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>25.04</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.385</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785593611</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>65.038961</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2827,7 +2827,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
+          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2842,12 +2842,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>25.04</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.2375</t>
+          <t>1.385</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2882,7 +2882,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785593186</t>
+          <t>1785593611</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>49.263158</t>
+          <t>65.038961</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2939,7 +2939,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
+          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2954,12 +2954,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.2375</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2969,32 +2969,32 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785592744</t>
+          <t>1785593186</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>7.088608</t>
+          <t>49.263158</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3051,7 +3051,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
+          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3066,7 +3066,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>3.59</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785592658</t>
+          <t>1785592744</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>9.088608</t>
+          <t>7.088608</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3163,7 +3163,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
+          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3178,7 +3178,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>22.05</t>
+          <t>3.59</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785592637</t>
+          <t>1785592658</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>55.822785</t>
+          <t>9.088608</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3275,7 +3275,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
+          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3283,15 +3283,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>36.31948</t>
+          <t>22.05</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3299,7 +3303,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -3352,7 +3360,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785589857</t>
+          <t>1785592637</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3362,7 +3370,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>58.816972</t>
+          <t>55.822785</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3379,7 +3387,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
+          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3390,7 +3398,7 @@
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>36.31948</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -3456,7 +3464,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785589600</t>
+          <t>1785589857</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3466,7 +3474,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>6.54251</t>
+          <t>58.816972</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3483,7 +3491,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
+          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3494,12 +3502,12 @@
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>18.36999</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.615</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3560,7 +3568,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785589491</t>
+          <t>1785589600</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3570,7 +3578,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>29.869902</t>
+          <t>6.54251</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3587,7 +3595,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
+          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3598,12 +3606,12 @@
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>18.54999</t>
+          <t>18.36999</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.615</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3664,7 +3672,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785588508</t>
+          <t>1785589491</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3674,7 +3682,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>30.597922</t>
+          <t>29.869902</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3691,27 +3699,23 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
+          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>15.21</t>
+          <t>18.54999</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3719,11 +3723,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -3776,7 +3776,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785587700</t>
+          <t>1785588508</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>54.08</t>
+          <t>30.597922</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3803,23 +3803,27 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
+          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>6.44999</t>
+          <t>15.21</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.7237</t>
+          <t>1.2812</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3827,7 +3831,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -3880,7 +3888,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785585922</t>
+          <t>1785587700</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3890,7 +3898,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>8.911903</t>
+          <t>54.08</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3907,7 +3915,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
+          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3918,12 +3926,12 @@
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>3.26</t>
+          <t>6.44999</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.7212</t>
+          <t>1.7237</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3984,7 +3992,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785579524</t>
+          <t>1785585922</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -3994,7 +4002,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>4.519931</t>
+          <t>8.911903</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4011,7 +4019,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
+          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4022,7 +4030,7 @@
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3.61999</t>
+          <t>3.26</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -4088,7 +4096,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785579365</t>
+          <t>1785579524</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4098,7 +4106,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>5.01905</t>
+          <t>4.519931</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4115,27 +4123,23 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
+          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>3.61999</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4143,26 +4147,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K35" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785577998</t>
+          <t>1785579365</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>59.143969</t>
+          <t>5.01905</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4227,7 +4227,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
+          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4242,12 +4242,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4257,7 +4257,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -4282,7 +4282,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785577962</t>
+          <t>1785577998</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4322,7 +4322,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>82.758621</t>
+          <t>59.143969</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4339,12 +4339,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
+          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -4354,12 +4354,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.3225</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4369,24 +4369,24 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K37" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -4394,7 +4394,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4424,7 +4424,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1785577789</t>
+          <t>1785577962</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>3.534884</t>
+          <t>82.758621</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4451,7 +4451,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
+          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4466,12 +4466,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>18.99909</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.3225</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785577788</t>
+          <t>1785577789</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4546,7 +4546,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>59.141136</t>
+          <t>3.534884</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4563,7 +4563,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
+          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>18.99909</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -4648,7 +4648,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785577788</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>6.101167</t>
+          <t>59.141136</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4675,7 +4675,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
+          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4690,12 +4690,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2.81824</t>
+          <t>1.96</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4770,7 +4770,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>8.807</t>
+          <t>6.101167</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
+          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4802,7 +4802,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>20.06</t>
+          <t>2.81824</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -4872,7 +4872,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1785576072</t>
+          <t>1785576753</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4882,7 +4882,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>62.6875</t>
+          <t>8.807</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4899,7 +4899,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
+          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>22.07</t>
+          <t>20.06</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1785575036</t>
+          <t>1785576072</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>68.96875</t>
+          <t>62.6875</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5011,7 +5011,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
+          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>22.07</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -5096,7 +5096,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1785574569</t>
+          <t>1785575036</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -5106,7 +5106,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>3.625</t>
+          <t>68.96875</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5123,7 +5123,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
+          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -5138,7 +5138,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>19.25059</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1785574187</t>
+          <t>1785574569</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -5218,7 +5218,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>60.158094</t>
+          <t>3.625</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5235,7 +5235,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
+          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5250,7 +5250,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>20.96</t>
+          <t>19.25059</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -5320,7 +5320,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785574187</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>65.5</t>
+          <t>60.158094</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5347,7 +5347,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
+          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5362,7 +5362,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2.69</t>
+          <t>20.96</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>8.40625</t>
+          <t>65.5</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5459,7 +5459,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
+          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5474,7 +5474,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>2.69</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1785574073</t>
+          <t>1785574186</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
@@ -5554,7 +5554,7 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>6.90625</t>
+          <t>8.40625</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5571,7 +5571,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
+          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5586,7 +5586,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -5656,7 +5656,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>1785573852</t>
+          <t>1785574073</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -5666,7 +5666,7 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>6.25</t>
+          <t>6.90625</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -5683,7 +5683,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
+          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5698,12 +5698,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5768,7 +5768,7 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>1785570690</t>
+          <t>1785573852</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
@@ -5778,7 +5778,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>6.256809</t>
+          <t>6.25</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -5795,7 +5795,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
+          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -5810,12 +5810,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2.01</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5880,7 +5880,7 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>1785570471</t>
+          <t>1785570690</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
@@ -5890,7 +5890,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>31.25</t>
+          <t>6.256809</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -5907,7 +5907,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
+          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -5915,15 +5915,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>19.72999</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5931,7 +5935,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
       <c r="H51" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -5954,7 +5962,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -5984,7 +5992,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>1785569792</t>
+          <t>1785570471</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -5994,7 +6002,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>32.544313</t>
+          <t>31.25</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -6011,7 +6019,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
+          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6019,19 +6027,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>19.72999</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6039,26 +6043,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K52" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -6066,7 +6066,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>1785569076</t>
+          <t>1785569792</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
@@ -6106,7 +6106,7 @@
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>6.59375</t>
+          <t>32.544313</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -6123,12 +6123,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
+          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -6138,12 +6138,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.11</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>1.605</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6153,7 +6153,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -6163,27 +6163,27 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298738</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -6208,17 +6208,17 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>1785512959</t>
+          <t>1785569076</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1785592800</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>1.652893</t>
+          <t>6.59375</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -6235,12 +6235,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -6250,12 +6250,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2.51</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.605</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6265,7 +6265,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -6275,27 +6275,27 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -6320,17 +6320,17 @@
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>1785497246</t>
+          <t>1785512959</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>5.97619</t>
+          <t>1.652893</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -6347,12 +6347,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -6362,12 +6362,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.51</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6432,7 +6432,7 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>1785346230</t>
+          <t>1785497246</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
@@ -6442,7 +6442,7 @@
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>2.173913</t>
+          <t>5.97619</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -6459,110 +6459,222 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>1785346230</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>2.173913</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>0xea48d5fe72de69b25067fdb4fdaf1d08ce7262ad75f6855864d3a656da39b313</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>1.46</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
+      <c r="G57" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
+      <c r="H57" t="inlineStr">
         <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
+      <c r="I57" t="inlineStr">
         <is>
           <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="J57" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
+      <c r="K57" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="L56" t="inlineStr">
+      <c r="L57" t="inlineStr">
         <is>
           <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr">
+      <c r="M57" t="inlineStr">
         <is>
           <t>L19298738</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O56" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P56" t="inlineStr">
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q56" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R56" t="inlineStr">
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
         <is>
           <t>1785345250</t>
         </is>
       </c>
-      <c r="S56" t="inlineStr">
+      <c r="S57" t="inlineStr">
         <is>
           <t>1785592800</t>
         </is>
       </c>
-      <c r="T56" t="inlineStr">
+      <c r="T57" t="inlineStr">
         <is>
           <t>2.173913</t>
         </is>
       </c>
-      <c r="U56" t="inlineStr">
+      <c r="U57" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V56" t="inlineStr">
+      <c r="V57" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-05 19:01:30 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/EFL Cup/trades.xlsx
+++ b/data/sxbet/ligas/EFL Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V57"/>
+  <dimension ref="A1:V58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xfcba109b300bea480abe542eaa7725c7fec13f0fedc18d9991df424ad450dc90</t>
+          <t>0x02c4621d6a830534abb9a71c7d2fcc46730afe8d3b686773dfd4c590f2060027</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x095B1B11E9C470934404Ba7F04da5F79930b2504</t>
+          <t>0x204e31304364d2A5f7B90dE28F507adc449Ae221</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,22 +546,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>14.58</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>AFC Wimbledon -1.5</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>AFC Wimbledon vs Newport County</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>AFC Wimbledon</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x30711e53de1ac1c4a025d48c70e4859ee55e52e5e57d10ed46259cc01bb5d46e</t>
+          <t>0x9f1f722832eb2e6381f3a0226a98c406eccc5bd7e76caaaebb931fdda305a642</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298736</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785778500</t>
+          <t>1785942153</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1786197600</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>2.941176</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x9b63fb9bdb0939e4fa277441c5160ae767a06c0723ae1697f56722a32c1dbbf4</t>
+          <t>0xfcba109b300bea480abe542eaa7725c7fec13f0fedc18d9991df424ad450dc90</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x095B1B11E9C470934404Ba7F04da5F79930b2504</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,39 +658,39 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.47999</t>
+          <t>14.58</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5762</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>York City vs Crawley Town</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>York City</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>York City vs Crawley Town</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>York City</t>
-        </is>
-      </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>Crawley Town</t>
@@ -698,7 +698,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0x30711e53de1ac1c4a025d48c70e4859ee55e52e5e57d10ed46259cc01bb5d46e</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785751617</t>
+          <t>1785778500</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2.568312</t>
+          <t>18.0</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,7 +755,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x34fd96c52ca66603743b136c029d1196926b8ea965b35ad916e9e624891a3c31</t>
+          <t>0x9b63fb9bdb0939e4fa277441c5160ae767a06c0723ae1697f56722a32c1dbbf4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -763,23 +763,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2.59999</t>
+          <t>1.47999</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.6887</t>
+          <t>1.5762</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>York City</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -802,7 +810,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xb943c3d4cb1b4aebd6296b959eb4168b4f43df52a8043a9e84d184a931ac076c</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -832,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785751591</t>
+          <t>1785751617</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -842,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>3.77494</t>
+          <t>2.568312</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,39 +867,31 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x92e4361325da8adb7d2c64339dc80666c0b8e0d69bcdd503c9dcdc859b32e858</t>
+          <t>0x34fd96c52ca66603743b136c029d1196926b8ea965b35ad916e9e624891a3c31</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>288.19</t>
+          <t>2.59999</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.555</t>
+          <t>1.6887</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -914,7 +914,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
+          <t>0xb943c3d4cb1b4aebd6296b959eb4168b4f43df52a8043a9e84d184a931ac076c</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785746436</t>
+          <t>1785751591</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>519.261261</t>
+          <t>3.77494</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,31 +971,39 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x2f280a5348c67d22f499a879111a6cd14ba32c30651f4b235087504d75fcb720</t>
+          <t>0x92e4361325da8adb7d2c64339dc80666c0b8e0d69bcdd503c9dcdc859b32e858</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>288.19</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.5263</t>
+          <t>1.555</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1018,7 +1026,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
+          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1048,7 +1056,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785743240</t>
+          <t>1785746436</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1058,7 +1066,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>9.501188</t>
+          <t>519.261261</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,7 +1083,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xe649643b38b6c14acf9bbbd3214bd63ce98d37feffda0c872c3665293f137b9c</t>
+          <t>0x2f280a5348c67d22f499a879111a6cd14ba32c30651f4b235087504d75fcb720</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1091,12 +1099,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.3862</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>EFL Cup</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -1122,7 +1130,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x75d0d882d84fabe75ec0ebfdf953c3267c7e17303f40762904f5aabc9353a5f5</t>
+          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1152,7 +1160,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785743239</t>
+          <t>1785743240</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1170,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>12.944984</t>
+          <t>9.501188</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,7 +1187,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x6da358c7d3a4cfc684658518c8cb0424ee2d0662e048d78a024625d5b4747aed</t>
+          <t>0xe649643b38b6c14acf9bbbd3214bd63ce98d37feffda0c872c3665293f137b9c</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1195,12 +1203,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.5263</t>
+          <t>1.3862</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>EFL Cup</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -1226,7 +1234,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0x75d0d882d84fabe75ec0ebfdf953c3267c7e17303f40762904f5aabc9353a5f5</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1266,7 +1274,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>9.501188</t>
+          <t>12.944984</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1283,7 +1291,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x22ee20a74b7feafe1f674ddfe8f64eb18b48a4aa83ee151db7142c920e3c6990</t>
+          <t>0x6da358c7d3a4cfc684658518c8cb0424ee2d0662e048d78a024625d5b4747aed</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1299,7 +1307,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.3862</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1370,7 +1378,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>12.944984</t>
+          <t>9.501188</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1387,7 +1395,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xe3c6c58c8dab85d1b37033a7121e1d3f4c42a16c31fe969f436aa82e973fe331</t>
+          <t>0x22ee20a74b7feafe1f674ddfe8f64eb18b48a4aa83ee151db7142c920e3c6990</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1398,17 +1406,17 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.3862</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1434,7 +1442,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1464,7 +1472,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785743238</t>
+          <t>1785743239</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1474,7 +1482,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>17.130621</t>
+          <t>12.944984</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1491,7 +1499,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x67892d913ba613f3f4808f12a89e3a4415421d7988b81f5c03035cac2e9e85b1</t>
+          <t>0xe3c6c58c8dab85d1b37033a7121e1d3f4c42a16c31fe969f436aa82e973fe331</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1507,12 +1515,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.445</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -1538,7 +1546,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1578,7 +1586,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>22.47191</t>
+          <t>17.130621</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1595,7 +1603,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x51e83e15ab97eefc2ccce2074368f96e4d6b2bc474d60fd48cec81194acc78e8</t>
+          <t>0x67892d913ba613f3f4808f12a89e3a4415421d7988b81f5c03035cac2e9e85b1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1603,11 +1611,7 @@
           <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>10</t>
@@ -1615,19 +1619,15 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.335</t>
+          <t>1.445</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1650,7 +1650,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x1b7328b49fa63aee1bd67882f5cac5a5686aebcb538af0959dcdd4181c5e2f57</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785742250</t>
+          <t>1785743238</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>29.850746</t>
+          <t>22.47191</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1707,7 +1707,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x0e0cffe2676af4f324fc06dde5b8beaeded42b973c319bbf3fb70687f8887f41</t>
+          <t>0x51e83e15ab97eefc2ccce2074368f96e4d6b2bc474d60fd48cec81194acc78e8</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1727,17 +1727,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.5587</t>
+          <t>1.335</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
+          <t>0x1b7328b49fa63aee1bd67882f5cac5a5686aebcb538af0959dcdd4181c5e2f57</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>17.897092</t>
+          <t>29.850746</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1819,12 +1819,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xb28bdee5a5bd24b5937965869b7830544160fac83e2df3848790121d4082d3d0</t>
+          <t>0x0e0cffe2676af4f324fc06dde5b8beaeded42b973c319bbf3fb70687f8887f41</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1834,22 +1834,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.5587</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785741714</t>
+          <t>1785742250</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>4.020101</t>
+          <t>17.897092</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1931,12 +1931,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xf27c17a15bfe9521fe22971af3d8cd2a8b3c9955888a401e463346a949eb3345</t>
+          <t>0xb28bdee5a5bd24b5937965869b7830544160fac83e2df3848790121d4082d3d0</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1946,22 +1946,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.4438</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x7c21a171d3ea8b89b468e5886d9b7cec062e0e10cc0a3ad080d701f2e478e0d8</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785740160</t>
+          <t>1785741714</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>22.535211</t>
+          <t>4.020101</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2043,12 +2043,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
+          <t>0xf27c17a15bfe9521fe22971af3d8cd2a8b3c9955888a401e463346a949eb3345</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2058,22 +2058,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.2475</t>
+          <t>1.4438</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2098,7 +2098,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0x7c21a171d3ea8b89b468e5886d9b7cec062e0e10cc0a3ad080d701f2e478e0d8</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785729810</t>
+          <t>1785740160</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>4.040404</t>
+          <t>22.535211</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2155,7 +2155,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
+          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2170,12 +2170,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>3.99987</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.2475</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785729635</t>
+          <t>1785729810</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>16.079879</t>
+          <t>4.040404</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
+          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2282,12 +2282,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>23.26</t>
+          <t>3.99987</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.4338</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2307,27 +2307,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2352,17 +2352,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785597225</t>
+          <t>1785729635</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>53.62536</t>
+          <t>16.079879</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2379,7 +2379,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
+          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2394,12 +2394,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>23.26</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2409,32 +2409,32 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785595661</t>
+          <t>1785597225</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>3.11284</t>
+          <t>53.62536</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2491,7 +2491,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
+          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2506,12 +2506,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785594340</t>
+          <t>1785595661</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>27.777778</t>
+          <t>3.11284</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2603,7 +2603,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
+          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2623,7 +2623,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2688,7 +2688,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785593884</t>
+          <t>1785594340</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2698,7 +2698,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>27.777778</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2715,7 +2715,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
+          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2827,7 +2827,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
+          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2842,12 +2842,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>25.04</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.385</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785593611</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>65.038961</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2939,7 +2939,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
+          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2954,12 +2954,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>25.04</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.2375</t>
+          <t>1.385</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785593186</t>
+          <t>1785593611</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>49.263158</t>
+          <t>65.038961</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3051,7 +3051,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
+          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3066,12 +3066,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.2375</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3081,32 +3081,32 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785592744</t>
+          <t>1785593186</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>7.088608</t>
+          <t>49.263158</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3163,7 +3163,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
+          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3178,7 +3178,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3.59</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785592658</t>
+          <t>1785592744</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>9.088608</t>
+          <t>7.088608</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3275,7 +3275,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
+          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>22.05</t>
+          <t>3.59</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785592637</t>
+          <t>1785592658</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>55.822785</t>
+          <t>9.088608</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3387,7 +3387,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
+          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3395,15 +3395,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>36.31948</t>
+          <t>22.05</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3411,7 +3415,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -3464,7 +3472,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785589857</t>
+          <t>1785592637</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3474,7 +3482,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>58.816972</t>
+          <t>55.822785</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3491,7 +3499,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
+          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3502,7 +3510,7 @@
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>36.31948</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -3568,7 +3576,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785589600</t>
+          <t>1785589857</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3578,7 +3586,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>6.54251</t>
+          <t>58.816972</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3595,7 +3603,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
+          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3606,12 +3614,12 @@
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>18.36999</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.615</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3672,7 +3680,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785589491</t>
+          <t>1785589600</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3682,7 +3690,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>29.869902</t>
+          <t>6.54251</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3699,7 +3707,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
+          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3710,12 +3718,12 @@
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>18.54999</t>
+          <t>18.36999</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.615</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3776,7 +3784,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785588508</t>
+          <t>1785589491</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3786,7 +3794,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>30.597922</t>
+          <t>29.869902</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3803,27 +3811,23 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
+          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>15.21</t>
+          <t>18.54999</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3831,11 +3835,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3888,7 +3888,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785587700</t>
+          <t>1785588508</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>54.08</t>
+          <t>30.597922</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3915,23 +3915,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
+          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>6.44999</t>
+          <t>15.21</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.7237</t>
+          <t>1.2812</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3939,7 +3943,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -3992,7 +4000,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785585922</t>
+          <t>1785587700</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -4002,7 +4010,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>8.911903</t>
+          <t>54.08</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4019,7 +4027,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
+          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4030,12 +4038,12 @@
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3.26</t>
+          <t>6.44999</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.7212</t>
+          <t>1.7237</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4096,7 +4104,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785579524</t>
+          <t>1785585922</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4106,7 +4114,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>4.519931</t>
+          <t>8.911903</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4123,7 +4131,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
+          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4134,7 +4142,7 @@
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>3.61999</t>
+          <t>3.26</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -4200,7 +4208,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785579365</t>
+          <t>1785579524</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4210,7 +4218,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>5.01905</t>
+          <t>4.519931</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4227,27 +4235,23 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
+          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>3.61999</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4255,26 +4259,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K36" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785577998</t>
+          <t>1785579365</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4322,7 +4322,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>59.143969</t>
+          <t>5.01905</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4339,7 +4339,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
+          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4354,12 +4354,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4369,7 +4369,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4424,7 +4424,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1785577962</t>
+          <t>1785577998</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>82.758621</t>
+          <t>59.143969</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4451,12 +4451,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
+          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4466,12 +4466,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.3225</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4481,24 +4481,24 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K38" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -4506,7 +4506,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785577789</t>
+          <t>1785577962</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4546,7 +4546,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>3.534884</t>
+          <t>82.758621</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4563,7 +4563,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
+          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4578,12 +4578,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>18.99909</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.3225</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4648,7 +4648,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1785577788</t>
+          <t>1785577789</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>59.141136</t>
+          <t>3.534884</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4675,7 +4675,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
+          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4690,7 +4690,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>18.99909</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785577788</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4770,7 +4770,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>6.101167</t>
+          <t>59.141136</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
+          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4802,12 +4802,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2.81824</t>
+          <t>1.96</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4882,7 +4882,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>8.807</t>
+          <t>6.101167</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4899,7 +4899,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
+          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>20.06</t>
+          <t>2.81824</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1785576072</t>
+          <t>1785576753</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>62.6875</t>
+          <t>8.807</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5011,7 +5011,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
+          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>22.07</t>
+          <t>20.06</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -5096,7 +5096,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1785575036</t>
+          <t>1785576072</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -5106,7 +5106,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>68.96875</t>
+          <t>62.6875</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5123,7 +5123,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
+          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -5138,7 +5138,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>22.07</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1785574569</t>
+          <t>1785575036</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -5218,7 +5218,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>3.625</t>
+          <t>68.96875</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5235,7 +5235,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
+          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5250,7 +5250,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>19.25059</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -5320,7 +5320,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1785574187</t>
+          <t>1785574569</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>60.158094</t>
+          <t>3.625</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5347,7 +5347,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
+          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5362,7 +5362,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>20.96</t>
+          <t>19.25059</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -5432,7 +5432,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785574187</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>65.5</t>
+          <t>60.158094</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5459,7 +5459,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
+          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5474,7 +5474,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2.69</t>
+          <t>20.96</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -5554,7 +5554,7 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>8.40625</t>
+          <t>65.5</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5571,7 +5571,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
+          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5586,7 +5586,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>2.69</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -5656,7 +5656,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>1785574073</t>
+          <t>1785574186</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -5666,7 +5666,7 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>6.90625</t>
+          <t>8.40625</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -5683,7 +5683,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
+          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5698,7 +5698,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -5768,7 +5768,7 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>1785573852</t>
+          <t>1785574073</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
@@ -5778,7 +5778,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>6.25</t>
+          <t>6.90625</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -5795,7 +5795,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
+          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -5810,12 +5810,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5880,7 +5880,7 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>1785570690</t>
+          <t>1785573852</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
@@ -5890,7 +5890,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>6.256809</t>
+          <t>6.25</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -5907,7 +5907,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
+          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -5922,12 +5922,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2.01</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5992,7 +5992,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>1785570471</t>
+          <t>1785570690</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -6002,7 +6002,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>31.25</t>
+          <t>6.256809</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -6019,7 +6019,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
+          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6027,15 +6027,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>19.72999</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6043,7 +6047,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
       <c r="H52" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -6066,7 +6074,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -6096,7 +6104,7 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>1785569792</t>
+          <t>1785570471</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
@@ -6106,7 +6114,7 @@
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>32.544313</t>
+          <t>31.25</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -6123,7 +6131,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
+          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6131,19 +6139,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>19.72999</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6151,26 +6155,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K53" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -6178,7 +6178,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -6208,7 +6208,7 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>1785569076</t>
+          <t>1785569792</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -6218,7 +6218,7 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>6.59375</t>
+          <t>32.544313</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -6235,12 +6235,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
+          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -6250,12 +6250,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.11</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>1.605</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6265,7 +6265,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -6275,27 +6275,27 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298738</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -6320,17 +6320,17 @@
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>1785512959</t>
+          <t>1785569076</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1785592800</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>1.652893</t>
+          <t>6.59375</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -6347,12 +6347,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -6362,12 +6362,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2.51</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.605</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6377,7 +6377,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -6387,27 +6387,27 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -6432,17 +6432,17 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>1785497246</t>
+          <t>1785512959</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>5.97619</t>
+          <t>1.652893</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -6459,12 +6459,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -6474,12 +6474,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.51</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>1785346230</t>
+          <t>1785497246</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
@@ -6554,7 +6554,7 @@
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>2.173913</t>
+          <t>5.97619</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -6571,110 +6571,222 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>1785346230</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>2.173913</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
           <t>0xea48d5fe72de69b25067fdb4fdaf1d08ce7262ad75f6855864d3a656da39b313</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
         <is>
           <t>1.46</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="G58" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="H58" t="inlineStr">
         <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
+      <c r="I58" t="inlineStr">
         <is>
           <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
+      <c r="J58" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr">
+      <c r="K58" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="L57" t="inlineStr">
+      <c r="L58" t="inlineStr">
         <is>
           <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr">
+      <c r="M58" t="inlineStr">
         <is>
           <t>L19298738</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O57" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P57" t="inlineStr">
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q57" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R57" t="inlineStr">
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
         <is>
           <t>1785345250</t>
         </is>
       </c>
-      <c r="S57" t="inlineStr">
+      <c r="S58" t="inlineStr">
         <is>
           <t>1785592800</t>
         </is>
       </c>
-      <c r="T57" t="inlineStr">
+      <c r="T58" t="inlineStr">
         <is>
           <t>2.173913</t>
         </is>
       </c>
-      <c r="U57" t="inlineStr">
+      <c r="U58" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V57" t="inlineStr">
+      <c r="V58" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-05 22:01:22 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/EFL Cup/trades.xlsx
+++ b/data/sxbet/ligas/EFL Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V58"/>
+  <dimension ref="A1:V62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x02c4621d6a830534abb9a71c7d2fcc46730afe8d3b686773dfd4c590f2060027</t>
+          <t>0x4da7133bca54b84184238baa7d30b02372340f739df06b943262742640837a0a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x204e31304364d2A5f7B90dE28F507adc449Ae221</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,22 +546,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>1.195</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>AFC Wimbledon -1.5</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x9f1f722832eb2e6381f3a0226a98c406eccc5bd7e76caaaebb931fdda305a642</t>
+          <t>0xea47b6c120c94ae31f3299be9d23585a5cbf1b0ada4b3059268dd4cc9712b5d8</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785942153</t>
+          <t>1785962236</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2.941176</t>
+          <t>153.846154</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xfcba109b300bea480abe542eaa7725c7fec13f0fedc18d9991df424ad450dc90</t>
+          <t>0xbae8ac7d4c8a6185b820438796f1f9f58ac63f2ed636b3e75be83914f2d44036</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x095B1B11E9C470934404Ba7F04da5F79930b2504</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,22 +658,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>14.58</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.1175</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -683,27 +683,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Bristol City FC vs Walsall</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Bristol City FC</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x30711e53de1ac1c4a025d48c70e4859ee55e52e5e57d10ed46259cc01bb5d46e</t>
+          <t>0xc9a261f972b5555c9a1e6c0f33be8eb6a6906d2cda51babdb51dd64314b2c091</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298734</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -728,17 +728,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785778500</t>
+          <t>1785961563</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1786041900</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>85.106383</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,12 +755,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x9b63fb9bdb0939e4fa277441c5160ae767a06c0723ae1697f56722a32c1dbbf4</t>
+          <t>0xdd62398a10f567ee5469950797393093a356b40e7fe5930931a6c998d441d9b9</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -770,12 +770,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.47999</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.5762</t>
+          <t>1.1975</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Cheltenham Town</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -795,27 +795,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Cheltenham Town vs Charlton Athletic</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Cheltenham Town</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Charlton Athletic</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0x6bf36843abe397fbc7c233e0ca342729b9cd199b53d9ee9a63b96ac9358c9a1a</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19299406</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -840,17 +840,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785751617</t>
+          <t>1785960783</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1786214700</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2.568312</t>
+          <t>15.189873</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,31 +867,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x34fd96c52ca66603743b136c029d1196926b8ea965b35ad916e9e624891a3c31</t>
+          <t>0xcb8aa49e12f3f29aa35ec5b7ff00195594f282ca0db4d0d9be5e2e477b96970d</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.59999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.6887</t>
+          <t>1.1175</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Walsall</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -899,27 +907,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Bristol City FC vs Walsall</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Bristol City FC</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xb943c3d4cb1b4aebd6296b959eb4168b4f43df52a8043a9e84d184a931ac076c</t>
+          <t>0xc9a261f972b5555c9a1e6c0f33be8eb6a6906d2cda51babdb51dd64314b2c091</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298734</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,17 +952,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785751591</t>
+          <t>1785960695</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1786041900</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>3.77494</t>
+          <t>59.574468</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,12 +979,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x92e4361325da8adb7d2c64339dc80666c0b8e0d69bcdd503c9dcdc859b32e858</t>
+          <t>0x02c4621d6a830534abb9a71c7d2fcc46730afe8d3b686773dfd4c590f2060027</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x204e31304364d2A5f7B90dE28F507adc449Ae221</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -986,22 +994,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>288.19</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.555</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>AFC Wimbledon -1.5</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1011,27 +1019,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>AFC Wimbledon vs Newport County</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>AFC Wimbledon</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
+          <t>0x9f1f722832eb2e6381f3a0226a98c406eccc5bd7e76caaaebb931fdda305a642</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298736</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1056,17 +1064,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785746436</t>
+          <t>1785942153</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1786197600</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>519.261261</t>
+          <t>2.941176</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,31 +1091,39 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x2f280a5348c67d22f499a879111a6cd14ba32c30651f4b235087504d75fcb720</t>
+          <t>0xfcba109b300bea480abe542eaa7725c7fec13f0fedc18d9991df424ad450dc90</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0x095B1B11E9C470934404Ba7F04da5F79930b2504</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>14.58</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.5263</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1130,7 +1146,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
+          <t>0x30711e53de1ac1c4a025d48c70e4859ee55e52e5e57d10ed46259cc01bb5d46e</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1160,7 +1176,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785743240</t>
+          <t>1785778500</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1170,7 +1186,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>9.501188</t>
+          <t>18.0</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,36 +1203,44 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xe649643b38b6c14acf9bbbd3214bd63ce98d37feffda0c872c3665293f137b9c</t>
+          <t>0x9b63fb9bdb0939e4fa277441c5160ae767a06c0723ae1697f56722a32c1dbbf4</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1.47999</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.3862</t>
+          <t>1.5762</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>York City</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>York City vs Crawley Town</t>
@@ -1234,7 +1258,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x75d0d882d84fabe75ec0ebfdf953c3267c7e17303f40762904f5aabc9353a5f5</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1264,7 +1288,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785743239</t>
+          <t>1785751617</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1274,7 +1298,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>12.944984</t>
+          <t>2.568312</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,28 +1315,28 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x6da358c7d3a4cfc684658518c8cb0424ee2d0662e048d78a024625d5b4747aed</t>
+          <t>0x34fd96c52ca66603743b136c029d1196926b8ea965b35ad916e9e624891a3c31</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2.59999</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.5263</t>
+          <t>1.6887</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1338,7 +1362,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0xb943c3d4cb1b4aebd6296b959eb4168b4f43df52a8043a9e84d184a931ac076c</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1368,7 +1392,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785743239</t>
+          <t>1785751591</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1378,7 +1402,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>9.501188</t>
+          <t>3.77494</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,31 +1419,39 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x22ee20a74b7feafe1f674ddfe8f64eb18b48a4aa83ee151db7142c920e3c6990</t>
+          <t>0x92e4361325da8adb7d2c64339dc80666c0b8e0d69bcdd503c9dcdc859b32e858</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>288.19</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.3862</t>
+          <t>1.555</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1442,7 +1474,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1472,7 +1504,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785743239</t>
+          <t>1785746436</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1482,7 +1514,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>12.944984</t>
+          <t>519.261261</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1499,7 +1531,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xe3c6c58c8dab85d1b37033a7121e1d3f4c42a16c31fe969f436aa82e973fe331</t>
+          <t>0x2f280a5348c67d22f499a879111a6cd14ba32c30651f4b235087504d75fcb720</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1510,12 +1542,12 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1576,7 +1608,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785743238</t>
+          <t>1785743240</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1586,7 +1618,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>17.130621</t>
+          <t>9.501188</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1603,7 +1635,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x67892d913ba613f3f4808f12a89e3a4415421d7988b81f5c03035cac2e9e85b1</t>
+          <t>0xe649643b38b6c14acf9bbbd3214bd63ce98d37feffda0c872c3665293f137b9c</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1614,17 +1646,17 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.445</t>
+          <t>1.3862</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>EFL Cup</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1650,7 +1682,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0x75d0d882d84fabe75ec0ebfdf953c3267c7e17303f40762904f5aabc9353a5f5</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1680,7 +1712,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785743238</t>
+          <t>1785743239</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1690,7 +1722,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>22.47191</t>
+          <t>12.944984</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1707,7 +1739,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x51e83e15ab97eefc2ccce2074368f96e4d6b2bc474d60fd48cec81194acc78e8</t>
+          <t>0x6da358c7d3a4cfc684658518c8cb0424ee2d0662e048d78a024625d5b4747aed</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1715,31 +1747,23 @@
           <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.335</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1762,7 +1786,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x1b7328b49fa63aee1bd67882f5cac5a5686aebcb538af0959dcdd4181c5e2f57</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1792,7 +1816,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785742250</t>
+          <t>1785743239</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1802,7 +1826,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>29.850746</t>
+          <t>9.501188</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1819,7 +1843,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x0e0cffe2676af4f324fc06dde5b8beaeded42b973c319bbf3fb70687f8887f41</t>
+          <t>0x22ee20a74b7feafe1f674ddfe8f64eb18b48a4aa83ee151db7142c920e3c6990</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1827,31 +1851,23 @@
           <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.5587</t>
+          <t>1.3862</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1874,7 +1890,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1904,7 +1920,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785742250</t>
+          <t>1785743239</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1914,7 +1930,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>17.897092</t>
+          <t>12.944984</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1931,39 +1947,31 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xb28bdee5a5bd24b5937965869b7830544160fac83e2df3848790121d4082d3d0</t>
+          <t>0xe3c6c58c8dab85d1b37033a7121e1d3f4c42a16c31fe969f436aa82e973fe331</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1986,7 +1994,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2016,7 +2024,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785741714</t>
+          <t>1785743238</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2026,7 +2034,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>4.020101</t>
+          <t>17.130621</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2043,7 +2051,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xf27c17a15bfe9521fe22971af3d8cd2a8b3c9955888a401e463346a949eb3345</t>
+          <t>0x67892d913ba613f3f4808f12a89e3a4415421d7988b81f5c03035cac2e9e85b1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2051,11 +2059,7 @@
           <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>10</t>
@@ -2063,19 +2067,15 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.4438</t>
+          <t>1.445</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2098,7 +2098,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x7c21a171d3ea8b89b468e5886d9b7cec062e0e10cc0a3ad080d701f2e478e0d8</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785740160</t>
+          <t>1785743238</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>22.535211</t>
+          <t>22.47191</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2155,12 +2155,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
+          <t>0x51e83e15ab97eefc2ccce2074368f96e4d6b2bc474d60fd48cec81194acc78e8</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2170,22 +2170,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.2475</t>
+          <t>1.335</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0x1b7328b49fa63aee1bd67882f5cac5a5686aebcb538af0959dcdd4181c5e2f57</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785729810</t>
+          <t>1785742250</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>4.040404</t>
+          <t>29.850746</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2267,12 +2267,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
+          <t>0x0e0cffe2676af4f324fc06dde5b8beaeded42b973c319bbf3fb70687f8887f41</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2282,22 +2282,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.99987</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.5587</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2322,7 +2322,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785729635</t>
+          <t>1785742250</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>16.079879</t>
+          <t>17.897092</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2379,7 +2379,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
+          <t>0xb28bdee5a5bd24b5937965869b7830544160fac83e2df3848790121d4082d3d0</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2394,12 +2394,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>23.26</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.4338</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2419,27 +2419,27 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2464,17 +2464,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785597225</t>
+          <t>1785741714</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>53.62536</t>
+          <t>4.020101</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2491,12 +2491,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
+          <t>0xf27c17a15bfe9521fe22971af3d8cd2a8b3c9955888a401e463346a949eb3345</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2506,22 +2506,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.4438</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2531,27 +2531,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x7c21a171d3ea8b89b468e5886d9b7cec062e0e10cc0a3ad080d701f2e478e0d8</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2576,17 +2576,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785595661</t>
+          <t>1785740160</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>3.11284</t>
+          <t>22.535211</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2603,7 +2603,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
+          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2618,12 +2618,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>1.2475</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2643,27 +2643,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2688,17 +2688,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785594340</t>
+          <t>1785729810</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>27.777778</t>
+          <t>4.040404</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2715,7 +2715,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
+          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2730,12 +2730,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3.99987</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2755,27 +2755,27 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2800,17 +2800,17 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785593884</t>
+          <t>1785729635</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>16.079879</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2827,7 +2827,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
+          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2842,12 +2842,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>23.26</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2857,32 +2857,32 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785593884</t>
+          <t>1785597225</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>53.62536</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2939,7 +2939,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
+          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2954,12 +2954,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>25.04</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.385</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785593611</t>
+          <t>1785595661</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>65.038961</t>
+          <t>3.11284</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3051,7 +3051,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
+          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3066,12 +3066,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.2375</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3081,7 +3081,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785593186</t>
+          <t>1785594340</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>49.263158</t>
+          <t>27.777778</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3163,7 +3163,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
+          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3178,12 +3178,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785592744</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>7.088608</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3275,7 +3275,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
+          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3290,12 +3290,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>3.59</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785592658</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>9.088608</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3387,7 +3387,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
+          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3402,12 +3402,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>22.05</t>
+          <t>25.04</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.385</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785592637</t>
+          <t>1785593611</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>55.822785</t>
+          <t>65.038961</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3499,7 +3499,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
+          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3507,15 +3507,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>36.31948</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.2375</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3523,7 +3527,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -3546,7 +3554,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3576,7 +3584,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785589857</t>
+          <t>1785593186</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3586,7 +3594,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>58.816972</t>
+          <t>49.263158</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3603,7 +3611,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
+          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3611,15 +3619,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3627,7 +3639,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -3680,7 +3696,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785589600</t>
+          <t>1785592744</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3690,7 +3706,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>6.54251</t>
+          <t>7.088608</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3707,7 +3723,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
+          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3715,15 +3731,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>18.36999</t>
+          <t>3.59</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.615</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3731,7 +3751,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -3784,7 +3808,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785589491</t>
+          <t>1785592658</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3794,7 +3818,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>29.869902</t>
+          <t>9.088608</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3811,7 +3835,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
+          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3819,15 +3843,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>18.54999</t>
+          <t>22.05</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3835,7 +3863,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -3888,7 +3920,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785588508</t>
+          <t>1785592637</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3898,7 +3930,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>30.597922</t>
+          <t>55.822785</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3915,27 +3947,23 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
+          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>15.21</t>
+          <t>36.31948</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3943,11 +3971,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -3970,7 +3994,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -4000,7 +4024,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785587700</t>
+          <t>1785589857</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -4010,7 +4034,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>54.08</t>
+          <t>58.816972</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4027,7 +4051,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
+          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4038,12 +4062,12 @@
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>6.44999</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.7237</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4074,7 +4098,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4104,7 +4128,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785585922</t>
+          <t>1785589600</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4114,7 +4138,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>8.911903</t>
+          <t>6.54251</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4131,7 +4155,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
+          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4142,12 +4166,12 @@
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>3.26</t>
+          <t>18.36999</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.7212</t>
+          <t>1.615</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4178,7 +4202,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4208,7 +4232,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785579524</t>
+          <t>1785589491</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4218,7 +4242,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>4.519931</t>
+          <t>29.869902</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4235,7 +4259,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
+          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4246,12 +4270,12 @@
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3.61999</t>
+          <t>18.54999</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.7212</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4282,7 +4306,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4312,7 +4336,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785579365</t>
+          <t>1785588508</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4322,7 +4346,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>5.01905</t>
+          <t>30.597922</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4339,12 +4363,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
+          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -4354,12 +4378,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>15.21</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.2812</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4369,24 +4393,24 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K37" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -4394,7 +4418,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4424,7 +4448,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1785577998</t>
+          <t>1785587700</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4434,7 +4458,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>59.143969</t>
+          <t>54.08</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4451,27 +4475,23 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
+          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>6.44999</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.7237</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4479,11 +4499,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4536,7 +4552,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785577962</t>
+          <t>1785585922</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4546,7 +4562,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>82.758621</t>
+          <t>8.911903</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4563,7 +4579,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
+          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4571,19 +4587,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>3.26</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.3225</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4591,26 +4603,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K39" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -4618,7 +4626,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4648,7 +4656,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1785577789</t>
+          <t>1785579524</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4658,7 +4666,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>3.534884</t>
+          <t>4.519931</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4675,7 +4683,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
+          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4683,19 +4691,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>18.99909</t>
+          <t>3.61999</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4703,26 +4707,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K40" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1785577788</t>
+          <t>1785579365</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4770,7 +4770,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>59.141136</t>
+          <t>5.01905</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4787,12 +4787,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
+          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -4802,7 +4802,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -4872,7 +4872,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785577998</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4882,7 +4882,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>6.101167</t>
+          <t>59.143969</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4899,12 +4899,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
+          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -4914,12 +4914,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2.81824</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -4929,24 +4929,24 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K42" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -4954,7 +4954,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785577962</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>8.807</t>
+          <t>82.758621</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5011,7 +5011,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
+          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -5026,12 +5026,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>20.06</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3225</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -5096,7 +5096,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1785576072</t>
+          <t>1785577789</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -5106,7 +5106,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>62.6875</t>
+          <t>3.534884</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5123,7 +5123,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
+          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -5138,12 +5138,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>22.07</t>
+          <t>18.99909</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1785575036</t>
+          <t>1785577788</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -5218,7 +5218,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>68.96875</t>
+          <t>59.141136</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5235,7 +5235,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
+          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5250,12 +5250,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.96</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -5320,7 +5320,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1785574569</t>
+          <t>1785576753</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>3.625</t>
+          <t>6.101167</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5347,7 +5347,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
+          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5362,7 +5362,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>19.25059</t>
+          <t>2.81824</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -5432,7 +5432,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>1785574187</t>
+          <t>1785576753</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>60.158094</t>
+          <t>8.807</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5459,7 +5459,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
+          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5474,7 +5474,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>20.96</t>
+          <t>20.06</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785576072</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
@@ -5554,7 +5554,7 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>65.5</t>
+          <t>62.6875</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5571,7 +5571,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
+          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5586,7 +5586,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2.69</t>
+          <t>22.07</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -5656,7 +5656,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785575036</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -5666,7 +5666,7 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>8.40625</t>
+          <t>68.96875</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -5683,7 +5683,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
+          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5698,7 +5698,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -5768,7 +5768,7 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>1785574073</t>
+          <t>1785574569</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
@@ -5778,7 +5778,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>6.90625</t>
+          <t>3.625</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -5795,7 +5795,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
+          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -5810,7 +5810,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>19.25059</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -5880,7 +5880,7 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>1785573852</t>
+          <t>1785574187</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
@@ -5890,7 +5890,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>6.25</t>
+          <t>60.158094</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -5907,7 +5907,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
+          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -5922,12 +5922,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>20.96</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5992,7 +5992,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>1785570690</t>
+          <t>1785574186</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -6002,7 +6002,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>6.256809</t>
+          <t>65.5</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -6019,7 +6019,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
+          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2.69</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -6104,7 +6104,7 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>1785570471</t>
+          <t>1785574186</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>31.25</t>
+          <t>8.40625</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -6131,7 +6131,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
+          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6139,15 +6139,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>19.72999</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6155,7 +6159,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
       <c r="H53" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -6178,7 +6186,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -6208,7 +6216,7 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>1785569792</t>
+          <t>1785574073</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -6218,7 +6226,7 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>32.544313</t>
+          <t>6.90625</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -6235,7 +6243,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
+          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -6250,7 +6258,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -6320,7 +6328,7 @@
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>1785569076</t>
+          <t>1785573852</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
@@ -6330,7 +6338,7 @@
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>6.59375</t>
+          <t>6.25</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -6347,12 +6355,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
+          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -6362,12 +6370,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.01</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>1.605</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6377,7 +6385,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -6387,27 +6395,27 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298738</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -6432,17 +6440,17 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>1785512959</t>
+          <t>1785570690</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1785592800</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>1.652893</t>
+          <t>6.256809</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -6459,12 +6467,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -6474,12 +6482,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>2.51</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -6489,32 +6497,32 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -6544,7 +6552,7 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>1785497246</t>
+          <t>1785570471</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
@@ -6554,7 +6562,7 @@
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>5.97619</t>
+          <t>31.25</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -6571,27 +6579,23 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>19.72999</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -6599,31 +6603,27 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L57" t="inlineStr">
         <is>
           <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
@@ -6656,7 +6656,7 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>1785346230</t>
+          <t>1785569792</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>2.173913</t>
+          <t>32.544313</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -6683,110 +6683,558 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>1785569076</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>6.59375</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>1.605</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>York City</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>York City vs Crawley Town</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>York City</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Crawley Town</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>L19299060</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>1785512959</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>1785781800</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>1.652893</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>1785497246</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>5.97619</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>1785346230</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>2.173913</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>0xea48d5fe72de69b25067fdb4fdaf1d08ce7262ad75f6855864d3a656da39b313</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>1.46</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F62" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
+      <c r="G62" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
+      <c r="H62" t="inlineStr">
         <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr">
+      <c r="I62" t="inlineStr">
         <is>
           <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
+      <c r="J62" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr">
+      <c r="K62" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="L58" t="inlineStr">
+      <c r="L62" t="inlineStr">
         <is>
           <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr">
+      <c r="M62" t="inlineStr">
         <is>
           <t>L19298738</t>
         </is>
       </c>
-      <c r="N58" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O58" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P58" t="inlineStr">
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q58" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R58" t="inlineStr">
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
         <is>
           <t>1785345250</t>
         </is>
       </c>
-      <c r="S58" t="inlineStr">
+      <c r="S62" t="inlineStr">
         <is>
           <t>1785592800</t>
         </is>
       </c>
-      <c r="T58" t="inlineStr">
+      <c r="T62" t="inlineStr">
         <is>
           <t>2.173913</t>
         </is>
       </c>
-      <c r="U58" t="inlineStr">
+      <c r="U62" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V58" t="inlineStr">
+      <c r="V62" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-06 00:01:33 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/EFL Cup/trades.xlsx
+++ b/data/sxbet/ligas/EFL Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V62"/>
+  <dimension ref="A1:V63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,27 +531,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x4da7133bca54b84184238baa7d30b02372340f739df06b943262742640837a0a</t>
+          <t>0x6f6060f620c519fe84b724f15820ae1a59301dcdb13b16825be361e1751a36ef</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.195</t>
+          <t>1.4425</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -559,11 +555,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Newport County</t>
-        </is>
-      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -571,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>AFC Wimbledon vs Newport County</t>
+          <t>Middlesbrough vs Wrexham</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>AFC Wimbledon</t>
+          <t>Middlesbrough</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Wrexham</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xea47b6c120c94ae31f3299be9d23585a5cbf1b0ada4b3059268dd4cc9712b5d8</t>
+          <t>0xd39b5412e3bdd35c245e5d0a2e08c3b7bbb0dccfab513161aa272b9c72edca35</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19298736</t>
+          <t>L19298910</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785962236</t>
+          <t>1785971523</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786197600</t>
+          <t>1786129200</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>153.846154</t>
+          <t>2.259887</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +635,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xbae8ac7d4c8a6185b820438796f1f9f58ac63f2ed636b3e75be83914f2d44036</t>
+          <t>0x4da7133bca54b84184238baa7d30b02372340f739df06b943262742640837a0a</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -658,12 +650,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.1175</t>
+          <t>1.195</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -673,7 +665,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Walsall</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -683,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Bristol City FC vs Walsall</t>
+          <t>AFC Wimbledon vs Newport County</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Bristol City FC</t>
+          <t>AFC Wimbledon</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Walsall</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xc9a261f972b5555c9a1e6c0f33be8eb6a6906d2cda51babdb51dd64314b2c091</t>
+          <t>0xea47b6c120c94ae31f3299be9d23585a5cbf1b0ada4b3059268dd4cc9712b5d8</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19298734</t>
+          <t>L19298736</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -728,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785961563</t>
+          <t>1785962236</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786041900</t>
+          <t>1786197600</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>85.106383</t>
+          <t>153.846154</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,7 +747,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xdd62398a10f567ee5469950797393093a356b40e7fe5930931a6c998d441d9b9</t>
+          <t>0xbae8ac7d4c8a6185b820438796f1f9f58ac63f2ed636b3e75be83914f2d44036</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -770,12 +762,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.1175</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -785,7 +777,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Cheltenham Town</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -795,27 +787,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Cheltenham Town vs Charlton Athletic</t>
+          <t>Bristol City FC vs Walsall</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Cheltenham Town</t>
+          <t>Bristol City FC</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Charlton Athletic</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x6bf36843abe397fbc7c233e0ca342729b9cd199b53d9ee9a63b96ac9358c9a1a</t>
+          <t>0xc9a261f972b5555c9a1e6c0f33be8eb6a6906d2cda51babdb51dd64314b2c091</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19299406</t>
+          <t>L19298734</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -840,17 +832,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785960783</t>
+          <t>1785961563</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786214700</t>
+          <t>1786041900</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>15.189873</t>
+          <t>85.106383</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,7 +859,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xcb8aa49e12f3f29aa35ec5b7ff00195594f282ca0db4d0d9be5e2e477b96970d</t>
+          <t>0xdd62398a10f567ee5469950797393093a356b40e7fe5930931a6c998d441d9b9</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -882,12 +874,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.1175</t>
+          <t>1.1975</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -897,7 +889,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Walsall</t>
+          <t>Cheltenham Town</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -907,27 +899,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Bristol City FC vs Walsall</t>
+          <t>Cheltenham Town vs Charlton Athletic</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Bristol City FC</t>
+          <t>Cheltenham Town</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Walsall</t>
+          <t>Charlton Athletic</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xc9a261f972b5555c9a1e6c0f33be8eb6a6906d2cda51babdb51dd64314b2c091</t>
+          <t>0x6bf36843abe397fbc7c233e0ca342729b9cd199b53d9ee9a63b96ac9358c9a1a</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19298734</t>
+          <t>L19299406</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -952,17 +944,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785960695</t>
+          <t>1785960783</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786041900</t>
+          <t>1786214700</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>59.574468</t>
+          <t>15.189873</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,12 +971,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x02c4621d6a830534abb9a71c7d2fcc46730afe8d3b686773dfd4c590f2060027</t>
+          <t>0xcb8aa49e12f3f29aa35ec5b7ff00195594f282ca0db4d0d9be5e2e477b96970d</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x204e31304364d2A5f7B90dE28F507adc449Ae221</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -994,22 +986,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>1.1175</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>AFC Wimbledon -1.5</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1019,27 +1011,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>AFC Wimbledon vs Newport County</t>
+          <t>Bristol City FC vs Walsall</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>AFC Wimbledon</t>
+          <t>Bristol City FC</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x9f1f722832eb2e6381f3a0226a98c406eccc5bd7e76caaaebb931fdda305a642</t>
+          <t>0xc9a261f972b5555c9a1e6c0f33be8eb6a6906d2cda51babdb51dd64314b2c091</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19298736</t>
+          <t>L19298734</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1064,17 +1056,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785942153</t>
+          <t>1785960695</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786197600</t>
+          <t>1786041900</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2.941176</t>
+          <t>59.574468</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1091,12 +1083,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xfcba109b300bea480abe542eaa7725c7fec13f0fedc18d9991df424ad450dc90</t>
+          <t>0x02c4621d6a830534abb9a71c7d2fcc46730afe8d3b686773dfd4c590f2060027</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x095B1B11E9C470934404Ba7F04da5F79930b2504</t>
+          <t>0x204e31304364d2A5f7B90dE28F507adc449Ae221</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1106,22 +1098,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>14.58</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>AFC Wimbledon -1.5</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1131,27 +1123,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>AFC Wimbledon vs Newport County</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>AFC Wimbledon</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x30711e53de1ac1c4a025d48c70e4859ee55e52e5e57d10ed46259cc01bb5d46e</t>
+          <t>0x9f1f722832eb2e6381f3a0226a98c406eccc5bd7e76caaaebb931fdda305a642</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298736</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1176,17 +1168,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785778500</t>
+          <t>1785942153</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1786197600</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>2.941176</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1203,12 +1195,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x9b63fb9bdb0939e4fa277441c5160ae767a06c0723ae1697f56722a32c1dbbf4</t>
+          <t>0xfcba109b300bea480abe542eaa7725c7fec13f0fedc18d9991df424ad450dc90</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x095B1B11E9C470934404Ba7F04da5F79930b2504</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1218,39 +1210,39 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.47999</t>
+          <t>14.58</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.5762</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>York City vs Crawley Town</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
           <t>York City</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>York City vs Crawley Town</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>York City</t>
-        </is>
-      </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>Crawley Town</t>
@@ -1258,7 +1250,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0x30711e53de1ac1c4a025d48c70e4859ee55e52e5e57d10ed46259cc01bb5d46e</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1288,7 +1280,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785751617</t>
+          <t>1785778500</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1298,7 +1290,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2.568312</t>
+          <t>18.0</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1315,7 +1307,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x34fd96c52ca66603743b136c029d1196926b8ea965b35ad916e9e624891a3c31</t>
+          <t>0x9b63fb9bdb0939e4fa277441c5160ae767a06c0723ae1697f56722a32c1dbbf4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1323,23 +1315,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.59999</t>
+          <t>1.47999</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.6887</t>
+          <t>1.5762</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>York City</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xb943c3d4cb1b4aebd6296b959eb4168b4f43df52a8043a9e84d184a931ac076c</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785751591</t>
+          <t>1785751617</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>3.77494</t>
+          <t>2.568312</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1419,39 +1419,31 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x92e4361325da8adb7d2c64339dc80666c0b8e0d69bcdd503c9dcdc859b32e858</t>
+          <t>0x34fd96c52ca66603743b136c029d1196926b8ea965b35ad916e9e624891a3c31</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>288.19</t>
+          <t>2.59999</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.555</t>
+          <t>1.6887</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1474,7 +1466,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
+          <t>0xb943c3d4cb1b4aebd6296b959eb4168b4f43df52a8043a9e84d184a931ac076c</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1504,7 +1496,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785746436</t>
+          <t>1785751591</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1514,7 +1506,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>519.261261</t>
+          <t>3.77494</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1531,31 +1523,39 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x2f280a5348c67d22f499a879111a6cd14ba32c30651f4b235087504d75fcb720</t>
+          <t>0x92e4361325da8adb7d2c64339dc80666c0b8e0d69bcdd503c9dcdc859b32e858</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>288.19</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.5263</t>
+          <t>1.555</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
+          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785743240</t>
+          <t>1785746436</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>9.501188</t>
+          <t>519.261261</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1635,7 +1635,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xe649643b38b6c14acf9bbbd3214bd63ce98d37feffda0c872c3665293f137b9c</t>
+          <t>0x2f280a5348c67d22f499a879111a6cd14ba32c30651f4b235087504d75fcb720</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1651,12 +1651,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.3862</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>EFL Cup</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x75d0d882d84fabe75ec0ebfdf953c3267c7e17303f40762904f5aabc9353a5f5</t>
+          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785743239</t>
+          <t>1785743240</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>12.944984</t>
+          <t>9.501188</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1739,7 +1739,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x6da358c7d3a4cfc684658518c8cb0424ee2d0662e048d78a024625d5b4747aed</t>
+          <t>0xe649643b38b6c14acf9bbbd3214bd63ce98d37feffda0c872c3665293f137b9c</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1755,12 +1755,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.5263</t>
+          <t>1.3862</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>EFL Cup</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0x75d0d882d84fabe75ec0ebfdf953c3267c7e17303f40762904f5aabc9353a5f5</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>9.501188</t>
+          <t>12.944984</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1843,7 +1843,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x22ee20a74b7feafe1f674ddfe8f64eb18b48a4aa83ee151db7142c920e3c6990</t>
+          <t>0x6da358c7d3a4cfc684658518c8cb0424ee2d0662e048d78a024625d5b4747aed</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.3862</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1930,7 +1930,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>12.944984</t>
+          <t>9.501188</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1947,7 +1947,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xe3c6c58c8dab85d1b37033a7121e1d3f4c42a16c31fe969f436aa82e973fe331</t>
+          <t>0x22ee20a74b7feafe1f674ddfe8f64eb18b48a4aa83ee151db7142c920e3c6990</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1958,17 +1958,17 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.3862</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2024,7 +2024,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785743238</t>
+          <t>1785743239</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>17.130621</t>
+          <t>12.944984</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2051,7 +2051,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x67892d913ba613f3f4808f12a89e3a4415421d7988b81f5c03035cac2e9e85b1</t>
+          <t>0xe3c6c58c8dab85d1b37033a7121e1d3f4c42a16c31fe969f436aa82e973fe331</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2067,12 +2067,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.445</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -2098,7 +2098,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>22.47191</t>
+          <t>17.130621</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2155,7 +2155,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x51e83e15ab97eefc2ccce2074368f96e4d6b2bc474d60fd48cec81194acc78e8</t>
+          <t>0x67892d913ba613f3f4808f12a89e3a4415421d7988b81f5c03035cac2e9e85b1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2163,11 +2163,7 @@
           <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>10</t>
@@ -2175,19 +2171,15 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.335</t>
+          <t>1.445</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2210,7 +2202,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x1b7328b49fa63aee1bd67882f5cac5a5686aebcb538af0959dcdd4181c5e2f57</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2240,7 +2232,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785742250</t>
+          <t>1785743238</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2250,7 +2242,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>29.850746</t>
+          <t>22.47191</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2267,7 +2259,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x0e0cffe2676af4f324fc06dde5b8beaeded42b973c319bbf3fb70687f8887f41</t>
+          <t>0x51e83e15ab97eefc2ccce2074368f96e4d6b2bc474d60fd48cec81194acc78e8</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2287,17 +2279,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.5587</t>
+          <t>1.335</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2322,7 +2314,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
+          <t>0x1b7328b49fa63aee1bd67882f5cac5a5686aebcb538af0959dcdd4181c5e2f57</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2362,7 +2354,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>17.897092</t>
+          <t>29.850746</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2379,12 +2371,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xb28bdee5a5bd24b5937965869b7830544160fac83e2df3848790121d4082d3d0</t>
+          <t>0x0e0cffe2676af4f324fc06dde5b8beaeded42b973c319bbf3fb70687f8887f41</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2394,22 +2386,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.5587</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2434,7 +2426,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2464,7 +2456,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785741714</t>
+          <t>1785742250</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2474,7 +2466,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>4.020101</t>
+          <t>17.897092</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2491,12 +2483,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xf27c17a15bfe9521fe22971af3d8cd2a8b3c9955888a401e463346a949eb3345</t>
+          <t>0xb28bdee5a5bd24b5937965869b7830544160fac83e2df3848790121d4082d3d0</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2506,22 +2498,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.4438</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2546,7 +2538,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x7c21a171d3ea8b89b468e5886d9b7cec062e0e10cc0a3ad080d701f2e478e0d8</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2576,7 +2568,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785740160</t>
+          <t>1785741714</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2586,7 +2578,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>22.535211</t>
+          <t>4.020101</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2603,12 +2595,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
+          <t>0xf27c17a15bfe9521fe22971af3d8cd2a8b3c9955888a401e463346a949eb3345</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2618,22 +2610,22 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.2475</t>
+          <t>1.4438</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2658,7 +2650,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0x7c21a171d3ea8b89b468e5886d9b7cec062e0e10cc0a3ad080d701f2e478e0d8</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2688,7 +2680,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785729810</t>
+          <t>1785740160</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2698,7 +2690,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>4.040404</t>
+          <t>22.535211</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2715,7 +2707,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
+          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2730,12 +2722,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>3.99987</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.2475</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2800,7 +2792,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785729635</t>
+          <t>1785729810</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2810,7 +2802,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>16.079879</t>
+          <t>4.040404</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2827,7 +2819,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
+          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2842,12 +2834,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>23.26</t>
+          <t>3.99987</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.4338</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2867,27 +2859,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2912,17 +2904,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785597225</t>
+          <t>1785729635</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>53.62536</t>
+          <t>16.079879</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2939,7 +2931,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
+          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2954,12 +2946,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>23.26</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2969,32 +2961,32 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3024,7 +3016,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785595661</t>
+          <t>1785597225</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3034,7 +3026,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>3.11284</t>
+          <t>53.62536</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3051,7 +3043,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
+          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3066,12 +3058,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3136,7 +3128,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785594340</t>
+          <t>1785595661</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3146,7 +3138,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>27.777778</t>
+          <t>3.11284</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3163,7 +3155,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
+          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3183,7 +3175,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3248,7 +3240,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785593884</t>
+          <t>1785594340</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3258,7 +3250,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>27.777778</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3275,7 +3267,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
+          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3387,7 +3379,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
+          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3402,12 +3394,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>25.04</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.385</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3472,7 +3464,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785593611</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3482,7 +3474,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>65.038961</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3499,7 +3491,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
+          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3514,12 +3506,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>25.04</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.2375</t>
+          <t>1.385</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3529,7 +3521,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3554,7 +3546,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3584,7 +3576,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785593186</t>
+          <t>1785593611</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3594,7 +3586,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>49.263158</t>
+          <t>65.038961</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3611,7 +3603,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
+          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3626,12 +3618,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.2375</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3641,32 +3633,32 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3696,7 +3688,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785592744</t>
+          <t>1785593186</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3706,7 +3698,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>7.088608</t>
+          <t>49.263158</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3723,7 +3715,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
+          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3738,7 +3730,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3.59</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3808,7 +3800,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785592658</t>
+          <t>1785592744</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3818,7 +3810,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>9.088608</t>
+          <t>7.088608</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3835,7 +3827,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
+          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3850,7 +3842,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>22.05</t>
+          <t>3.59</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3920,7 +3912,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785592637</t>
+          <t>1785592658</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3930,7 +3922,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>55.822785</t>
+          <t>9.088608</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3947,7 +3939,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
+          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3955,15 +3947,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>36.31948</t>
+          <t>22.05</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3971,7 +3967,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4024,7 +4024,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785589857</t>
+          <t>1785592637</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -4034,7 +4034,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>58.816972</t>
+          <t>55.822785</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4051,7 +4051,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
+          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4062,7 +4062,7 @@
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>36.31948</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -4128,7 +4128,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785589600</t>
+          <t>1785589857</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4138,7 +4138,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>6.54251</t>
+          <t>58.816972</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4155,7 +4155,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
+          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4166,12 +4166,12 @@
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>18.36999</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.615</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4232,7 +4232,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785589491</t>
+          <t>1785589600</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4242,7 +4242,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>29.869902</t>
+          <t>6.54251</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4259,7 +4259,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
+          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4270,12 +4270,12 @@
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>18.54999</t>
+          <t>18.36999</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.615</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785588508</t>
+          <t>1785589491</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4346,7 +4346,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>30.597922</t>
+          <t>29.869902</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4363,27 +4363,23 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
+          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>15.21</t>
+          <t>18.54999</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4391,11 +4387,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4418,7 +4410,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4448,7 +4440,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1785587700</t>
+          <t>1785588508</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4458,7 +4450,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>54.08</t>
+          <t>30.597922</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4475,23 +4467,27 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
+          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>6.44999</t>
+          <t>15.21</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.7237</t>
+          <t>1.2812</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4499,7 +4495,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4552,7 +4552,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785585922</t>
+          <t>1785587700</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>8.911903</t>
+          <t>54.08</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4579,7 +4579,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
+          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4590,12 +4590,12 @@
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3.26</t>
+          <t>6.44999</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.7212</t>
+          <t>1.7237</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1785579524</t>
+          <t>1785585922</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>4.519931</t>
+          <t>8.911903</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4683,7 +4683,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
+          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4694,7 +4694,7 @@
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>3.61999</t>
+          <t>3.26</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1785579365</t>
+          <t>1785579524</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4770,7 +4770,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>5.01905</t>
+          <t>4.519931</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4787,27 +4787,23 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
+          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>3.61999</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4815,26 +4811,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K41" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -4842,7 +4834,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -4872,7 +4864,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1785577998</t>
+          <t>1785579365</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4882,7 +4874,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>59.143969</t>
+          <t>5.01905</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4899,7 +4891,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
+          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4914,12 +4906,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -4929,7 +4921,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -4954,7 +4946,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -4984,7 +4976,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1785577962</t>
+          <t>1785577998</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -4994,7 +4986,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>82.758621</t>
+          <t>59.143969</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5011,12 +5003,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
+          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -5026,12 +5018,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.3225</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -5041,24 +5033,24 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K43" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -5066,7 +5058,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -5096,7 +5088,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1785577789</t>
+          <t>1785577962</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -5106,7 +5098,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>3.534884</t>
+          <t>82.758621</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5123,7 +5115,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
+          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -5138,12 +5130,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>18.99909</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.3225</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -5208,7 +5200,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1785577788</t>
+          <t>1785577789</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -5218,7 +5210,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>59.141136</t>
+          <t>3.534884</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5235,7 +5227,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
+          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5250,7 +5242,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>18.99909</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -5320,7 +5312,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785577788</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -5330,7 +5322,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>6.101167</t>
+          <t>59.141136</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5347,7 +5339,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
+          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5362,12 +5354,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2.81824</t>
+          <t>1.96</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -5442,7 +5434,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>8.807</t>
+          <t>6.101167</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5459,7 +5451,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
+          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5474,7 +5466,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>20.06</t>
+          <t>2.81824</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -5544,7 +5536,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1785576072</t>
+          <t>1785576753</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
@@ -5554,7 +5546,7 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>62.6875</t>
+          <t>8.807</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5571,7 +5563,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
+          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5586,7 +5578,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>22.07</t>
+          <t>20.06</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -5656,7 +5648,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>1785575036</t>
+          <t>1785576072</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -5666,7 +5658,7 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>68.96875</t>
+          <t>62.6875</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -5683,7 +5675,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
+          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5698,7 +5690,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>22.07</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -5768,7 +5760,7 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>1785574569</t>
+          <t>1785575036</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
@@ -5778,7 +5770,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>3.625</t>
+          <t>68.96875</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -5795,7 +5787,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
+          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -5810,7 +5802,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>19.25059</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -5880,7 +5872,7 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>1785574187</t>
+          <t>1785574569</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
@@ -5890,7 +5882,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>60.158094</t>
+          <t>3.625</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -5907,7 +5899,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
+          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -5922,7 +5914,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>20.96</t>
+          <t>19.25059</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -5992,7 +5984,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785574187</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -6002,7 +5994,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>65.5</t>
+          <t>60.158094</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -6019,7 +6011,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
+          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6034,7 +6026,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>2.69</t>
+          <t>20.96</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -6114,7 +6106,7 @@
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>8.40625</t>
+          <t>65.5</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -6131,7 +6123,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
+          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6146,7 +6138,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>2.69</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -6216,7 +6208,7 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>1785574073</t>
+          <t>1785574186</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -6226,7 +6218,7 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>6.90625</t>
+          <t>8.40625</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -6243,7 +6235,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
+          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -6258,7 +6250,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -6328,7 +6320,7 @@
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>1785573852</t>
+          <t>1785574073</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
@@ -6338,7 +6330,7 @@
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>6.25</t>
+          <t>6.90625</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -6355,7 +6347,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
+          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -6370,12 +6362,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6440,7 +6432,7 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>1785570690</t>
+          <t>1785573852</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
@@ -6450,7 +6442,7 @@
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>6.256809</t>
+          <t>6.25</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -6467,7 +6459,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
+          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -6482,12 +6474,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2.01</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -6552,7 +6544,7 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>1785570471</t>
+          <t>1785570690</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
@@ -6562,7 +6554,7 @@
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>31.25</t>
+          <t>6.256809</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -6579,7 +6571,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
+          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -6587,15 +6579,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>19.72999</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -6603,7 +6599,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
       <c r="H57" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -6626,7 +6626,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>1785569792</t>
+          <t>1785570471</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>32.544313</t>
+          <t>31.25</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -6683,7 +6683,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
+          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -6691,19 +6691,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>19.72999</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -6711,26 +6707,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K58" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -6738,7 +6730,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
@@ -6768,7 +6760,7 @@
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>1785569076</t>
+          <t>1785569792</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
@@ -6778,7 +6770,7 @@
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>6.59375</t>
+          <t>32.544313</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
@@ -6795,12 +6787,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
+          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -6810,12 +6802,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.11</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>1.605</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -6825,7 +6817,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -6835,27 +6827,27 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298738</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -6880,17 +6872,17 @@
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>1785512959</t>
+          <t>1785569076</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1785592800</t>
         </is>
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>1.652893</t>
+          <t>6.59375</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
@@ -6907,12 +6899,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -6922,12 +6914,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>2.51</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.605</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -6937,7 +6929,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -6947,27 +6939,27 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -6992,17 +6984,17 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>1785497246</t>
+          <t>1785512959</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T60" t="inlineStr">
         <is>
-          <t>5.97619</t>
+          <t>1.652893</t>
         </is>
       </c>
       <c r="U60" t="inlineStr">
@@ -7019,12 +7011,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -7034,12 +7026,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.51</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -7104,7 +7096,7 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>1785346230</t>
+          <t>1785497246</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
@@ -7114,7 +7106,7 @@
       </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>2.173913</t>
+          <t>5.97619</t>
         </is>
       </c>
       <c r="U61" t="inlineStr">
@@ -7131,110 +7123,222 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>1785346230</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>2.173913</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>0xea48d5fe72de69b25067fdb4fdaf1d08ce7262ad75f6855864d3a656da39b313</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
         <is>
           <t>1.46</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="F63" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
+      <c r="G63" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr">
+      <c r="H63" t="inlineStr">
         <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr">
+      <c r="I63" t="inlineStr">
         <is>
           <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr">
+      <c r="J63" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr">
+      <c r="K63" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="L62" t="inlineStr">
+      <c r="L63" t="inlineStr">
         <is>
           <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr">
+      <c r="M63" t="inlineStr">
         <is>
           <t>L19298738</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O62" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P62" t="inlineStr">
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q62" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R62" t="inlineStr">
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
         <is>
           <t>1785345250</t>
         </is>
       </c>
-      <c r="S62" t="inlineStr">
+      <c r="S63" t="inlineStr">
         <is>
           <t>1785592800</t>
         </is>
       </c>
-      <c r="T62" t="inlineStr">
+      <c r="T63" t="inlineStr">
         <is>
           <t>2.173913</t>
         </is>
       </c>
-      <c r="U62" t="inlineStr">
+      <c r="U63" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V62" t="inlineStr">
+      <c r="V63" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-06 03:01:52 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/EFL Cup/trades.xlsx
+++ b/data/sxbet/ligas/EFL Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V63"/>
+  <dimension ref="A1:V65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,28 +531,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x6f6060f620c519fe84b724f15820ae1a59301dcdb13b16825be361e1751a36ef</t>
+          <t>0x9eeed2b966213cd3e1c03ecd18ebae97e3bdccaa3b690be36f141b37998d5271</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0x1aD0dE948858F4DeaCBEa7b44be9459c1486b543</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15.02343</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.4425</t>
+          <t>1.8013</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (4.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -563,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Middlesbrough vs Wrexham</t>
+          <t>Cardiff City vs Swindon Town</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Middlesbrough</t>
+          <t>Cardiff City</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Wrexham</t>
+          <t>Swindon Town</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xd39b5412e3bdd35c245e5d0a2e08c3b7bbb0dccfab513161aa272b9c72edca35</t>
+          <t>0xb537cfe2d0e516b2ff03db523f6c643dabb99be113085ba2d6af88754af7464c</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19298910</t>
+          <t>L19299400</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785971523</t>
+          <t>1785985128</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786129200</t>
+          <t>1786197600</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2.259887</t>
+          <t>18.749991</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,12 +635,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x4da7133bca54b84184238baa7d30b02372340f739df06b943262742640837a0a</t>
+          <t>0x5fbf0f7a0310f9abc0793e9101a9adc8673eb773a7cc1d40c6daae6c36914fb2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+          <t>0xa3786b93377213A42Bf1d3261d373cE67Cf2AA67</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -650,12 +650,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>24.21</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.195</t>
+          <t>1.0825</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -675,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>AFC Wimbledon vs Newport County</t>
+          <t>Watford vs Crawley Town</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>AFC Wimbledon</t>
+          <t>Watford</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xea47b6c120c94ae31f3299be9d23585a5cbf1b0ada4b3059268dd4cc9712b5d8</t>
+          <t>0x5d9b97d51b6818d3cd9824517a3ea8f42d223346ae6156eded748cbedb8f386f</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19298736</t>
+          <t>L19692421</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785962236</t>
+          <t>1785978809</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>153.846154</t>
+          <t>293.454545</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,27 +747,23 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xbae8ac7d4c8a6185b820438796f1f9f58ac63f2ed636b3e75be83914f2d44036</t>
+          <t>0x6f6060f620c519fe84b724f15820ae1a59301dcdb13b16825be361e1751a36ef</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.1175</t>
+          <t>1.4425</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -775,11 +771,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Walsall</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -787,27 +779,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Bristol City FC vs Walsall</t>
+          <t>Middlesbrough vs Wrexham</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Bristol City FC</t>
+          <t>Middlesbrough</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Walsall</t>
+          <t>Wrexham</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xc9a261f972b5555c9a1e6c0f33be8eb6a6906d2cda51babdb51dd64314b2c091</t>
+          <t>0xd39b5412e3bdd35c245e5d0a2e08c3b7bbb0dccfab513161aa272b9c72edca35</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19298734</t>
+          <t>L19298910</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,17 +824,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785961563</t>
+          <t>1785971523</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786041900</t>
+          <t>1786129200</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>85.106383</t>
+          <t>2.259887</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,7 +851,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xdd62398a10f567ee5469950797393093a356b40e7fe5930931a6c998d441d9b9</t>
+          <t>0x4da7133bca54b84184238baa7d30b02372340f739df06b943262742640837a0a</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -874,12 +866,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.195</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -889,7 +881,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Cheltenham Town</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -899,27 +891,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Cheltenham Town vs Charlton Athletic</t>
+          <t>AFC Wimbledon vs Newport County</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Cheltenham Town</t>
+          <t>AFC Wimbledon</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Charlton Athletic</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x6bf36843abe397fbc7c233e0ca342729b9cd199b53d9ee9a63b96ac9358c9a1a</t>
+          <t>0xea47b6c120c94ae31f3299be9d23585a5cbf1b0ada4b3059268dd4cc9712b5d8</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19299406</t>
+          <t>L19298736</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,17 +936,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785960783</t>
+          <t>1785962236</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786214700</t>
+          <t>1786197600</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>15.189873</t>
+          <t>153.846154</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,7 +963,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xcb8aa49e12f3f29aa35ec5b7ff00195594f282ca0db4d0d9be5e2e477b96970d</t>
+          <t>0xbae8ac7d4c8a6185b820438796f1f9f58ac63f2ed636b3e75be83914f2d44036</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -986,7 +978,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1056,7 +1048,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785960695</t>
+          <t>1785961563</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1058,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>59.574468</t>
+          <t>85.106383</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,12 +1075,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x02c4621d6a830534abb9a71c7d2fcc46730afe8d3b686773dfd4c590f2060027</t>
+          <t>0xdd62398a10f567ee5469950797393093a356b40e7fe5930931a6c998d441d9b9</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x204e31304364d2A5f7B90dE28F507adc449Ae221</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1098,22 +1090,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>1.1975</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>AFC Wimbledon -1.5</t>
+          <t>Cheltenham Town</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1123,27 +1115,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>AFC Wimbledon vs Newport County</t>
+          <t>Cheltenham Town vs Charlton Athletic</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>AFC Wimbledon</t>
+          <t>Cheltenham Town</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Charlton Athletic</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x9f1f722832eb2e6381f3a0226a98c406eccc5bd7e76caaaebb931fdda305a642</t>
+          <t>0x6bf36843abe397fbc7c233e0ca342729b9cd199b53d9ee9a63b96ac9358c9a1a</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19298736</t>
+          <t>L19299406</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1168,17 +1160,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785942153</t>
+          <t>1785960783</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786197600</t>
+          <t>1786214700</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2.941176</t>
+          <t>15.189873</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1195,12 +1187,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xfcba109b300bea480abe542eaa7725c7fec13f0fedc18d9991df424ad450dc90</t>
+          <t>0xcb8aa49e12f3f29aa35ec5b7ff00195594f282ca0db4d0d9be5e2e477b96970d</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x095B1B11E9C470934404Ba7F04da5F79930b2504</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1210,22 +1202,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>14.58</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.1175</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1235,27 +1227,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Bristol City FC vs Walsall</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Bristol City FC</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x30711e53de1ac1c4a025d48c70e4859ee55e52e5e57d10ed46259cc01bb5d46e</t>
+          <t>0xc9a261f972b5555c9a1e6c0f33be8eb6a6906d2cda51babdb51dd64314b2c091</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298734</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1280,17 +1272,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785778500</t>
+          <t>1785960695</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1786041900</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>59.574468</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1307,12 +1299,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x9b63fb9bdb0939e4fa277441c5160ae767a06c0723ae1697f56722a32c1dbbf4</t>
+          <t>0x02c4621d6a830534abb9a71c7d2fcc46730afe8d3b686773dfd4c590f2060027</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x204e31304364d2A5f7B90dE28F507adc449Ae221</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1322,22 +1314,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.47999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.5762</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>AFC Wimbledon -1.5</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1347,27 +1339,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>AFC Wimbledon vs Newport County</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>AFC Wimbledon</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0x9f1f722832eb2e6381f3a0226a98c406eccc5bd7e76caaaebb931fdda305a642</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298736</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1392,17 +1384,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785751617</t>
+          <t>1785942153</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1786197600</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2.568312</t>
+          <t>2.941176</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1419,31 +1411,39 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x34fd96c52ca66603743b136c029d1196926b8ea965b35ad916e9e624891a3c31</t>
+          <t>0xfcba109b300bea480abe542eaa7725c7fec13f0fedc18d9991df424ad450dc90</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+          <t>0x095B1B11E9C470934404Ba7F04da5F79930b2504</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.59999</t>
+          <t>14.58</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.6887</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1466,7 +1466,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xb943c3d4cb1b4aebd6296b959eb4168b4f43df52a8043a9e84d184a931ac076c</t>
+          <t>0x30711e53de1ac1c4a025d48c70e4859ee55e52e5e57d10ed46259cc01bb5d46e</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785751591</t>
+          <t>1785778500</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>3.77494</t>
+          <t>18.0</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1523,12 +1523,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x92e4361325da8adb7d2c64339dc80666c0b8e0d69bcdd503c9dcdc859b32e858</t>
+          <t>0x9b63fb9bdb0939e4fa277441c5160ae767a06c0723ae1697f56722a32c1dbbf4</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1538,22 +1538,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>288.19</t>
+          <t>1.47999</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.555</t>
+          <t>1.5762</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785746436</t>
+          <t>1785751617</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>519.261261</t>
+          <t>2.568312</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1635,28 +1635,28 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x2f280a5348c67d22f499a879111a6cd14ba32c30651f4b235087504d75fcb720</t>
+          <t>0x34fd96c52ca66603743b136c029d1196926b8ea965b35ad916e9e624891a3c31</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2.59999</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.5263</t>
+          <t>1.6887</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
+          <t>0xb943c3d4cb1b4aebd6296b959eb4168b4f43df52a8043a9e84d184a931ac076c</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785743240</t>
+          <t>1785751591</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>9.501188</t>
+          <t>3.77494</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1739,36 +1739,44 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xe649643b38b6c14acf9bbbd3214bd63ce98d37feffda0c872c3665293f137b9c</t>
+          <t>0x92e4361325da8adb7d2c64339dc80666c0b8e0d69bcdd503c9dcdc859b32e858</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>288.19</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.3862</t>
+          <t>1.555</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
           <t>York City vs Crawley Town</t>
@@ -1786,7 +1794,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x75d0d882d84fabe75ec0ebfdf953c3267c7e17303f40762904f5aabc9353a5f5</t>
+          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1816,7 +1824,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785743239</t>
+          <t>1785746436</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1826,7 +1834,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>12.944984</t>
+          <t>519.261261</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1843,7 +1851,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x6da358c7d3a4cfc684658518c8cb0424ee2d0662e048d78a024625d5b4747aed</t>
+          <t>0x2f280a5348c67d22f499a879111a6cd14ba32c30651f4b235087504d75fcb720</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1864,7 +1872,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1890,7 +1898,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1920,7 +1928,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785743239</t>
+          <t>1785743240</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1947,7 +1955,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x22ee20a74b7feafe1f674ddfe8f64eb18b48a4aa83ee151db7142c920e3c6990</t>
+          <t>0xe649643b38b6c14acf9bbbd3214bd63ce98d37feffda0c872c3665293f137b9c</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1968,7 +1976,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>EFL Cup</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1994,7 +2002,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0x75d0d882d84fabe75ec0ebfdf953c3267c7e17303f40762904f5aabc9353a5f5</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2051,7 +2059,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xe3c6c58c8dab85d1b37033a7121e1d3f4c42a16c31fe969f436aa82e973fe331</t>
+          <t>0x6da358c7d3a4cfc684658518c8cb0424ee2d0662e048d78a024625d5b4747aed</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2062,17 +2070,17 @@
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -2098,7 +2106,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2128,7 +2136,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785743238</t>
+          <t>1785743239</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2138,7 +2146,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>17.130621</t>
+          <t>9.501188</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2155,7 +2163,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x67892d913ba613f3f4808f12a89e3a4415421d7988b81f5c03035cac2e9e85b1</t>
+          <t>0x22ee20a74b7feafe1f674ddfe8f64eb18b48a4aa83ee151db7142c920e3c6990</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2166,12 +2174,12 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.445</t>
+          <t>1.3862</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2232,7 +2240,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785743238</t>
+          <t>1785743239</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2242,7 +2250,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>22.47191</t>
+          <t>12.944984</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2259,7 +2267,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x51e83e15ab97eefc2ccce2074368f96e4d6b2bc474d60fd48cec81194acc78e8</t>
+          <t>0xe3c6c58c8dab85d1b37033a7121e1d3f4c42a16c31fe969f436aa82e973fe331</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2267,11 +2275,7 @@
           <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>10</t>
@@ -2279,19 +2283,15 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.335</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2314,7 +2314,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x1b7328b49fa63aee1bd67882f5cac5a5686aebcb538af0959dcdd4181c5e2f57</t>
+          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785742250</t>
+          <t>1785743238</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>29.850746</t>
+          <t>17.130621</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2371,7 +2371,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x0e0cffe2676af4f324fc06dde5b8beaeded42b973c319bbf3fb70687f8887f41</t>
+          <t>0x67892d913ba613f3f4808f12a89e3a4415421d7988b81f5c03035cac2e9e85b1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2379,11 +2379,7 @@
           <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>10</t>
@@ -2391,19 +2387,15 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.5587</t>
+          <t>1.445</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2426,7 +2418,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2456,7 +2448,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785742250</t>
+          <t>1785743238</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2466,7 +2458,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>17.897092</t>
+          <t>22.47191</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2483,12 +2475,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xb28bdee5a5bd24b5937965869b7830544160fac83e2df3848790121d4082d3d0</t>
+          <t>0x51e83e15ab97eefc2ccce2074368f96e4d6b2bc474d60fd48cec81194acc78e8</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2498,22 +2490,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.335</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2538,7 +2530,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0x1b7328b49fa63aee1bd67882f5cac5a5686aebcb538af0959dcdd4181c5e2f57</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2568,7 +2560,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785741714</t>
+          <t>1785742250</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2578,7 +2570,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>4.020101</t>
+          <t>29.850746</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2595,7 +2587,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xf27c17a15bfe9521fe22971af3d8cd2a8b3c9955888a401e463346a949eb3345</t>
+          <t>0x0e0cffe2676af4f324fc06dde5b8beaeded42b973c319bbf3fb70687f8887f41</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2615,17 +2607,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.4438</t>
+          <t>1.5587</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2650,7 +2642,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x7c21a171d3ea8b89b468e5886d9b7cec062e0e10cc0a3ad080d701f2e478e0d8</t>
+          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2680,7 +2672,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785740160</t>
+          <t>1785742250</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2690,7 +2682,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>22.535211</t>
+          <t>17.897092</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2707,7 +2699,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
+          <t>0xb28bdee5a5bd24b5937965869b7830544160fac83e2df3848790121d4082d3d0</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2727,7 +2719,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.2475</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2792,7 +2784,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785729810</t>
+          <t>1785741714</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2802,7 +2794,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>4.040404</t>
+          <t>4.020101</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2819,12 +2811,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
+          <t>0xf27c17a15bfe9521fe22971af3d8cd2a8b3c9955888a401e463346a949eb3345</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2834,22 +2826,22 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3.99987</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.4438</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2874,7 +2866,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0x7c21a171d3ea8b89b468e5886d9b7cec062e0e10cc0a3ad080d701f2e478e0d8</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2904,7 +2896,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785729635</t>
+          <t>1785740160</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2914,7 +2906,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>16.079879</t>
+          <t>22.535211</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2931,7 +2923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
+          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2946,12 +2938,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>23.26</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.4338</t>
+          <t>1.2475</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2971,27 +2963,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -3016,17 +3008,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785597225</t>
+          <t>1785729810</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>53.62536</t>
+          <t>4.040404</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3043,7 +3035,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
+          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3058,12 +3050,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3.99987</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3073,7 +3065,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -3083,27 +3075,27 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -3128,17 +3120,17 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785595661</t>
+          <t>1785729635</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>3.11284</t>
+          <t>16.079879</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3155,7 +3147,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
+          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3170,12 +3162,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>23.26</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3185,32 +3177,32 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3240,7 +3232,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785594340</t>
+          <t>1785597225</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3250,7 +3242,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>27.777778</t>
+          <t>53.62536</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3267,7 +3259,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
+          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3282,12 +3274,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3352,7 +3344,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785593884</t>
+          <t>1785595661</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3362,7 +3354,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>3.11284</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3379,7 +3371,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
+          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3399,7 +3391,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3464,7 +3456,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785593884</t>
+          <t>1785594340</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3474,7 +3466,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>27.777778</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3491,7 +3483,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
+          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3506,12 +3498,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>25.04</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.385</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3576,7 +3568,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785593611</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3586,7 +3578,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>65.038961</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3603,7 +3595,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
+          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3618,12 +3610,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.2375</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3633,7 +3625,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3658,7 +3650,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3688,7 +3680,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785593186</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3698,7 +3690,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>49.263158</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3715,7 +3707,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
+          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3730,12 +3722,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>25.04</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.385</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3800,7 +3792,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785592744</t>
+          <t>1785593611</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3810,7 +3802,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>7.088608</t>
+          <t>65.038961</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3827,7 +3819,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
+          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3842,12 +3834,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>3.59</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.2375</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3857,32 +3849,32 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3912,7 +3904,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785592658</t>
+          <t>1785593186</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3922,7 +3914,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>9.088608</t>
+          <t>49.263158</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3939,7 +3931,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
+          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3954,7 +3946,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>22.05</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -4024,7 +4016,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785592637</t>
+          <t>1785592744</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -4034,7 +4026,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>55.822785</t>
+          <t>7.088608</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4051,7 +4043,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
+          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4059,15 +4051,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>36.31948</t>
+          <t>3.59</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4075,7 +4071,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785589857</t>
+          <t>1785592658</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4138,7 +4138,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>58.816972</t>
+          <t>9.088608</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4155,7 +4155,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
+          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4163,15 +4163,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>22.05</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4179,7 +4183,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4232,7 +4240,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785589600</t>
+          <t>1785592637</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4242,7 +4250,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>6.54251</t>
+          <t>55.822785</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4259,7 +4267,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
+          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4270,12 +4278,12 @@
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>18.36999</t>
+          <t>36.31948</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.615</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4336,7 +4344,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785589491</t>
+          <t>1785589857</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4346,7 +4354,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>29.869902</t>
+          <t>58.816972</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4363,7 +4371,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
+          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4374,12 +4382,12 @@
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>18.54999</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4440,7 +4448,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1785588508</t>
+          <t>1785589600</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4450,7 +4458,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>30.597922</t>
+          <t>6.54251</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4467,27 +4475,23 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
+          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>15.21</t>
+          <t>18.36999</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.615</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4495,11 +4499,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4522,7 +4522,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4552,7 +4552,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785587700</t>
+          <t>1785589491</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>54.08</t>
+          <t>29.869902</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4579,7 +4579,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
+          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4590,12 +4590,12 @@
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>6.44999</t>
+          <t>18.54999</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.7237</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4626,7 +4626,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1785585922</t>
+          <t>1785588508</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>8.911903</t>
+          <t>30.597922</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4683,23 +4683,27 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
+          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>3.26</t>
+          <t>15.21</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.7212</t>
+          <t>1.2812</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4707,7 +4711,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4760,7 +4768,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1785579524</t>
+          <t>1785587700</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4770,7 +4778,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>4.519931</t>
+          <t>54.08</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4787,7 +4795,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
+          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4798,12 +4806,12 @@
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>3.61999</t>
+          <t>6.44999</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.7212</t>
+          <t>1.7237</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4864,7 +4872,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1785579365</t>
+          <t>1785585922</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4874,7 +4882,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>5.01905</t>
+          <t>8.911903</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4891,27 +4899,23 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
+          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>3.26</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -4919,26 +4923,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K42" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -4946,7 +4946,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -4976,7 +4976,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1785577998</t>
+          <t>1785579524</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -4986,7 +4986,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>59.143969</t>
+          <t>4.519931</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5003,27 +5003,23 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
+          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>3.61999</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -5031,11 +5027,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -5088,7 +5080,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1785577962</t>
+          <t>1785579365</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -5098,7 +5090,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>82.758621</t>
+          <t>5.01905</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5115,12 +5107,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
+          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -5130,12 +5122,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.3225</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -5200,7 +5192,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1785577789</t>
+          <t>1785577998</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -5210,7 +5202,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>3.534884</t>
+          <t>59.143969</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5227,12 +5219,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
+          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -5242,12 +5234,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>18.99909</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -5257,24 +5249,24 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K45" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -5282,7 +5274,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -5312,7 +5304,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1785577788</t>
+          <t>1785577962</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -5322,7 +5314,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>59.141136</t>
+          <t>82.758621</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5339,7 +5331,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
+          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5354,12 +5346,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.3225</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -5424,7 +5416,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785577789</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -5434,7 +5426,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>6.101167</t>
+          <t>3.534884</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5451,7 +5443,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
+          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5466,12 +5458,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2.81824</t>
+          <t>18.99909</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5536,7 +5528,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785577788</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
@@ -5546,7 +5538,7 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>8.807</t>
+          <t>59.141136</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5563,7 +5555,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
+          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5578,12 +5570,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>20.06</t>
+          <t>1.96</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5648,7 +5640,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>1785576072</t>
+          <t>1785576753</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -5658,7 +5650,7 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>62.6875</t>
+          <t>6.101167</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -5675,7 +5667,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
+          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5690,7 +5682,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>22.07</t>
+          <t>2.81824</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -5760,7 +5752,7 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>1785575036</t>
+          <t>1785576753</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
@@ -5770,7 +5762,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>68.96875</t>
+          <t>8.807</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -5787,7 +5779,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
+          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -5802,7 +5794,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>20.06</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -5872,7 +5864,7 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>1785574569</t>
+          <t>1785576072</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
@@ -5882,7 +5874,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>3.625</t>
+          <t>62.6875</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -5899,7 +5891,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
+          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -5914,7 +5906,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>19.25059</t>
+          <t>22.07</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -5984,7 +5976,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>1785574187</t>
+          <t>1785575036</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -5994,7 +5986,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>60.158094</t>
+          <t>68.96875</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -6011,7 +6003,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
+          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6026,7 +6018,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>20.96</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -6096,7 +6088,7 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785574569</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
@@ -6106,7 +6098,7 @@
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>65.5</t>
+          <t>3.625</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -6123,7 +6115,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
+          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6138,7 +6130,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2.69</t>
+          <t>19.25059</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -6208,7 +6200,7 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785574187</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -6218,7 +6210,7 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>8.40625</t>
+          <t>60.158094</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -6235,7 +6227,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
+          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -6250,7 +6242,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>20.96</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -6320,7 +6312,7 @@
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>1785574073</t>
+          <t>1785574186</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
@@ -6330,7 +6322,7 @@
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>6.90625</t>
+          <t>65.5</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -6347,7 +6339,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
+          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -6362,7 +6354,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.69</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -6432,7 +6424,7 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>1785573852</t>
+          <t>1785574186</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
@@ -6442,7 +6434,7 @@
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>6.25</t>
+          <t>8.40625</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -6459,7 +6451,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
+          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -6474,12 +6466,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -6544,7 +6536,7 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>1785570690</t>
+          <t>1785574073</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
@@ -6554,7 +6546,7 @@
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>6.256809</t>
+          <t>6.90625</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -6571,7 +6563,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
+          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -6586,7 +6578,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -6656,7 +6648,7 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>1785570471</t>
+          <t>1785573852</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
@@ -6666,7 +6658,7 @@
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>31.25</t>
+          <t>6.25</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -6683,7 +6675,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
+          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -6691,15 +6683,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>19.72999</t>
+          <t>2.01</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -6707,7 +6703,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
       <c r="H58" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -6730,7 +6730,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>1785569792</t>
+          <t>1785570690</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
@@ -6770,7 +6770,7 @@
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>32.544313</t>
+          <t>6.256809</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
@@ -6787,7 +6787,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
+          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -6802,7 +6802,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -6872,7 +6872,7 @@
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>1785569076</t>
+          <t>1785570471</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
@@ -6882,7 +6882,7 @@
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>6.59375</t>
+          <t>31.25</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
@@ -6899,27 +6899,23 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
+          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>19.72999</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>1.605</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -6927,11 +6923,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>York City</t>
-        </is>
-      </c>
+      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -6939,27 +6931,27 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298738</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -6984,17 +6976,17 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>1785512959</t>
+          <t>1785569792</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1785592800</t>
         </is>
       </c>
       <c r="T60" t="inlineStr">
         <is>
-          <t>1.652893</t>
+          <t>32.544313</t>
         </is>
       </c>
       <c r="U60" t="inlineStr">
@@ -7011,12 +7003,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -7026,12 +7018,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>2.51</t>
+          <t>2.11</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -7041,32 +7033,32 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -7096,7 +7088,7 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>1785497246</t>
+          <t>1785569076</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
@@ -7106,7 +7098,7 @@
       </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>5.97619</t>
+          <t>6.59375</t>
         </is>
       </c>
       <c r="U61" t="inlineStr">
@@ -7123,7 +7115,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -7143,7 +7135,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>1.605</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -7153,7 +7145,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -7163,27 +7155,27 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -7208,17 +7200,17 @@
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>1785346230</t>
+          <t>1785512959</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T62" t="inlineStr">
         <is>
-          <t>2.173913</t>
+          <t>1.652893</t>
         </is>
       </c>
       <c r="U62" t="inlineStr">
@@ -7235,110 +7227,334 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
+          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>1785497246</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>5.97619</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>1785346230</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>2.173913</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
           <t>0xea48d5fe72de69b25067fdb4fdaf1d08ce7262ad75f6855864d3a656da39b313</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
         <is>
           <t>1.46</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F65" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr">
+      <c r="G65" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
+      <c r="H65" t="inlineStr">
         <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr">
+      <c r="I65" t="inlineStr">
         <is>
           <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr">
+      <c r="J65" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr">
+      <c r="K65" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="L63" t="inlineStr">
+      <c r="L65" t="inlineStr">
         <is>
           <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr">
+      <c r="M65" t="inlineStr">
         <is>
           <t>L19298738</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O63" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P63" t="inlineStr">
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q63" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R63" t="inlineStr">
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
         <is>
           <t>1785345250</t>
         </is>
       </c>
-      <c r="S63" t="inlineStr">
+      <c r="S65" t="inlineStr">
         <is>
           <t>1785592800</t>
         </is>
       </c>
-      <c r="T63" t="inlineStr">
+      <c r="T65" t="inlineStr">
         <is>
           <t>2.173913</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr">
+      <c r="U65" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V63" t="inlineStr">
+      <c r="V65" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-06 04:01:26 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/EFL Cup/trades.xlsx
+++ b/data/sxbet/ligas/EFL Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V65"/>
+  <dimension ref="A1:V67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x9eeed2b966213cd3e1c03ecd18ebae97e3bdccaa3b690be36f141b37998d5271</t>
+          <t>0xfae81c9ef4b09ca767761b34d1d7ccc503ab3f53fac7cce04e907192fdd54e75</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -542,12 +542,12 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>15.02343</t>
+          <t>15.37496</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.8013</t>
+          <t>1.82</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785985128</t>
+          <t>1785986186</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>18.749991</t>
+          <t>18.749951</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,39 +635,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x5fbf0f7a0310f9abc0793e9101a9adc8673eb773a7cc1d40c6daae6c36914fb2</t>
+          <t>0x0099b3b9f809fea9ff4d1045745c131bda7ab30b5b0c0aaa7c161af784b6da82</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xa3786b93377213A42Bf1d3261d373cE67Cf2AA67</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x1aD0dE948858F4DeaCBEa7b44be9459c1486b543</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>24.21</t>
+          <t>15.37497</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.0825</t>
+          <t>1.8013</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Crawley Town</t>
-        </is>
-      </c>
+          <t>Under/Over (4.5)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -675,27 +667,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Watford vs Crawley Town</t>
+          <t>Cardiff City vs Swindon Town</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Watford</t>
+          <t>Cardiff City</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Swindon Town</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x5d9b97d51b6818d3cd9824517a3ea8f42d223346ae6156eded748cbedb8f386f</t>
+          <t>0xb537cfe2d0e516b2ff03db523f6c643dabb99be113085ba2d6af88754af7464c</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19692421</t>
+          <t>L19299400</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,7 +712,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785978809</t>
+          <t>1785985511</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>293.454545</t>
+          <t>19.18873</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,28 +739,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x6f6060f620c519fe84b724f15820ae1a59301dcdb13b16825be361e1751a36ef</t>
+          <t>0x9eeed2b966213cd3e1c03ecd18ebae97e3bdccaa3b690be36f141b37998d5271</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0x1aD0dE948858F4DeaCBEa7b44be9459c1486b543</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15.02343</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.4425</t>
+          <t>1.8013</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (4.5)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -779,27 +771,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Middlesbrough vs Wrexham</t>
+          <t>Cardiff City vs Swindon Town</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Middlesbrough</t>
+          <t>Cardiff City</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Wrexham</t>
+          <t>Swindon Town</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xd39b5412e3bdd35c245e5d0a2e08c3b7bbb0dccfab513161aa272b9c72edca35</t>
+          <t>0xb537cfe2d0e516b2ff03db523f6c643dabb99be113085ba2d6af88754af7464c</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19298910</t>
+          <t>L19299400</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -824,17 +816,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785971523</t>
+          <t>1785985128</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786129200</t>
+          <t>1786197600</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2.259887</t>
+          <t>18.749991</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,12 +843,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x4da7133bca54b84184238baa7d30b02372340f739df06b943262742640837a0a</t>
+          <t>0x5fbf0f7a0310f9abc0793e9101a9adc8673eb773a7cc1d40c6daae6c36914fb2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+          <t>0xa3786b93377213A42Bf1d3261d373cE67Cf2AA67</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -866,12 +858,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>24.21</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.195</t>
+          <t>1.0825</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -881,7 +873,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -891,27 +883,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>AFC Wimbledon vs Newport County</t>
+          <t>Watford vs Crawley Town</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>AFC Wimbledon</t>
+          <t>Watford</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xea47b6c120c94ae31f3299be9d23585a5cbf1b0ada4b3059268dd4cc9712b5d8</t>
+          <t>0x5d9b97d51b6818d3cd9824517a3ea8f42d223346ae6156eded748cbedb8f386f</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19298736</t>
+          <t>L19692421</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -936,7 +928,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785962236</t>
+          <t>1785978809</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -946,7 +938,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>153.846154</t>
+          <t>293.454545</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,27 +955,23 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xbae8ac7d4c8a6185b820438796f1f9f58ac63f2ed636b3e75be83914f2d44036</t>
+          <t>0x6f6060f620c519fe84b724f15820ae1a59301dcdb13b16825be361e1751a36ef</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.1175</t>
+          <t>1.4425</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -991,11 +979,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Walsall</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1003,27 +987,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Bristol City FC vs Walsall</t>
+          <t>Middlesbrough vs Wrexham</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Bristol City FC</t>
+          <t>Middlesbrough</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Walsall</t>
+          <t>Wrexham</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xc9a261f972b5555c9a1e6c0f33be8eb6a6906d2cda51babdb51dd64314b2c091</t>
+          <t>0xd39b5412e3bdd35c245e5d0a2e08c3b7bbb0dccfab513161aa272b9c72edca35</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19298734</t>
+          <t>L19298910</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1048,17 +1032,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785961563</t>
+          <t>1785971523</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786041900</t>
+          <t>1786129200</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>85.106383</t>
+          <t>2.259887</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,7 +1059,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xdd62398a10f567ee5469950797393093a356b40e7fe5930931a6c998d441d9b9</t>
+          <t>0x4da7133bca54b84184238baa7d30b02372340f739df06b943262742640837a0a</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1090,12 +1074,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.195</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1105,7 +1089,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Cheltenham Town</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1115,27 +1099,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Cheltenham Town vs Charlton Athletic</t>
+          <t>AFC Wimbledon vs Newport County</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Cheltenham Town</t>
+          <t>AFC Wimbledon</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Charlton Athletic</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x6bf36843abe397fbc7c233e0ca342729b9cd199b53d9ee9a63b96ac9358c9a1a</t>
+          <t>0xea47b6c120c94ae31f3299be9d23585a5cbf1b0ada4b3059268dd4cc9712b5d8</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19299406</t>
+          <t>L19298736</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1160,17 +1144,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785960783</t>
+          <t>1785962236</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786214700</t>
+          <t>1786197600</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>15.189873</t>
+          <t>153.846154</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,7 +1171,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xcb8aa49e12f3f29aa35ec5b7ff00195594f282ca0db4d0d9be5e2e477b96970d</t>
+          <t>0xbae8ac7d4c8a6185b820438796f1f9f58ac63f2ed636b3e75be83914f2d44036</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1202,7 +1186,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1272,7 +1256,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785960695</t>
+          <t>1785961563</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1282,7 +1266,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>59.574468</t>
+          <t>85.106383</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,12 +1283,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x02c4621d6a830534abb9a71c7d2fcc46730afe8d3b686773dfd4c590f2060027</t>
+          <t>0xdd62398a10f567ee5469950797393093a356b40e7fe5930931a6c998d441d9b9</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x204e31304364d2A5f7B90dE28F507adc449Ae221</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1314,22 +1298,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>1.1975</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>AFC Wimbledon -1.5</t>
+          <t>Cheltenham Town</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1339,27 +1323,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>AFC Wimbledon vs Newport County</t>
+          <t>Cheltenham Town vs Charlton Athletic</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>AFC Wimbledon</t>
+          <t>Cheltenham Town</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Charlton Athletic</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x9f1f722832eb2e6381f3a0226a98c406eccc5bd7e76caaaebb931fdda305a642</t>
+          <t>0x6bf36843abe397fbc7c233e0ca342729b9cd199b53d9ee9a63b96ac9358c9a1a</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19298736</t>
+          <t>L19299406</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1384,17 +1368,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785942153</t>
+          <t>1785960783</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786197600</t>
+          <t>1786214700</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2.941176</t>
+          <t>15.189873</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1411,12 +1395,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xfcba109b300bea480abe542eaa7725c7fec13f0fedc18d9991df424ad450dc90</t>
+          <t>0xcb8aa49e12f3f29aa35ec5b7ff00195594f282ca0db4d0d9be5e2e477b96970d</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x095B1B11E9C470934404Ba7F04da5F79930b2504</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1426,22 +1410,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>14.58</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.1175</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1451,27 +1435,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Bristol City FC vs Walsall</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Bristol City FC</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x30711e53de1ac1c4a025d48c70e4859ee55e52e5e57d10ed46259cc01bb5d46e</t>
+          <t>0xc9a261f972b5555c9a1e6c0f33be8eb6a6906d2cda51babdb51dd64314b2c091</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298734</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1496,17 +1480,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785778500</t>
+          <t>1785960695</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1786041900</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>59.574468</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1523,12 +1507,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x9b63fb9bdb0939e4fa277441c5160ae767a06c0723ae1697f56722a32c1dbbf4</t>
+          <t>0x02c4621d6a830534abb9a71c7d2fcc46730afe8d3b686773dfd4c590f2060027</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x204e31304364d2A5f7B90dE28F507adc449Ae221</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1538,22 +1522,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.47999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.5762</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>AFC Wimbledon -1.5</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1563,27 +1547,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>AFC Wimbledon vs Newport County</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>AFC Wimbledon</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0x9f1f722832eb2e6381f3a0226a98c406eccc5bd7e76caaaebb931fdda305a642</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298736</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1608,17 +1592,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785751617</t>
+          <t>1785942153</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1786197600</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2.568312</t>
+          <t>2.941176</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1635,31 +1619,39 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x34fd96c52ca66603743b136c029d1196926b8ea965b35ad916e9e624891a3c31</t>
+          <t>0xfcba109b300bea480abe542eaa7725c7fec13f0fedc18d9991df424ad450dc90</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>0x095B1B11E9C470934404Ba7F04da5F79930b2504</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2.59999</t>
+          <t>14.58</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.6887</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1682,7 +1674,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xb943c3d4cb1b4aebd6296b959eb4168b4f43df52a8043a9e84d184a931ac076c</t>
+          <t>0x30711e53de1ac1c4a025d48c70e4859ee55e52e5e57d10ed46259cc01bb5d46e</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1712,7 +1704,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785751591</t>
+          <t>1785778500</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1722,7 +1714,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>3.77494</t>
+          <t>18.0</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1739,12 +1731,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x92e4361325da8adb7d2c64339dc80666c0b8e0d69bcdd503c9dcdc859b32e858</t>
+          <t>0x9b63fb9bdb0939e4fa277441c5160ae767a06c0723ae1697f56722a32c1dbbf4</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1754,22 +1746,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>288.19</t>
+          <t>1.47999</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.555</t>
+          <t>1.5762</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1794,7 +1786,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1824,7 +1816,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785746436</t>
+          <t>1785751617</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1834,7 +1826,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>519.261261</t>
+          <t>2.568312</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1851,28 +1843,28 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x2f280a5348c67d22f499a879111a6cd14ba32c30651f4b235087504d75fcb720</t>
+          <t>0x34fd96c52ca66603743b136c029d1196926b8ea965b35ad916e9e624891a3c31</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2.59999</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.5263</t>
+          <t>1.6887</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1898,7 +1890,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
+          <t>0xb943c3d4cb1b4aebd6296b959eb4168b4f43df52a8043a9e84d184a931ac076c</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1928,7 +1920,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785743240</t>
+          <t>1785751591</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1938,7 +1930,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>9.501188</t>
+          <t>3.77494</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1955,36 +1947,44 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xe649643b38b6c14acf9bbbd3214bd63ce98d37feffda0c872c3665293f137b9c</t>
+          <t>0x92e4361325da8adb7d2c64339dc80666c0b8e0d69bcdd503c9dcdc859b32e858</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>288.19</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.3862</t>
+          <t>1.555</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
       <c r="I15" t="inlineStr">
         <is>
           <t>York City vs Crawley Town</t>
@@ -2002,7 +2002,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x75d0d882d84fabe75ec0ebfdf953c3267c7e17303f40762904f5aabc9353a5f5</t>
+          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785743239</t>
+          <t>1785746436</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>12.944984</t>
+          <t>519.261261</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2059,7 +2059,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x6da358c7d3a4cfc684658518c8cb0424ee2d0662e048d78a024625d5b4747aed</t>
+          <t>0x2f280a5348c67d22f499a879111a6cd14ba32c30651f4b235087504d75fcb720</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -2106,7 +2106,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2136,7 +2136,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785743239</t>
+          <t>1785743240</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2163,7 +2163,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x22ee20a74b7feafe1f674ddfe8f64eb18b48a4aa83ee151db7142c920e3c6990</t>
+          <t>0xe649643b38b6c14acf9bbbd3214bd63ce98d37feffda0c872c3665293f137b9c</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>EFL Cup</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0x75d0d882d84fabe75ec0ebfdf953c3267c7e17303f40762904f5aabc9353a5f5</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0xe3c6c58c8dab85d1b37033a7121e1d3f4c42a16c31fe969f436aa82e973fe331</t>
+          <t>0x6da358c7d3a4cfc684658518c8cb0424ee2d0662e048d78a024625d5b4747aed</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2278,17 +2278,17 @@
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -2314,7 +2314,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785743238</t>
+          <t>1785743239</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>17.130621</t>
+          <t>9.501188</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2371,7 +2371,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x67892d913ba613f3f4808f12a89e3a4415421d7988b81f5c03035cac2e9e85b1</t>
+          <t>0x22ee20a74b7feafe1f674ddfe8f64eb18b48a4aa83ee151db7142c920e3c6990</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2382,12 +2382,12 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.445</t>
+          <t>1.3862</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785743238</t>
+          <t>1785743239</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>22.47191</t>
+          <t>12.944984</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2475,7 +2475,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x51e83e15ab97eefc2ccce2074368f96e4d6b2bc474d60fd48cec81194acc78e8</t>
+          <t>0xe3c6c58c8dab85d1b37033a7121e1d3f4c42a16c31fe969f436aa82e973fe331</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2483,11 +2483,7 @@
           <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>10</t>
@@ -2495,19 +2491,15 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.335</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2530,7 +2522,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x1b7328b49fa63aee1bd67882f5cac5a5686aebcb538af0959dcdd4181c5e2f57</t>
+          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2560,7 +2552,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785742250</t>
+          <t>1785743238</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2570,7 +2562,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>29.850746</t>
+          <t>17.130621</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2587,7 +2579,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x0e0cffe2676af4f324fc06dde5b8beaeded42b973c319bbf3fb70687f8887f41</t>
+          <t>0x67892d913ba613f3f4808f12a89e3a4415421d7988b81f5c03035cac2e9e85b1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2595,11 +2587,7 @@
           <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>10</t>
@@ -2607,19 +2595,15 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.5587</t>
+          <t>1.445</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2642,7 +2626,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2672,7 +2656,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785742250</t>
+          <t>1785743238</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2682,7 +2666,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>17.897092</t>
+          <t>22.47191</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2699,12 +2683,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xb28bdee5a5bd24b5937965869b7830544160fac83e2df3848790121d4082d3d0</t>
+          <t>0x51e83e15ab97eefc2ccce2074368f96e4d6b2bc474d60fd48cec81194acc78e8</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2714,22 +2698,22 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.335</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2754,7 +2738,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0x1b7328b49fa63aee1bd67882f5cac5a5686aebcb538af0959dcdd4181c5e2f57</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2784,7 +2768,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785741714</t>
+          <t>1785742250</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2794,7 +2778,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>4.020101</t>
+          <t>29.850746</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2811,7 +2795,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xf27c17a15bfe9521fe22971af3d8cd2a8b3c9955888a401e463346a949eb3345</t>
+          <t>0x0e0cffe2676af4f324fc06dde5b8beaeded42b973c319bbf3fb70687f8887f41</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2831,17 +2815,17 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.4438</t>
+          <t>1.5587</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2866,7 +2850,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x7c21a171d3ea8b89b468e5886d9b7cec062e0e10cc0a3ad080d701f2e478e0d8</t>
+          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2896,7 +2880,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785740160</t>
+          <t>1785742250</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2906,7 +2890,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>22.535211</t>
+          <t>17.897092</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2923,7 +2907,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
+          <t>0xb28bdee5a5bd24b5937965869b7830544160fac83e2df3848790121d4082d3d0</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2943,7 +2927,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.2475</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3008,7 +2992,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785729810</t>
+          <t>1785741714</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3018,7 +3002,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>4.040404</t>
+          <t>4.020101</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3035,12 +3019,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
+          <t>0xf27c17a15bfe9521fe22971af3d8cd2a8b3c9955888a401e463346a949eb3345</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3050,22 +3034,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>3.99987</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.4438</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -3090,7 +3074,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0x7c21a171d3ea8b89b468e5886d9b7cec062e0e10cc0a3ad080d701f2e478e0d8</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3120,7 +3104,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785729635</t>
+          <t>1785740160</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3130,7 +3114,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>16.079879</t>
+          <t>22.535211</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3147,7 +3131,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
+          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3162,12 +3146,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>23.26</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.4338</t>
+          <t>1.2475</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3187,27 +3171,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3232,17 +3216,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785597225</t>
+          <t>1785729810</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>53.62536</t>
+          <t>4.040404</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3259,7 +3243,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
+          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3274,12 +3258,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3.99987</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3289,7 +3273,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3299,27 +3283,27 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -3344,17 +3328,17 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785595661</t>
+          <t>1785729635</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>3.11284</t>
+          <t>16.079879</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3371,7 +3355,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
+          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3386,12 +3370,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>23.26</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3401,32 +3385,32 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3456,7 +3440,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785594340</t>
+          <t>1785597225</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3466,7 +3450,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>27.777778</t>
+          <t>53.62536</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3483,7 +3467,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
+          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3498,12 +3482,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3568,7 +3552,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785593884</t>
+          <t>1785595661</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3578,7 +3562,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>3.11284</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3595,7 +3579,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
+          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3615,7 +3599,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3680,7 +3664,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785593884</t>
+          <t>1785594340</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3690,7 +3674,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>27.777778</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3707,7 +3691,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
+          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3722,12 +3706,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>25.04</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.385</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3792,7 +3776,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785593611</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3802,7 +3786,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>65.038961</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3819,7 +3803,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
+          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3834,12 +3818,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.2375</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3849,7 +3833,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3874,7 +3858,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3904,7 +3888,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785593186</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3914,7 +3898,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>49.263158</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3931,7 +3915,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
+          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3946,12 +3930,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>25.04</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.385</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -4016,7 +4000,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785592744</t>
+          <t>1785593611</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -4026,7 +4010,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>7.088608</t>
+          <t>65.038961</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4043,7 +4027,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
+          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4058,12 +4042,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3.59</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.2375</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4073,32 +4057,32 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4128,7 +4112,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785592658</t>
+          <t>1785593186</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4138,7 +4122,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>9.088608</t>
+          <t>49.263158</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4155,7 +4139,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
+          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4170,7 +4154,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>22.05</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -4240,7 +4224,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785592637</t>
+          <t>1785592744</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4250,7 +4234,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>55.822785</t>
+          <t>7.088608</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4267,7 +4251,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
+          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4275,15 +4259,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>36.31948</t>
+          <t>3.59</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4291,7 +4279,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4344,7 +4336,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785589857</t>
+          <t>1785592658</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4354,7 +4346,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>58.816972</t>
+          <t>9.088608</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4371,7 +4363,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
+          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4379,15 +4371,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>22.05</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4395,7 +4391,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4448,7 +4448,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1785589600</t>
+          <t>1785592637</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>6.54251</t>
+          <t>55.822785</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4475,7 +4475,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
+          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4486,12 +4486,12 @@
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>18.36999</t>
+          <t>36.31948</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.615</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4552,7 +4552,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785589491</t>
+          <t>1785589857</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>29.869902</t>
+          <t>58.816972</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4579,7 +4579,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
+          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4590,12 +4590,12 @@
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>18.54999</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1785588508</t>
+          <t>1785589600</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>30.597922</t>
+          <t>6.54251</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4683,27 +4683,23 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
+          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>15.21</t>
+          <t>18.36999</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.615</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4711,11 +4707,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4738,7 +4730,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -4768,7 +4760,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1785587700</t>
+          <t>1785589491</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4778,7 +4770,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>54.08</t>
+          <t>29.869902</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4795,7 +4787,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
+          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4806,12 +4798,12 @@
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>6.44999</t>
+          <t>18.54999</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.7237</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4842,7 +4834,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -4872,7 +4864,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1785585922</t>
+          <t>1785588508</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4882,7 +4874,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>8.911903</t>
+          <t>30.597922</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4899,23 +4891,27 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
+          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>3.26</t>
+          <t>15.21</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.7212</t>
+          <t>1.2812</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -4923,7 +4919,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4976,7 +4976,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1785579524</t>
+          <t>1785587700</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -4986,7 +4986,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>4.519931</t>
+          <t>54.08</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5003,7 +5003,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
+          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -5014,12 +5014,12 @@
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>3.61999</t>
+          <t>6.44999</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.7212</t>
+          <t>1.7237</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -5080,7 +5080,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1785579365</t>
+          <t>1785585922</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -5090,7 +5090,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>5.01905</t>
+          <t>8.911903</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5107,27 +5107,23 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
+          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>3.26</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -5135,26 +5131,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K44" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -5162,7 +5154,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -5192,7 +5184,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1785577998</t>
+          <t>1785579524</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -5202,7 +5194,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>59.143969</t>
+          <t>4.519931</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5219,27 +5211,23 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
+          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>3.61999</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -5247,11 +5235,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -5304,7 +5288,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1785577962</t>
+          <t>1785579365</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -5314,7 +5298,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>82.758621</t>
+          <t>5.01905</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5331,12 +5315,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
+          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -5346,12 +5330,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>1.3225</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -5416,7 +5400,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>1785577789</t>
+          <t>1785577998</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -5426,7 +5410,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>3.534884</t>
+          <t>59.143969</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5443,12 +5427,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
+          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -5458,12 +5442,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>18.99909</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5473,24 +5457,24 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K47" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -5498,7 +5482,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -5528,7 +5512,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1785577788</t>
+          <t>1785577962</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
@@ -5538,7 +5522,7 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>59.141136</t>
+          <t>82.758621</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5555,7 +5539,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
+          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5570,12 +5554,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.3225</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5640,7 +5624,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785577789</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -5650,7 +5634,7 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>6.101167</t>
+          <t>3.534884</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -5667,7 +5651,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
+          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5682,12 +5666,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2.81824</t>
+          <t>18.99909</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5752,7 +5736,7 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785577788</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
@@ -5762,7 +5746,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>8.807</t>
+          <t>59.141136</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -5779,7 +5763,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
+          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -5794,12 +5778,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>20.06</t>
+          <t>1.96</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5864,7 +5848,7 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>1785576072</t>
+          <t>1785576753</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
@@ -5874,7 +5858,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>62.6875</t>
+          <t>6.101167</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -5891,7 +5875,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
+          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -5906,7 +5890,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>22.07</t>
+          <t>2.81824</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -5976,7 +5960,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>1785575036</t>
+          <t>1785576753</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -5986,7 +5970,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>68.96875</t>
+          <t>8.807</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -6003,7 +5987,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
+          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6018,7 +6002,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>20.06</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -6088,7 +6072,7 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>1785574569</t>
+          <t>1785576072</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
@@ -6098,7 +6082,7 @@
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>3.625</t>
+          <t>62.6875</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -6115,7 +6099,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
+          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6130,7 +6114,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>19.25059</t>
+          <t>22.07</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -6200,7 +6184,7 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>1785574187</t>
+          <t>1785575036</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -6210,7 +6194,7 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>60.158094</t>
+          <t>68.96875</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -6227,7 +6211,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
+          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -6242,7 +6226,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>20.96</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -6312,7 +6296,7 @@
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785574569</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
@@ -6322,7 +6306,7 @@
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>65.5</t>
+          <t>3.625</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -6339,7 +6323,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
+          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -6354,7 +6338,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2.69</t>
+          <t>19.25059</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -6424,7 +6408,7 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785574187</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
@@ -6434,7 +6418,7 @@
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>8.40625</t>
+          <t>60.158094</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -6451,7 +6435,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
+          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -6466,7 +6450,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>20.96</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -6536,7 +6520,7 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>1785574073</t>
+          <t>1785574186</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
@@ -6546,7 +6530,7 @@
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>6.90625</t>
+          <t>65.5</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -6563,7 +6547,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
+          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -6578,7 +6562,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.69</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -6648,7 +6632,7 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>1785573852</t>
+          <t>1785574186</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
@@ -6658,7 +6642,7 @@
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>6.25</t>
+          <t>8.40625</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -6675,7 +6659,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
+          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -6690,12 +6674,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -6760,7 +6744,7 @@
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>1785570690</t>
+          <t>1785574073</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
@@ -6770,7 +6754,7 @@
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>6.256809</t>
+          <t>6.90625</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
@@ -6787,7 +6771,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
+          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -6802,7 +6786,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -6872,7 +6856,7 @@
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>1785570471</t>
+          <t>1785573852</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
@@ -6882,7 +6866,7 @@
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>31.25</t>
+          <t>6.25</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
@@ -6899,7 +6883,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
+          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -6907,15 +6891,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>19.72999</t>
+          <t>2.01</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -6923,7 +6911,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
       <c r="H60" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -6946,7 +6938,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -6976,7 +6968,7 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>1785569792</t>
+          <t>1785570690</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
@@ -6986,7 +6978,7 @@
       </c>
       <c r="T60" t="inlineStr">
         <is>
-          <t>32.544313</t>
+          <t>6.256809</t>
         </is>
       </c>
       <c r="U60" t="inlineStr">
@@ -7003,7 +6995,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
+          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -7018,7 +7010,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -7088,7 +7080,7 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>1785569076</t>
+          <t>1785570471</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
@@ -7098,7 +7090,7 @@
       </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>6.59375</t>
+          <t>31.25</t>
         </is>
       </c>
       <c r="U61" t="inlineStr">
@@ -7115,27 +7107,23 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
+          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>19.72999</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>1.605</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -7143,11 +7131,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>York City</t>
-        </is>
-      </c>
+      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -7155,27 +7139,27 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298738</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -7200,17 +7184,17 @@
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>1785512959</t>
+          <t>1785569792</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1785592800</t>
         </is>
       </c>
       <c r="T62" t="inlineStr">
         <is>
-          <t>1.652893</t>
+          <t>32.544313</t>
         </is>
       </c>
       <c r="U62" t="inlineStr">
@@ -7227,12 +7211,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -7242,12 +7226,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2.51</t>
+          <t>2.11</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -7257,32 +7241,32 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -7312,7 +7296,7 @@
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>1785497246</t>
+          <t>1785569076</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
@@ -7322,7 +7306,7 @@
       </c>
       <c r="T63" t="inlineStr">
         <is>
-          <t>5.97619</t>
+          <t>6.59375</t>
         </is>
       </c>
       <c r="U63" t="inlineStr">
@@ -7339,7 +7323,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -7359,7 +7343,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>1.605</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -7369,7 +7353,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -7379,27 +7363,27 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -7424,17 +7408,17 @@
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>1785346230</t>
+          <t>1785512959</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T64" t="inlineStr">
         <is>
-          <t>2.173913</t>
+          <t>1.652893</t>
         </is>
       </c>
       <c r="U64" t="inlineStr">
@@ -7451,110 +7435,334 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
+          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>1785497246</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>5.97619</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>1785346230</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>2.173913</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
           <t>0xea48d5fe72de69b25067fdb4fdaf1d08ce7262ad75f6855864d3a656da39b313</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B67" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
         <is>
           <t>1.46</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F67" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
+      <c r="G67" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="H67" t="inlineStr">
         <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr">
+      <c r="I67" t="inlineStr">
         <is>
           <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr">
+      <c r="J67" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr">
+      <c r="K67" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="L65" t="inlineStr">
+      <c r="L67" t="inlineStr">
         <is>
           <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
-      <c r="M65" t="inlineStr">
+      <c r="M67" t="inlineStr">
         <is>
           <t>L19298738</t>
         </is>
       </c>
-      <c r="N65" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O65" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P65" t="inlineStr">
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q65" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R65" t="inlineStr">
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
         <is>
           <t>1785345250</t>
         </is>
       </c>
-      <c r="S65" t="inlineStr">
+      <c r="S67" t="inlineStr">
         <is>
           <t>1785592800</t>
         </is>
       </c>
-      <c r="T65" t="inlineStr">
+      <c r="T67" t="inlineStr">
         <is>
           <t>2.173913</t>
         </is>
       </c>
-      <c r="U65" t="inlineStr">
+      <c r="U67" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V65" t="inlineStr">
+      <c r="V67" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-06 13:01:42 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/EFL Cup/trades.xlsx
+++ b/data/sxbet/ligas/EFL Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V67"/>
+  <dimension ref="A1:V69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,31 +531,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xfae81c9ef4b09ca767761b34d1d7ccc503ab3f53fac7cce04e907192fdd54e75</t>
+          <t>0x0b38365d5b799eadd00c518f32be55db166cfad4ceb029c192937d69361f6cdc</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x1aD0dE948858F4DeaCBEa7b44be9459c1486b543</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>15.37496</t>
+          <t>14.01</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.82</t>
+          <t>1.325</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (4.5)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>Asian Handicap (-2)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Bristol City FC -2</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -563,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Cardiff City vs Swindon Town</t>
+          <t>Bristol City FC vs Walsall</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Cardiff City</t>
+          <t>Bristol City FC</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Swindon Town</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xb537cfe2d0e516b2ff03db523f6c643dabb99be113085ba2d6af88754af7464c</t>
+          <t>0x3ca10be4347ce1293ced974a10089ced99b6e34d6387bad5b2dcd541fca6ca63</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19299400</t>
+          <t>L19298734</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785986186</t>
+          <t>1786020403</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786197600</t>
+          <t>1786041900</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>18.749951</t>
+          <t>43.107692</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,31 +643,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x0099b3b9f809fea9ff4d1045745c131bda7ab30b5b0c0aaa7c161af784b6da82</t>
+          <t>0xd276a2b149eeb9ab91e4a24b55762c7cb0b5c278fa9f79f20d11574ad297ca5d</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x1aD0dE948858F4DeaCBEa7b44be9459c1486b543</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>15.37497</t>
+          <t>15.61926</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.8013</t>
+          <t>1.325</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (4.5)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>Asian Handicap (-2)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Bristol City FC -2</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -667,27 +683,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Cardiff City vs Swindon Town</t>
+          <t>Bristol City FC vs Walsall</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Cardiff City</t>
+          <t>Bristol City FC</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Swindon Town</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xb537cfe2d0e516b2ff03db523f6c643dabb99be113085ba2d6af88754af7464c</t>
+          <t>0x3ca10be4347ce1293ced974a10089ced99b6e34d6387bad5b2dcd541fca6ca63</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19299400</t>
+          <t>L19298734</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -712,17 +728,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785985511</t>
+          <t>1786020371</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786197600</t>
+          <t>1786041900</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>19.18873</t>
+          <t>48.059262</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,7 +755,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x9eeed2b966213cd3e1c03ecd18ebae97e3bdccaa3b690be36f141b37998d5271</t>
+          <t>0xfae81c9ef4b09ca767761b34d1d7ccc503ab3f53fac7cce04e907192fdd54e75</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -750,12 +766,12 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>15.02343</t>
+          <t>15.37496</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.8013</t>
+          <t>1.82</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -816,7 +832,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785985128</t>
+          <t>1785986186</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -826,7 +842,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>18.749991</t>
+          <t>18.749951</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -843,39 +859,31 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x5fbf0f7a0310f9abc0793e9101a9adc8673eb773a7cc1d40c6daae6c36914fb2</t>
+          <t>0x0099b3b9f809fea9ff4d1045745c131bda7ab30b5b0c0aaa7c161af784b6da82</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xa3786b93377213A42Bf1d3261d373cE67Cf2AA67</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x1aD0dE948858F4DeaCBEa7b44be9459c1486b543</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>24.21</t>
+          <t>15.37497</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.0825</t>
+          <t>1.8013</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Crawley Town</t>
-        </is>
-      </c>
+          <t>Under/Over (4.5)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -883,27 +891,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Watford vs Crawley Town</t>
+          <t>Cardiff City vs Swindon Town</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Watford</t>
+          <t>Cardiff City</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Swindon Town</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x5d9b97d51b6818d3cd9824517a3ea8f42d223346ae6156eded748cbedb8f386f</t>
+          <t>0xb537cfe2d0e516b2ff03db523f6c643dabb99be113085ba2d6af88754af7464c</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19692421</t>
+          <t>L19299400</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -928,7 +936,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785978809</t>
+          <t>1785985511</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -938,7 +946,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>293.454545</t>
+          <t>19.18873</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -955,28 +963,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x6f6060f620c519fe84b724f15820ae1a59301dcdb13b16825be361e1751a36ef</t>
+          <t>0x9eeed2b966213cd3e1c03ecd18ebae97e3bdccaa3b690be36f141b37998d5271</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0x1aD0dE948858F4DeaCBEa7b44be9459c1486b543</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15.02343</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.4425</t>
+          <t>1.8013</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (4.5)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -987,27 +995,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Middlesbrough vs Wrexham</t>
+          <t>Cardiff City vs Swindon Town</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Middlesbrough</t>
+          <t>Cardiff City</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Wrexham</t>
+          <t>Swindon Town</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xd39b5412e3bdd35c245e5d0a2e08c3b7bbb0dccfab513161aa272b9c72edca35</t>
+          <t>0xb537cfe2d0e516b2ff03db523f6c643dabb99be113085ba2d6af88754af7464c</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19298910</t>
+          <t>L19299400</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1032,17 +1040,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785971523</t>
+          <t>1785985128</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786129200</t>
+          <t>1786197600</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2.259887</t>
+          <t>18.749991</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1059,12 +1067,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x4da7133bca54b84184238baa7d30b02372340f739df06b943262742640837a0a</t>
+          <t>0x5fbf0f7a0310f9abc0793e9101a9adc8673eb773a7cc1d40c6daae6c36914fb2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+          <t>0xa3786b93377213A42Bf1d3261d373cE67Cf2AA67</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1074,12 +1082,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>24.21</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.195</t>
+          <t>1.0825</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1089,7 +1097,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1099,27 +1107,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>AFC Wimbledon vs Newport County</t>
+          <t>Watford vs Crawley Town</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>AFC Wimbledon</t>
+          <t>Watford</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xea47b6c120c94ae31f3299be9d23585a5cbf1b0ada4b3059268dd4cc9712b5d8</t>
+          <t>0x5d9b97d51b6818d3cd9824517a3ea8f42d223346ae6156eded748cbedb8f386f</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19298736</t>
+          <t>L19692421</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1144,7 +1152,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785962236</t>
+          <t>1785978809</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1154,7 +1162,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>153.846154</t>
+          <t>293.454545</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1171,27 +1179,23 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xbae8ac7d4c8a6185b820438796f1f9f58ac63f2ed636b3e75be83914f2d44036</t>
+          <t>0x6f6060f620c519fe84b724f15820ae1a59301dcdb13b16825be361e1751a36ef</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.1175</t>
+          <t>1.4425</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1199,11 +1203,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Walsall</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1211,27 +1211,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Bristol City FC vs Walsall</t>
+          <t>Middlesbrough vs Wrexham</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Bristol City FC</t>
+          <t>Middlesbrough</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Walsall</t>
+          <t>Wrexham</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xc9a261f972b5555c9a1e6c0f33be8eb6a6906d2cda51babdb51dd64314b2c091</t>
+          <t>0xd39b5412e3bdd35c245e5d0a2e08c3b7bbb0dccfab513161aa272b9c72edca35</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19298734</t>
+          <t>L19298910</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1256,17 +1256,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785961563</t>
+          <t>1785971523</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786041900</t>
+          <t>1786129200</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>85.106383</t>
+          <t>2.259887</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1283,7 +1283,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xdd62398a10f567ee5469950797393093a356b40e7fe5930931a6c998d441d9b9</t>
+          <t>0x4da7133bca54b84184238baa7d30b02372340f739df06b943262742640837a0a</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1298,12 +1298,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.195</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Cheltenham Town</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1323,27 +1323,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Cheltenham Town vs Charlton Athletic</t>
+          <t>AFC Wimbledon vs Newport County</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Cheltenham Town</t>
+          <t>AFC Wimbledon</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Charlton Athletic</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x6bf36843abe397fbc7c233e0ca342729b9cd199b53d9ee9a63b96ac9358c9a1a</t>
+          <t>0xea47b6c120c94ae31f3299be9d23585a5cbf1b0ada4b3059268dd4cc9712b5d8</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19299406</t>
+          <t>L19298736</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1368,17 +1368,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785960783</t>
+          <t>1785962236</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786214700</t>
+          <t>1786197600</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>15.189873</t>
+          <t>153.846154</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,7 +1395,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xcb8aa49e12f3f29aa35ec5b7ff00195594f282ca0db4d0d9be5e2e477b96970d</t>
+          <t>0xbae8ac7d4c8a6185b820438796f1f9f58ac63f2ed636b3e75be83914f2d44036</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785960695</t>
+          <t>1785961563</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>59.574468</t>
+          <t>85.106383</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1507,12 +1507,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x02c4621d6a830534abb9a71c7d2fcc46730afe8d3b686773dfd4c590f2060027</t>
+          <t>0xdd62398a10f567ee5469950797393093a356b40e7fe5930931a6c998d441d9b9</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x204e31304364d2A5f7B90dE28F507adc449Ae221</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1522,22 +1522,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>1.1975</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>AFC Wimbledon -1.5</t>
+          <t>Cheltenham Town</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1547,27 +1547,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>AFC Wimbledon vs Newport County</t>
+          <t>Cheltenham Town vs Charlton Athletic</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>AFC Wimbledon</t>
+          <t>Cheltenham Town</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Charlton Athletic</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x9f1f722832eb2e6381f3a0226a98c406eccc5bd7e76caaaebb931fdda305a642</t>
+          <t>0x6bf36843abe397fbc7c233e0ca342729b9cd199b53d9ee9a63b96ac9358c9a1a</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19298736</t>
+          <t>L19299406</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1592,17 +1592,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785942153</t>
+          <t>1785960783</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1786197600</t>
+          <t>1786214700</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2.941176</t>
+          <t>15.189873</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1619,12 +1619,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xfcba109b300bea480abe542eaa7725c7fec13f0fedc18d9991df424ad450dc90</t>
+          <t>0xcb8aa49e12f3f29aa35ec5b7ff00195594f282ca0db4d0d9be5e2e477b96970d</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x095B1B11E9C470934404Ba7F04da5F79930b2504</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1634,22 +1634,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>14.58</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.1175</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1659,27 +1659,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Bristol City FC vs Walsall</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Bristol City FC</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x30711e53de1ac1c4a025d48c70e4859ee55e52e5e57d10ed46259cc01bb5d46e</t>
+          <t>0xc9a261f972b5555c9a1e6c0f33be8eb6a6906d2cda51babdb51dd64314b2c091</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298734</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1704,17 +1704,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785778500</t>
+          <t>1785960695</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1786041900</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>59.574468</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1731,12 +1731,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x9b63fb9bdb0939e4fa277441c5160ae767a06c0723ae1697f56722a32c1dbbf4</t>
+          <t>0x02c4621d6a830534abb9a71c7d2fcc46730afe8d3b686773dfd4c590f2060027</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x204e31304364d2A5f7B90dE28F507adc449Ae221</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1746,22 +1746,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1.47999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.5762</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>AFC Wimbledon -1.5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1771,27 +1771,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>AFC Wimbledon vs Newport County</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>AFC Wimbledon</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0x9f1f722832eb2e6381f3a0226a98c406eccc5bd7e76caaaebb931fdda305a642</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298736</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1816,17 +1816,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785751617</t>
+          <t>1785942153</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1786197600</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2.568312</t>
+          <t>2.941176</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1843,31 +1843,39 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x34fd96c52ca66603743b136c029d1196926b8ea965b35ad916e9e624891a3c31</t>
+          <t>0xfcba109b300bea480abe542eaa7725c7fec13f0fedc18d9991df424ad450dc90</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
+          <t>0x095B1B11E9C470934404Ba7F04da5F79930b2504</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2.59999</t>
+          <t>14.58</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.6887</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1890,7 +1898,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xb943c3d4cb1b4aebd6296b959eb4168b4f43df52a8043a9e84d184a931ac076c</t>
+          <t>0x30711e53de1ac1c4a025d48c70e4859ee55e52e5e57d10ed46259cc01bb5d46e</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1920,7 +1928,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785751591</t>
+          <t>1785778500</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1930,7 +1938,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>3.77494</t>
+          <t>18.0</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1947,12 +1955,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x92e4361325da8adb7d2c64339dc80666c0b8e0d69bcdd503c9dcdc859b32e858</t>
+          <t>0x9b63fb9bdb0939e4fa277441c5160ae767a06c0723ae1697f56722a32c1dbbf4</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1962,22 +1970,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>288.19</t>
+          <t>1.47999</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.555</t>
+          <t>1.5762</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2002,7 +2010,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2032,7 +2040,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785746436</t>
+          <t>1785751617</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2042,7 +2050,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>519.261261</t>
+          <t>2.568312</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2059,28 +2067,28 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x2f280a5348c67d22f499a879111a6cd14ba32c30651f4b235087504d75fcb720</t>
+          <t>0x34fd96c52ca66603743b136c029d1196926b8ea965b35ad916e9e624891a3c31</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2.59999</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.5263</t>
+          <t>1.6887</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -2106,7 +2114,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
+          <t>0xb943c3d4cb1b4aebd6296b959eb4168b4f43df52a8043a9e84d184a931ac076c</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2136,7 +2144,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785743240</t>
+          <t>1785751591</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2146,7 +2154,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>9.501188</t>
+          <t>3.77494</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2163,36 +2171,44 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xe649643b38b6c14acf9bbbd3214bd63ce98d37feffda0c872c3665293f137b9c</t>
+          <t>0x92e4361325da8adb7d2c64339dc80666c0b8e0d69bcdd503c9dcdc859b32e858</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>288.19</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.3862</t>
+          <t>1.555</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>York City vs Crawley Town</t>
@@ -2210,7 +2226,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x75d0d882d84fabe75ec0ebfdf953c3267c7e17303f40762904f5aabc9353a5f5</t>
+          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2240,7 +2256,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785743239</t>
+          <t>1785746436</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2250,7 +2266,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>12.944984</t>
+          <t>519.261261</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2267,7 +2283,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x6da358c7d3a4cfc684658518c8cb0424ee2d0662e048d78a024625d5b4747aed</t>
+          <t>0x2f280a5348c67d22f499a879111a6cd14ba32c30651f4b235087504d75fcb720</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2288,7 +2304,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -2314,7 +2330,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2344,7 +2360,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785743239</t>
+          <t>1785743240</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2371,7 +2387,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x22ee20a74b7feafe1f674ddfe8f64eb18b48a4aa83ee151db7142c920e3c6990</t>
+          <t>0xe649643b38b6c14acf9bbbd3214bd63ce98d37feffda0c872c3665293f137b9c</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2392,7 +2408,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>EFL Cup</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
@@ -2418,7 +2434,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0x75d0d882d84fabe75ec0ebfdf953c3267c7e17303f40762904f5aabc9353a5f5</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2475,7 +2491,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xe3c6c58c8dab85d1b37033a7121e1d3f4c42a16c31fe969f436aa82e973fe331</t>
+          <t>0x6da358c7d3a4cfc684658518c8cb0424ee2d0662e048d78a024625d5b4747aed</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2486,17 +2502,17 @@
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -2522,7 +2538,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2552,7 +2568,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785743238</t>
+          <t>1785743239</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2562,7 +2578,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>17.130621</t>
+          <t>9.501188</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2579,7 +2595,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x67892d913ba613f3f4808f12a89e3a4415421d7988b81f5c03035cac2e9e85b1</t>
+          <t>0x22ee20a74b7feafe1f674ddfe8f64eb18b48a4aa83ee151db7142c920e3c6990</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2590,12 +2606,12 @@
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.445</t>
+          <t>1.3862</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2656,7 +2672,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785743238</t>
+          <t>1785743239</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2666,7 +2682,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>22.47191</t>
+          <t>12.944984</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2683,7 +2699,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x51e83e15ab97eefc2ccce2074368f96e4d6b2bc474d60fd48cec81194acc78e8</t>
+          <t>0xe3c6c58c8dab85d1b37033a7121e1d3f4c42a16c31fe969f436aa82e973fe331</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2691,11 +2707,7 @@
           <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>10</t>
@@ -2703,19 +2715,15 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.335</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2738,7 +2746,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x1b7328b49fa63aee1bd67882f5cac5a5686aebcb538af0959dcdd4181c5e2f57</t>
+          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2768,7 +2776,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785742250</t>
+          <t>1785743238</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2778,7 +2786,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>29.850746</t>
+          <t>17.130621</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2795,7 +2803,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x0e0cffe2676af4f324fc06dde5b8beaeded42b973c319bbf3fb70687f8887f41</t>
+          <t>0x67892d913ba613f3f4808f12a89e3a4415421d7988b81f5c03035cac2e9e85b1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2803,11 +2811,7 @@
           <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>10</t>
@@ -2815,19 +2819,15 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.5587</t>
+          <t>1.445</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785742250</t>
+          <t>1785743238</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>17.897092</t>
+          <t>22.47191</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2907,12 +2907,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xb28bdee5a5bd24b5937965869b7830544160fac83e2df3848790121d4082d3d0</t>
+          <t>0x51e83e15ab97eefc2ccce2074368f96e4d6b2bc474d60fd48cec81194acc78e8</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2922,22 +2922,22 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.335</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2962,7 +2962,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0x1b7328b49fa63aee1bd67882f5cac5a5686aebcb538af0959dcdd4181c5e2f57</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785741714</t>
+          <t>1785742250</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>4.020101</t>
+          <t>29.850746</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3019,7 +3019,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0xf27c17a15bfe9521fe22971af3d8cd2a8b3c9955888a401e463346a949eb3345</t>
+          <t>0x0e0cffe2676af4f324fc06dde5b8beaeded42b973c319bbf3fb70687f8887f41</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3039,17 +3039,17 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.4438</t>
+          <t>1.5587</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x7c21a171d3ea8b89b468e5886d9b7cec062e0e10cc0a3ad080d701f2e478e0d8</t>
+          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3104,7 +3104,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785740160</t>
+          <t>1785742250</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>22.535211</t>
+          <t>17.897092</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3131,7 +3131,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
+          <t>0xb28bdee5a5bd24b5937965869b7830544160fac83e2df3848790121d4082d3d0</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.2475</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785729810</t>
+          <t>1785741714</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3226,7 +3226,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>4.040404</t>
+          <t>4.020101</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3243,12 +3243,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
+          <t>0xf27c17a15bfe9521fe22971af3d8cd2a8b3c9955888a401e463346a949eb3345</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3258,22 +3258,22 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>3.99987</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.4438</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3298,7 +3298,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0x7c21a171d3ea8b89b468e5886d9b7cec062e0e10cc0a3ad080d701f2e478e0d8</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3328,7 +3328,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785729635</t>
+          <t>1785740160</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3338,7 +3338,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>16.079879</t>
+          <t>22.535211</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3355,7 +3355,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
+          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3370,12 +3370,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>23.26</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.4338</t>
+          <t>1.2475</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3395,27 +3395,27 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -3440,17 +3440,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785597225</t>
+          <t>1785729810</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>53.62536</t>
+          <t>4.040404</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
+          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3482,12 +3482,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3.99987</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3497,7 +3497,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3507,27 +3507,27 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -3552,17 +3552,17 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785595661</t>
+          <t>1785729635</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>3.11284</t>
+          <t>16.079879</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3579,7 +3579,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
+          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3594,12 +3594,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>23.26</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3609,32 +3609,32 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785594340</t>
+          <t>1785597225</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>27.777778</t>
+          <t>53.62536</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3691,7 +3691,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
+          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3706,12 +3706,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3776,7 +3776,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785593884</t>
+          <t>1785595661</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>3.11284</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3803,7 +3803,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
+          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3823,7 +3823,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3888,7 +3888,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785593884</t>
+          <t>1785594340</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>27.777778</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3915,7 +3915,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
+          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3930,12 +3930,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>25.04</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.385</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -4000,7 +4000,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785593611</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -4010,7 +4010,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>65.038961</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4027,7 +4027,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
+          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4042,12 +4042,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.2375</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4057,7 +4057,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785593186</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>49.263158</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4139,7 +4139,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
+          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4154,12 +4154,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>25.04</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.385</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4224,7 +4224,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785592744</t>
+          <t>1785593611</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4234,7 +4234,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>7.088608</t>
+          <t>65.038961</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4251,7 +4251,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
+          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4266,12 +4266,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3.59</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.2375</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4281,32 +4281,32 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785592658</t>
+          <t>1785593186</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4346,7 +4346,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>9.088608</t>
+          <t>49.263158</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4363,7 +4363,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
+          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4378,7 +4378,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>22.05</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1785592637</t>
+          <t>1785592744</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>55.822785</t>
+          <t>7.088608</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4475,7 +4475,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
+          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4483,15 +4483,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>36.31948</t>
+          <t>3.59</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4499,7 +4503,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4552,7 +4560,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785589857</t>
+          <t>1785592658</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4562,7 +4570,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>58.816972</t>
+          <t>9.088608</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4579,7 +4587,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
+          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4587,15 +4595,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>22.05</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4603,7 +4615,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4656,7 +4672,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1785589600</t>
+          <t>1785592637</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4666,7 +4682,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>6.54251</t>
+          <t>55.822785</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4683,7 +4699,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
+          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4694,12 +4710,12 @@
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>18.36999</t>
+          <t>36.31948</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.615</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4760,7 +4776,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1785589491</t>
+          <t>1785589857</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4770,7 +4786,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>29.869902</t>
+          <t>58.816972</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4787,7 +4803,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
+          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4798,12 +4814,12 @@
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>18.54999</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4864,7 +4880,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1785588508</t>
+          <t>1785589600</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4874,7 +4890,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>30.597922</t>
+          <t>6.54251</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4891,27 +4907,23 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
+          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>15.21</t>
+          <t>18.36999</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.615</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -4919,11 +4931,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4946,7 +4954,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -4976,7 +4984,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1785587700</t>
+          <t>1785589491</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -4986,7 +4994,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>54.08</t>
+          <t>29.869902</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5003,7 +5011,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
+          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -5014,12 +5022,12 @@
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>6.44999</t>
+          <t>18.54999</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.7237</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -5050,7 +5058,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -5080,7 +5088,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1785585922</t>
+          <t>1785588508</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -5090,7 +5098,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>8.911903</t>
+          <t>30.597922</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5107,23 +5115,27 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
+          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>3.26</t>
+          <t>15.21</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.7212</t>
+          <t>1.2812</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -5131,7 +5143,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -5184,7 +5200,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1785579524</t>
+          <t>1785587700</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -5194,7 +5210,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>4.519931</t>
+          <t>54.08</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5211,7 +5227,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
+          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5222,12 +5238,12 @@
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>3.61999</t>
+          <t>6.44999</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.7212</t>
+          <t>1.7237</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -5288,7 +5304,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1785579365</t>
+          <t>1785585922</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -5298,7 +5314,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>5.01905</t>
+          <t>8.911903</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5315,27 +5331,23 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
+          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>3.26</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -5343,26 +5355,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K46" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -5370,7 +5378,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -5400,7 +5408,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>1785577998</t>
+          <t>1785579524</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -5410,7 +5418,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>59.143969</t>
+          <t>4.519931</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5427,27 +5435,23 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
+          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>3.61999</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5455,11 +5459,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -5512,7 +5512,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1785577962</t>
+          <t>1785579365</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>82.758621</t>
+          <t>5.01905</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5539,12 +5539,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
+          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -5554,12 +5554,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>1.3225</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5624,7 +5624,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>1785577789</t>
+          <t>1785577998</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -5634,7 +5634,7 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>3.534884</t>
+          <t>59.143969</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -5651,12 +5651,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
+          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -5666,12 +5666,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>18.99909</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5681,24 +5681,24 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K49" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -5706,7 +5706,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -5736,7 +5736,7 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>1785577788</t>
+          <t>1785577962</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
@@ -5746,7 +5746,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>59.141136</t>
+          <t>82.758621</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -5763,7 +5763,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
+          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -5778,12 +5778,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.3225</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5848,7 +5848,7 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785577789</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
@@ -5858,7 +5858,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>6.101167</t>
+          <t>3.534884</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -5875,7 +5875,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
+          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -5890,12 +5890,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2.81824</t>
+          <t>18.99909</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5960,7 +5960,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785577788</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -5970,7 +5970,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>8.807</t>
+          <t>59.141136</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
+          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6002,12 +6002,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>20.06</t>
+          <t>1.96</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6072,7 +6072,7 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>1785576072</t>
+          <t>1785576753</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
@@ -6082,7 +6082,7 @@
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>62.6875</t>
+          <t>6.101167</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -6099,7 +6099,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
+          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>22.07</t>
+          <t>2.81824</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -6184,7 +6184,7 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>1785575036</t>
+          <t>1785576753</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -6194,7 +6194,7 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>68.96875</t>
+          <t>8.807</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -6211,7 +6211,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
+          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -6226,7 +6226,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>20.06</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>1785574569</t>
+          <t>1785576072</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>3.625</t>
+          <t>62.6875</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -6323,7 +6323,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
+          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -6338,7 +6338,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>19.25059</t>
+          <t>22.07</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>1785574187</t>
+          <t>1785575036</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
@@ -6418,7 +6418,7 @@
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>60.158094</t>
+          <t>68.96875</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -6435,7 +6435,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
+          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -6450,7 +6450,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>20.96</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -6520,7 +6520,7 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785574569</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
@@ -6530,7 +6530,7 @@
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>65.5</t>
+          <t>3.625</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -6547,7 +6547,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
+          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>2.69</t>
+          <t>19.25059</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -6632,7 +6632,7 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785574187</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
@@ -6642,7 +6642,7 @@
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>8.40625</t>
+          <t>60.158094</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -6659,7 +6659,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
+          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -6674,7 +6674,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>20.96</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -6744,7 +6744,7 @@
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>1785574073</t>
+          <t>1785574186</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
@@ -6754,7 +6754,7 @@
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>6.90625</t>
+          <t>65.5</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
@@ -6771,7 +6771,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
+          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -6786,7 +6786,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.69</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -6856,7 +6856,7 @@
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>1785573852</t>
+          <t>1785574186</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
@@ -6866,7 +6866,7 @@
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>6.25</t>
+          <t>8.40625</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
@@ -6883,7 +6883,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
+          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -6898,12 +6898,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -6968,7 +6968,7 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>1785570690</t>
+          <t>1785574073</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
@@ -6978,7 +6978,7 @@
       </c>
       <c r="T60" t="inlineStr">
         <is>
-          <t>6.256809</t>
+          <t>6.90625</t>
         </is>
       </c>
       <c r="U60" t="inlineStr">
@@ -6995,7 +6995,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
+          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -7010,7 +7010,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -7080,7 +7080,7 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>1785570471</t>
+          <t>1785573852</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
@@ -7090,7 +7090,7 @@
       </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>31.25</t>
+          <t>6.25</t>
         </is>
       </c>
       <c r="U61" t="inlineStr">
@@ -7107,7 +7107,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
+          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -7115,15 +7115,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>19.72999</t>
+          <t>2.01</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -7131,7 +7135,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
       <c r="H62" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -7154,7 +7162,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -7184,7 +7192,7 @@
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>1785569792</t>
+          <t>1785570690</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
@@ -7194,7 +7202,7 @@
       </c>
       <c r="T62" t="inlineStr">
         <is>
-          <t>32.544313</t>
+          <t>6.256809</t>
         </is>
       </c>
       <c r="U62" t="inlineStr">
@@ -7211,7 +7219,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
+          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -7226,7 +7234,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -7296,7 +7304,7 @@
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>1785569076</t>
+          <t>1785570471</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
@@ -7306,7 +7314,7 @@
       </c>
       <c r="T63" t="inlineStr">
         <is>
-          <t>6.59375</t>
+          <t>31.25</t>
         </is>
       </c>
       <c r="U63" t="inlineStr">
@@ -7323,27 +7331,23 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
+          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>19.72999</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>1.605</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -7351,11 +7355,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>York City</t>
-        </is>
-      </c>
+      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -7363,27 +7363,27 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298738</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -7408,17 +7408,17 @@
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>1785512959</t>
+          <t>1785569792</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1785592800</t>
         </is>
       </c>
       <c r="T64" t="inlineStr">
         <is>
-          <t>1.652893</t>
+          <t>32.544313</t>
         </is>
       </c>
       <c r="U64" t="inlineStr">
@@ -7435,12 +7435,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -7450,12 +7450,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2.51</t>
+          <t>2.11</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -7465,32 +7465,32 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -7520,7 +7520,7 @@
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>1785497246</t>
+          <t>1785569076</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
@@ -7530,7 +7530,7 @@
       </c>
       <c r="T65" t="inlineStr">
         <is>
-          <t>5.97619</t>
+          <t>6.59375</t>
         </is>
       </c>
       <c r="U65" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -7567,7 +7567,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>1.605</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -7577,7 +7577,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -7587,27 +7587,27 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -7632,17 +7632,17 @@
       </c>
       <c r="R66" t="inlineStr">
         <is>
-          <t>1785346230</t>
+          <t>1785512959</t>
         </is>
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T66" t="inlineStr">
         <is>
-          <t>2.173913</t>
+          <t>1.652893</t>
         </is>
       </c>
       <c r="U66" t="inlineStr">
@@ -7659,110 +7659,334 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
+          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>1785497246</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>5.97619</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>1785346230</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>2.173913</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
           <t>0xea48d5fe72de69b25067fdb4fdaf1d08ce7262ad75f6855864d3a656da39b313</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B69" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
         <is>
           <t>1.46</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="F69" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr">
+      <c r="G69" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
+      <c r="H69" t="inlineStr">
         <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr">
+      <c r="I69" t="inlineStr">
         <is>
           <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr">
+      <c r="J69" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr">
+      <c r="K69" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="L67" t="inlineStr">
+      <c r="L69" t="inlineStr">
         <is>
           <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
-      <c r="M67" t="inlineStr">
+      <c r="M69" t="inlineStr">
         <is>
           <t>L19298738</t>
         </is>
       </c>
-      <c r="N67" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O67" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P67" t="inlineStr">
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q67" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R67" t="inlineStr">
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
         <is>
           <t>1785345250</t>
         </is>
       </c>
-      <c r="S67" t="inlineStr">
+      <c r="S69" t="inlineStr">
         <is>
           <t>1785592800</t>
         </is>
       </c>
-      <c r="T67" t="inlineStr">
+      <c r="T69" t="inlineStr">
         <is>
           <t>2.173913</t>
         </is>
       </c>
-      <c r="U67" t="inlineStr">
+      <c r="U69" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V67" t="inlineStr">
+      <c r="V69" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-06 14:01:42 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/EFL Cup/trades.xlsx
+++ b/data/sxbet/ligas/EFL Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V69"/>
+  <dimension ref="A1:V71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,39 +531,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x0b38365d5b799eadd00c518f32be55db166cfad4ceb029c192937d69361f6cdc</t>
+          <t>0x262b25eb7234bdeed55ef18582086a41c69d4a611e2bd9abd2a7fa6f0a8ad55a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>14.01</t>
+          <t>7.59</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.325</t>
+          <t>1.4075</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Asian Handicap (-2)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Bristol City FC -2</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -586,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x3ca10be4347ce1293ced974a10089ced99b6e34d6387bad5b2dcd541fca6ca63</t>
+          <t>0x4822d15d04e505f4dd3cd578b479004c99d54d611a00b8362f654229fd356954</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786020403</t>
+          <t>1786023828</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>43.107692</t>
+          <t>18.625767</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,39 +635,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xd276a2b149eeb9ab91e4a24b55762c7cb0b5c278fa9f79f20d11574ad297ca5d</t>
+          <t>0xd547fb326ce8e6c94e2a7ea09c7bdac9d13dfedbcd1cf16a791fe9a75ea416b1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>15.61926</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.325</t>
+          <t>1.2925</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Asian Handicap (-2)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Bristol City FC -2</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -698,7 +682,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x3ca10be4347ce1293ced974a10089ced99b6e34d6387bad5b2dcd541fca6ca63</t>
+          <t>0xec232eeef0113c821800c4331e9294d40693adaea445f17da39670a388f83470</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +712,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786020371</t>
+          <t>1786022401</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>48.059262</t>
+          <t>3.418803</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,31 +739,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xfae81c9ef4b09ca767761b34d1d7ccc503ab3f53fac7cce04e907192fdd54e75</t>
+          <t>0x0b38365d5b799eadd00c518f32be55db166cfad4ceb029c192937d69361f6cdc</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x1aD0dE948858F4DeaCBEa7b44be9459c1486b543</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>15.37496</t>
+          <t>14.01</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.82</t>
+          <t>1.325</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (4.5)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>Asian Handicap (-2)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Bristol City FC -2</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -787,27 +779,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Cardiff City vs Swindon Town</t>
+          <t>Bristol City FC vs Walsall</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Cardiff City</t>
+          <t>Bristol City FC</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Swindon Town</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xb537cfe2d0e516b2ff03db523f6c643dabb99be113085ba2d6af88754af7464c</t>
+          <t>0x3ca10be4347ce1293ced974a10089ced99b6e34d6387bad5b2dcd541fca6ca63</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19299400</t>
+          <t>L19298734</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,17 +824,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785986186</t>
+          <t>1786020403</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786197600</t>
+          <t>1786041900</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>18.749951</t>
+          <t>43.107692</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,31 +851,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x0099b3b9f809fea9ff4d1045745c131bda7ab30b5b0c0aaa7c161af784b6da82</t>
+          <t>0xd276a2b149eeb9ab91e4a24b55762c7cb0b5c278fa9f79f20d11574ad297ca5d</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x1aD0dE948858F4DeaCBEa7b44be9459c1486b543</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>15.37497</t>
+          <t>15.61926</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.8013</t>
+          <t>1.325</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (4.5)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>Asian Handicap (-2)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Bristol City FC -2</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -891,27 +891,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Cardiff City vs Swindon Town</t>
+          <t>Bristol City FC vs Walsall</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Cardiff City</t>
+          <t>Bristol City FC</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Swindon Town</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xb537cfe2d0e516b2ff03db523f6c643dabb99be113085ba2d6af88754af7464c</t>
+          <t>0x3ca10be4347ce1293ced974a10089ced99b6e34d6387bad5b2dcd541fca6ca63</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19299400</t>
+          <t>L19298734</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -936,17 +936,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785985511</t>
+          <t>1786020371</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786197600</t>
+          <t>1786041900</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>19.18873</t>
+          <t>48.059262</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,7 +963,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x9eeed2b966213cd3e1c03ecd18ebae97e3bdccaa3b690be36f141b37998d5271</t>
+          <t>0xfae81c9ef4b09ca767761b34d1d7ccc503ab3f53fac7cce04e907192fdd54e75</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -974,12 +974,12 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>15.02343</t>
+          <t>15.37496</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.8013</t>
+          <t>1.82</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785985128</t>
+          <t>1785986186</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>18.749991</t>
+          <t>18.749951</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1067,39 +1067,31 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x5fbf0f7a0310f9abc0793e9101a9adc8673eb773a7cc1d40c6daae6c36914fb2</t>
+          <t>0x0099b3b9f809fea9ff4d1045745c131bda7ab30b5b0c0aaa7c161af784b6da82</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xa3786b93377213A42Bf1d3261d373cE67Cf2AA67</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x1aD0dE948858F4DeaCBEa7b44be9459c1486b543</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>24.21</t>
+          <t>15.37497</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.0825</t>
+          <t>1.8013</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Crawley Town</t>
-        </is>
-      </c>
+          <t>Under/Over (4.5)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1107,27 +1099,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Watford vs Crawley Town</t>
+          <t>Cardiff City vs Swindon Town</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Watford</t>
+          <t>Cardiff City</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Swindon Town</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x5d9b97d51b6818d3cd9824517a3ea8f42d223346ae6156eded748cbedb8f386f</t>
+          <t>0xb537cfe2d0e516b2ff03db523f6c643dabb99be113085ba2d6af88754af7464c</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19692421</t>
+          <t>L19299400</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1152,7 +1144,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785978809</t>
+          <t>1785985511</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1154,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>293.454545</t>
+          <t>19.18873</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,28 +1171,28 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x6f6060f620c519fe84b724f15820ae1a59301dcdb13b16825be361e1751a36ef</t>
+          <t>0x9eeed2b966213cd3e1c03ecd18ebae97e3bdccaa3b690be36f141b37998d5271</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0x1aD0dE948858F4DeaCBEa7b44be9459c1486b543</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15.02343</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.4425</t>
+          <t>1.8013</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (4.5)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -1211,27 +1203,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Middlesbrough vs Wrexham</t>
+          <t>Cardiff City vs Swindon Town</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Middlesbrough</t>
+          <t>Cardiff City</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Wrexham</t>
+          <t>Swindon Town</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xd39b5412e3bdd35c245e5d0a2e08c3b7bbb0dccfab513161aa272b9c72edca35</t>
+          <t>0xb537cfe2d0e516b2ff03db523f6c643dabb99be113085ba2d6af88754af7464c</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19298910</t>
+          <t>L19299400</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1256,17 +1248,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785971523</t>
+          <t>1785985128</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786129200</t>
+          <t>1786197600</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2.259887</t>
+          <t>18.749991</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1283,12 +1275,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x4da7133bca54b84184238baa7d30b02372340f739df06b943262742640837a0a</t>
+          <t>0x5fbf0f7a0310f9abc0793e9101a9adc8673eb773a7cc1d40c6daae6c36914fb2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+          <t>0xa3786b93377213A42Bf1d3261d373cE67Cf2AA67</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1298,12 +1290,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>24.21</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.195</t>
+          <t>1.0825</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1313,7 +1305,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1323,27 +1315,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>AFC Wimbledon vs Newport County</t>
+          <t>Watford vs Crawley Town</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>AFC Wimbledon</t>
+          <t>Watford</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xea47b6c120c94ae31f3299be9d23585a5cbf1b0ada4b3059268dd4cc9712b5d8</t>
+          <t>0x5d9b97d51b6818d3cd9824517a3ea8f42d223346ae6156eded748cbedb8f386f</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19298736</t>
+          <t>L19692421</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1368,7 +1360,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785962236</t>
+          <t>1785978809</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1378,7 +1370,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>153.846154</t>
+          <t>293.454545</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,27 +1387,23 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xbae8ac7d4c8a6185b820438796f1f9f58ac63f2ed636b3e75be83914f2d44036</t>
+          <t>0x6f6060f620c519fe84b724f15820ae1a59301dcdb13b16825be361e1751a36ef</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.1175</t>
+          <t>1.4425</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1423,11 +1411,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Walsall</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -1435,27 +1419,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Bristol City FC vs Walsall</t>
+          <t>Middlesbrough vs Wrexham</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Bristol City FC</t>
+          <t>Middlesbrough</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Walsall</t>
+          <t>Wrexham</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xc9a261f972b5555c9a1e6c0f33be8eb6a6906d2cda51babdb51dd64314b2c091</t>
+          <t>0xd39b5412e3bdd35c245e5d0a2e08c3b7bbb0dccfab513161aa272b9c72edca35</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19298734</t>
+          <t>L19298910</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1480,17 +1464,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785961563</t>
+          <t>1785971523</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786041900</t>
+          <t>1786129200</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>85.106383</t>
+          <t>2.259887</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1507,7 +1491,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xdd62398a10f567ee5469950797393093a356b40e7fe5930931a6c998d441d9b9</t>
+          <t>0x4da7133bca54b84184238baa7d30b02372340f739df06b943262742640837a0a</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1522,12 +1506,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.195</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1537,7 +1521,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Cheltenham Town</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1547,27 +1531,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Cheltenham Town vs Charlton Athletic</t>
+          <t>AFC Wimbledon vs Newport County</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Cheltenham Town</t>
+          <t>AFC Wimbledon</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Charlton Athletic</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x6bf36843abe397fbc7c233e0ca342729b9cd199b53d9ee9a63b96ac9358c9a1a</t>
+          <t>0xea47b6c120c94ae31f3299be9d23585a5cbf1b0ada4b3059268dd4cc9712b5d8</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19299406</t>
+          <t>L19298736</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1592,17 +1576,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785960783</t>
+          <t>1785962236</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1786214700</t>
+          <t>1786197600</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>15.189873</t>
+          <t>153.846154</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1619,7 +1603,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xcb8aa49e12f3f29aa35ec5b7ff00195594f282ca0db4d0d9be5e2e477b96970d</t>
+          <t>0xbae8ac7d4c8a6185b820438796f1f9f58ac63f2ed636b3e75be83914f2d44036</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1634,7 +1618,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1704,7 +1688,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785960695</t>
+          <t>1785961563</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1714,7 +1698,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>59.574468</t>
+          <t>85.106383</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1731,12 +1715,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x02c4621d6a830534abb9a71c7d2fcc46730afe8d3b686773dfd4c590f2060027</t>
+          <t>0xdd62398a10f567ee5469950797393093a356b40e7fe5930931a6c998d441d9b9</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x204e31304364d2A5f7B90dE28F507adc449Ae221</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1746,22 +1730,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>1.1975</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>AFC Wimbledon -1.5</t>
+          <t>Cheltenham Town</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1771,27 +1755,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>AFC Wimbledon vs Newport County</t>
+          <t>Cheltenham Town vs Charlton Athletic</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>AFC Wimbledon</t>
+          <t>Cheltenham Town</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Charlton Athletic</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x9f1f722832eb2e6381f3a0226a98c406eccc5bd7e76caaaebb931fdda305a642</t>
+          <t>0x6bf36843abe397fbc7c233e0ca342729b9cd199b53d9ee9a63b96ac9358c9a1a</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19298736</t>
+          <t>L19299406</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1816,17 +1800,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785942153</t>
+          <t>1785960783</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1786197600</t>
+          <t>1786214700</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2.941176</t>
+          <t>15.189873</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1843,12 +1827,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xfcba109b300bea480abe542eaa7725c7fec13f0fedc18d9991df424ad450dc90</t>
+          <t>0xcb8aa49e12f3f29aa35ec5b7ff00195594f282ca0db4d0d9be5e2e477b96970d</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x095B1B11E9C470934404Ba7F04da5F79930b2504</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1858,22 +1842,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>14.58</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.1175</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1883,27 +1867,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Bristol City FC vs Walsall</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Bristol City FC</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x30711e53de1ac1c4a025d48c70e4859ee55e52e5e57d10ed46259cc01bb5d46e</t>
+          <t>0xc9a261f972b5555c9a1e6c0f33be8eb6a6906d2cda51babdb51dd64314b2c091</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298734</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1928,17 +1912,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785778500</t>
+          <t>1785960695</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1786041900</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>59.574468</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1955,12 +1939,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x9b63fb9bdb0939e4fa277441c5160ae767a06c0723ae1697f56722a32c1dbbf4</t>
+          <t>0x02c4621d6a830534abb9a71c7d2fcc46730afe8d3b686773dfd4c590f2060027</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x204e31304364d2A5f7B90dE28F507adc449Ae221</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1970,22 +1954,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1.47999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.5762</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>AFC Wimbledon -1.5</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1995,27 +1979,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>AFC Wimbledon vs Newport County</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>AFC Wimbledon</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0x9f1f722832eb2e6381f3a0226a98c406eccc5bd7e76caaaebb931fdda305a642</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298736</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2040,17 +2024,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785751617</t>
+          <t>1785942153</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1786197600</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2.568312</t>
+          <t>2.941176</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2067,31 +2051,39 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x34fd96c52ca66603743b136c029d1196926b8ea965b35ad916e9e624891a3c31</t>
+          <t>0xfcba109b300bea480abe542eaa7725c7fec13f0fedc18d9991df424ad450dc90</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
+          <t>0x095B1B11E9C470934404Ba7F04da5F79930b2504</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2.59999</t>
+          <t>14.58</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.6887</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr"/>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2114,7 +2106,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xb943c3d4cb1b4aebd6296b959eb4168b4f43df52a8043a9e84d184a931ac076c</t>
+          <t>0x30711e53de1ac1c4a025d48c70e4859ee55e52e5e57d10ed46259cc01bb5d46e</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2144,7 +2136,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785751591</t>
+          <t>1785778500</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2154,7 +2146,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>3.77494</t>
+          <t>18.0</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2171,12 +2163,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x92e4361325da8adb7d2c64339dc80666c0b8e0d69bcdd503c9dcdc859b32e858</t>
+          <t>0x9b63fb9bdb0939e4fa277441c5160ae767a06c0723ae1697f56722a32c1dbbf4</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2186,22 +2178,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>288.19</t>
+          <t>1.47999</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.555</t>
+          <t>1.5762</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2226,7 +2218,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2256,7 +2248,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785746436</t>
+          <t>1785751617</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2266,7 +2258,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>519.261261</t>
+          <t>2.568312</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2283,28 +2275,28 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x2f280a5348c67d22f499a879111a6cd14ba32c30651f4b235087504d75fcb720</t>
+          <t>0x34fd96c52ca66603743b136c029d1196926b8ea965b35ad916e9e624891a3c31</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2.59999</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.5263</t>
+          <t>1.6887</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -2330,7 +2322,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
+          <t>0xb943c3d4cb1b4aebd6296b959eb4168b4f43df52a8043a9e84d184a931ac076c</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2360,7 +2352,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785743240</t>
+          <t>1785751591</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2370,7 +2362,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>9.501188</t>
+          <t>3.77494</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2387,36 +2379,44 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xe649643b38b6c14acf9bbbd3214bd63ce98d37feffda0c872c3665293f137b9c</t>
+          <t>0x92e4361325da8adb7d2c64339dc80666c0b8e0d69bcdd503c9dcdc859b32e858</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>288.19</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.3862</t>
+          <t>1.555</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>York City vs Crawley Town</t>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x75d0d882d84fabe75ec0ebfdf953c3267c7e17303f40762904f5aabc9353a5f5</t>
+          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785743239</t>
+          <t>1785746436</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>12.944984</t>
+          <t>519.261261</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2491,7 +2491,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x6da358c7d3a4cfc684658518c8cb0424ee2d0662e048d78a024625d5b4747aed</t>
+          <t>0x2f280a5348c67d22f499a879111a6cd14ba32c30651f4b235087504d75fcb720</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -2538,7 +2538,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2568,7 +2568,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785743239</t>
+          <t>1785743240</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2595,7 +2595,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x22ee20a74b7feafe1f674ddfe8f64eb18b48a4aa83ee151db7142c920e3c6990</t>
+          <t>0xe649643b38b6c14acf9bbbd3214bd63ce98d37feffda0c872c3665293f137b9c</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>EFL Cup</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
+          <t>0x75d0d882d84fabe75ec0ebfdf953c3267c7e17303f40762904f5aabc9353a5f5</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2699,7 +2699,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xe3c6c58c8dab85d1b37033a7121e1d3f4c42a16c31fe969f436aa82e973fe331</t>
+          <t>0x6da358c7d3a4cfc684658518c8cb0424ee2d0662e048d78a024625d5b4747aed</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2710,17 +2710,17 @@
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -2746,7 +2746,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2776,7 +2776,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785743238</t>
+          <t>1785743239</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>17.130621</t>
+          <t>9.501188</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2803,7 +2803,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x67892d913ba613f3f4808f12a89e3a4415421d7988b81f5c03035cac2e9e85b1</t>
+          <t>0x22ee20a74b7feafe1f674ddfe8f64eb18b48a4aa83ee151db7142c920e3c6990</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2814,12 +2814,12 @@
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.445</t>
+          <t>1.3862</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785743238</t>
+          <t>1785743239</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>22.47191</t>
+          <t>12.944984</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2907,7 +2907,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x51e83e15ab97eefc2ccce2074368f96e4d6b2bc474d60fd48cec81194acc78e8</t>
+          <t>0xe3c6c58c8dab85d1b37033a7121e1d3f4c42a16c31fe969f436aa82e973fe331</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2915,11 +2915,7 @@
           <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>10</t>
@@ -2927,19 +2923,15 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.335</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -2962,7 +2954,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x1b7328b49fa63aee1bd67882f5cac5a5686aebcb538af0959dcdd4181c5e2f57</t>
+          <t>0xa673a473011377f0e432cf60301e8ad1da72423bc61634de7bf7db43407a4246</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2992,7 +2984,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785742250</t>
+          <t>1785743238</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3002,7 +2994,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>29.850746</t>
+          <t>17.130621</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3019,7 +3011,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x0e0cffe2676af4f324fc06dde5b8beaeded42b973c319bbf3fb70687f8887f41</t>
+          <t>0x67892d913ba613f3f4808f12a89e3a4415421d7988b81f5c03035cac2e9e85b1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3027,11 +3019,7 @@
           <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>10</t>
@@ -3039,19 +3027,15 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.5587</t>
+          <t>1.445</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -3074,7 +3058,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
+          <t>0x1027436024b118b7583cccaab5c7c410130e0e17447904eb5cefbefb34836df7</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3104,7 +3088,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785742250</t>
+          <t>1785743238</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3114,7 +3098,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>17.897092</t>
+          <t>22.47191</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3131,12 +3115,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xb28bdee5a5bd24b5937965869b7830544160fac83e2df3848790121d4082d3d0</t>
+          <t>0x51e83e15ab97eefc2ccce2074368f96e4d6b2bc474d60fd48cec81194acc78e8</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3146,22 +3130,22 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.335</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3186,7 +3170,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0x1b7328b49fa63aee1bd67882f5cac5a5686aebcb538af0959dcdd4181c5e2f57</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3216,7 +3200,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785741714</t>
+          <t>1785742250</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3226,7 +3210,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>4.020101</t>
+          <t>29.850746</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3243,7 +3227,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0xf27c17a15bfe9521fe22971af3d8cd2a8b3c9955888a401e463346a949eb3345</t>
+          <t>0x0e0cffe2676af4f324fc06dde5b8beaeded42b973c319bbf3fb70687f8887f41</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3263,17 +3247,17 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.4438</t>
+          <t>1.5587</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3298,7 +3282,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x7c21a171d3ea8b89b468e5886d9b7cec062e0e10cc0a3ad080d701f2e478e0d8</t>
+          <t>0x9251e8acd176e46776145df7c8323e80dcd72277ee007f0fa60ecdaa77a19950</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3328,7 +3312,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785740160</t>
+          <t>1785742250</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3338,7 +3322,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>22.535211</t>
+          <t>17.897092</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3355,7 +3339,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
+          <t>0xb28bdee5a5bd24b5937965869b7830544160fac83e2df3848790121d4082d3d0</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3375,7 +3359,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.2475</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3440,7 +3424,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785729810</t>
+          <t>1785741714</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3450,7 +3434,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>4.040404</t>
+          <t>4.020101</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3467,12 +3451,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
+          <t>0xf27c17a15bfe9521fe22971af3d8cd2a8b3c9955888a401e463346a949eb3345</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8AaDb828882f34790D0C35aE0534a6BbDDA6ad19</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3482,22 +3466,22 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>3.99987</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.2488</t>
+          <t>1.4438</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3522,7 +3506,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
+          <t>0x7c21a171d3ea8b89b468e5886d9b7cec062e0e10cc0a3ad080d701f2e478e0d8</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3552,7 +3536,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785729635</t>
+          <t>1785740160</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3562,7 +3546,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>16.079879</t>
+          <t>22.535211</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3579,7 +3563,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
+          <t>0x40b13e9da40eeb7ff88dcf2f7a9105f49a21f846a695e9fa4420be94ee7016fd</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3594,12 +3578,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>23.26</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.4338</t>
+          <t>1.2475</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3619,27 +3603,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3664,17 +3648,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785597225</t>
+          <t>1785729810</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>53.62536</t>
+          <t>4.040404</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3691,7 +3675,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
+          <t>0x66196e60df54d2322e70ce7c61a20cf5ce0d71d5015fa3266e2f3d9a13c435ed</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3706,12 +3690,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3.99987</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.2488</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3721,7 +3705,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3731,27 +3715,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x32518c345846dd6c47978b764fb98cdd69101325ea8828ed514c3e274fb2f43f</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3776,17 +3760,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785595661</t>
+          <t>1785729635</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>3.11284</t>
+          <t>16.079879</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3803,7 +3787,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
+          <t>0x4fa9b312d30771292a7a5ad3c5622749c3bbff9816ffce10029fa7157dc916ea</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3818,12 +3802,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>23.26</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3833,32 +3817,32 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3888,7 +3872,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785594340</t>
+          <t>1785597225</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3898,7 +3882,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>27.777778</t>
+          <t>53.62536</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3915,7 +3899,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
+          <t>0x7a5c40735ecdd2469a0d2ed59e06cf76e82667911a6594d6954897b6ec70b2d1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3930,12 +3914,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -4000,7 +3984,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785593884</t>
+          <t>1785595661</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -4010,7 +3994,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>3.11284</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4027,7 +4011,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
+          <t>0x88c234acb2b6ba6a66f82473bbb6cd2d46b9c9e59cf52a99ce263a54ceecf4eb</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4047,7 +4031,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4112,7 +4096,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785593884</t>
+          <t>1785594340</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4122,7 +4106,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>27.777778</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4139,7 +4123,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
+          <t>0xad72793f41906a56945d290fcef1eab4c8684dad34f06a7b7f2f9149fa6588d1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4154,12 +4138,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>25.04</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.385</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4224,7 +4208,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785593611</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4234,7 +4218,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>65.038961</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4251,7 +4235,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
+          <t>0x9f418c4371bbff74f459e763fa041342287827e644c1f610bc90ca61246b0518</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4266,12 +4250,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.2375</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4281,7 +4265,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -4306,7 +4290,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4336,7 +4320,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785593186</t>
+          <t>1785593884</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4346,7 +4330,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>49.263158</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4363,7 +4347,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
+          <t>0xe2a510a8866a0fccc4b4fc0f5e2eefb5ea80619f77ead0e0412d66449e39d659</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4378,12 +4362,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>25.04</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.385</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4448,7 +4432,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1785592744</t>
+          <t>1785593611</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4458,7 +4442,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>7.088608</t>
+          <t>65.038961</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4475,7 +4459,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
+          <t>0x65d8592e264f1e6ee75586271f168eb30f53f13bdce00905556ffe9a6a34f934</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4490,12 +4474,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>3.59</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.2375</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4505,32 +4489,32 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4560,7 +4544,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785592658</t>
+          <t>1785593186</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4570,7 +4554,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>9.088608</t>
+          <t>49.263158</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4587,7 +4571,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
+          <t>0xfe6919c9dea3cdecf5f7183c2ee249c8757df72dbf1906eaa10524ed4314441f</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4602,7 +4586,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>22.05</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -4672,7 +4656,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1785592637</t>
+          <t>1785592744</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4682,7 +4666,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>55.822785</t>
+          <t>7.088608</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4699,7 +4683,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
+          <t>0x6383957460f589e00702616c9efed479de06c7139221e1d5583f5c10eb193730</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4707,15 +4691,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>36.31948</t>
+          <t>3.59</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4723,7 +4711,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4776,7 +4768,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1785589857</t>
+          <t>1785592658</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4786,7 +4778,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>58.816972</t>
+          <t>9.088608</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4803,7 +4795,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
+          <t>0xbd8076498441ae3b6ea35d5bdf92a3b8c1e0438bd32e8af682830f10700151ba</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4811,15 +4803,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>22.05</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.395</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4827,7 +4823,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
       <c r="H41" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -4880,7 +4880,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1785589600</t>
+          <t>1785592637</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4890,7 +4890,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>6.54251</t>
+          <t>55.822785</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
+          <t>0x4dc533a664201049d6075df64902ddf207ff5e1eb4183a1876ec7ae88303cdfc</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4918,12 +4918,12 @@
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>18.36999</t>
+          <t>36.31948</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.615</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1785589491</t>
+          <t>1785589857</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>29.869902</t>
+          <t>58.816972</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5011,7 +5011,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
+          <t>0x204d81a09f9d3575b3e0f1145019b59d98be2e97cf81685d6cfd0c5bcd97d0e5</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -5022,12 +5022,12 @@
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>18.54999</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1785588508</t>
+          <t>1785589600</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -5098,7 +5098,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>30.597922</t>
+          <t>6.54251</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5115,27 +5115,23 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
+          <t>0x49b7d612371416e922a453ddf757954b2ba5bf87a67c4218eea7367d9e8657ee</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>15.21</t>
+          <t>18.36999</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.615</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -5143,11 +5139,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -5170,7 +5162,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -5200,7 +5192,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1785587700</t>
+          <t>1785589491</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -5210,7 +5202,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>54.08</t>
+          <t>29.869902</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5227,7 +5219,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
+          <t>0x15e4c559a69849435e74cf74008ccc235717ca3e24a588e7b5573d508f1bb611</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5238,12 +5230,12 @@
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>6.44999</t>
+          <t>18.54999</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.7237</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -5274,7 +5266,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -5304,7 +5296,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1785585922</t>
+          <t>1785588508</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -5314,7 +5306,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>8.911903</t>
+          <t>30.597922</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5331,23 +5323,27 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
+          <t>0xf271a9e3deb8f5a5bc5f349c37e800cd6cb885dce7068ad2384a6ac2e7226719</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>3.26</t>
+          <t>15.21</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>1.7212</t>
+          <t>1.2812</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -5355,7 +5351,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H46" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -5408,7 +5408,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>1785579524</t>
+          <t>1785587700</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -5418,7 +5418,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>4.519931</t>
+          <t>54.08</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5435,7 +5435,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
+          <t>0x42b68af80f3c71051db156db7c0a68e1027fae2d571459e0a56bd8df71f10895</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5446,12 +5446,12 @@
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>3.61999</t>
+          <t>6.44999</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1.7212</t>
+          <t>1.7237</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5512,7 +5512,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1785579365</t>
+          <t>1785585922</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>5.01905</t>
+          <t>8.911903</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5539,27 +5539,23 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
+          <t>0x69b8ad7378f32dec64bbaeac971919dd0d8180619506128d1e5063493617cb8a</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>3.26</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5567,26 +5563,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K48" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -5594,7 +5586,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -5624,7 +5616,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>1785577998</t>
+          <t>1785579524</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -5634,7 +5626,7 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>59.143969</t>
+          <t>4.519931</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -5651,27 +5643,23 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
+          <t>0xa805497a7f48ee52efab9785627b0203aab9befd7aaa0be783f233ae3cd59232</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>3.61999</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.7212</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5679,11 +5667,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -5736,7 +5720,7 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>1785577962</t>
+          <t>1785579365</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
@@ -5746,7 +5730,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>82.758621</t>
+          <t>5.01905</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -5763,12 +5747,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
+          <t>0x4b2bc49487f6fb2a3dd7d0ab4d8453dbd5cfa18b5ca58dee45b32f2b7574eafa</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -5778,12 +5762,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>1.3225</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5848,7 +5832,7 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>1785577789</t>
+          <t>1785577998</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
@@ -5858,7 +5842,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>3.534884</t>
+          <t>59.143969</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -5875,12 +5859,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
+          <t>0x9d9f582f85f3f87c606ab39423cd1236096cc37f080cf058bce005cf4e7a3a8e</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -5890,12 +5874,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>18.99909</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5905,24 +5889,24 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
       <c r="K51" t="inlineStr">
         <is>
           <t>Rochdale</t>
@@ -5930,7 +5914,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
+          <t>0x5e62e81a24fb14aeb8c973177b2b77f2762adf2fad4806df4263174fd7f13173</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -5960,7 +5944,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>1785577788</t>
+          <t>1785577962</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -5970,7 +5954,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>59.141136</t>
+          <t>82.758621</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -5987,7 +5971,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
+          <t>0x85a4801a1a1ea2ea89012f58f8eb3562a7ed03f4ecff0b8f931feee05fbb40bd</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6002,12 +5986,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.3225</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6072,7 +6056,7 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785577789</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
@@ -6082,7 +6066,7 @@
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>6.101167</t>
+          <t>3.534884</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -6099,7 +6083,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
+          <t>0xef7346570dc9ff9b1b144424f4df34d06c37c8a3cf40bc70d3feddb6b91c66fa</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6114,12 +6098,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2.81824</t>
+          <t>18.99909</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6184,7 +6168,7 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>1785576753</t>
+          <t>1785577788</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -6194,7 +6178,7 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>8.807</t>
+          <t>59.141136</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -6211,7 +6195,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
+          <t>0xb56b0fc03db0ec5e87106782f22e284962f3607a90ac462ea1260f3472d90f10</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -6226,12 +6210,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>20.06</t>
+          <t>1.96</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6296,7 +6280,7 @@
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>1785576072</t>
+          <t>1785576753</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
@@ -6306,7 +6290,7 @@
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>62.6875</t>
+          <t>6.101167</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -6323,7 +6307,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
+          <t>0xab06e186eb6f94924f38578fbfea69469253011bd9dd9f693335288a9e8d9137</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -6338,7 +6322,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>22.07</t>
+          <t>2.81824</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -6408,7 +6392,7 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>1785575036</t>
+          <t>1785576753</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
@@ -6418,7 +6402,7 @@
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>68.96875</t>
+          <t>8.807</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -6435,7 +6419,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
+          <t>0x4d89df1e5f026abdd36dd618c133402cadfd96305880c597c0ef79333ecf4390</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -6450,7 +6434,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>20.06</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -6520,7 +6504,7 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>1785574569</t>
+          <t>1785576072</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
@@ -6530,7 +6514,7 @@
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>3.625</t>
+          <t>62.6875</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -6547,7 +6531,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
+          <t>0xf25db49e8fc9f2ce6cf3fddab418f63548fce93d96ebc3b47343055c1af9a98c</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -6562,7 +6546,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>19.25059</t>
+          <t>22.07</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -6632,7 +6616,7 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>1785574187</t>
+          <t>1785575036</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
@@ -6642,7 +6626,7 @@
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>60.158094</t>
+          <t>68.96875</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -6659,7 +6643,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
+          <t>0x6d9f9428710ff42266ad95b11037f1cbe6b06820e495aef5f501b3d44fbba800</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -6674,7 +6658,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>20.96</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -6744,7 +6728,7 @@
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785574569</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
@@ -6754,7 +6738,7 @@
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>65.5</t>
+          <t>3.625</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
@@ -6771,7 +6755,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
+          <t>0xa108556fe6e9554cee06c861b695a707b43979ac2dfcad7e19eb09b8c41e5abc</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -6786,7 +6770,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2.69</t>
+          <t>19.25059</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -6856,7 +6840,7 @@
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>1785574186</t>
+          <t>1785574187</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
@@ -6866,7 +6850,7 @@
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>8.40625</t>
+          <t>60.158094</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
@@ -6883,7 +6867,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
+          <t>0x8c8d33c320c7286ce57487f4392c2ac6218366c41db02ef38d125e1528bc6d83</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -6898,7 +6882,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>20.96</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -6968,7 +6952,7 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>1785574073</t>
+          <t>1785574186</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
@@ -6978,7 +6962,7 @@
       </c>
       <c r="T60" t="inlineStr">
         <is>
-          <t>6.90625</t>
+          <t>65.5</t>
         </is>
       </c>
       <c r="U60" t="inlineStr">
@@ -6995,7 +6979,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
+          <t>0x844cab6956497a72bc73fabb7a540ce7db8f2f74cd09984a97d8afb7424400bf</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -7010,7 +6994,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.69</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -7080,7 +7064,7 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>1785573852</t>
+          <t>1785574186</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
@@ -7090,7 +7074,7 @@
       </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>6.25</t>
+          <t>8.40625</t>
         </is>
       </c>
       <c r="U61" t="inlineStr">
@@ -7107,7 +7091,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
+          <t>0xf003621150977b89835af589846044f3e939170630c05a67014e24cea95a22f7</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -7122,12 +7106,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>1.3213</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -7192,7 +7176,7 @@
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>1785570690</t>
+          <t>1785574073</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
@@ -7202,7 +7186,7 @@
       </c>
       <c r="T62" t="inlineStr">
         <is>
-          <t>6.256809</t>
+          <t>6.90625</t>
         </is>
       </c>
       <c r="U62" t="inlineStr">
@@ -7219,7 +7203,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
+          <t>0x4ac1b52add1af7d04b10cd622cc21ebc4d110c9375e328585bac8721fd50ae6d</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -7234,7 +7218,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -7304,7 +7288,7 @@
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>1785570471</t>
+          <t>1785573852</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
@@ -7314,7 +7298,7 @@
       </c>
       <c r="T63" t="inlineStr">
         <is>
-          <t>31.25</t>
+          <t>6.25</t>
         </is>
       </c>
       <c r="U63" t="inlineStr">
@@ -7331,7 +7315,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
+          <t>0x4e13eb060aea33c74ceacea714fc96551e2661bb3ec45a5329f3e627fd8bac79</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -7339,15 +7323,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>19.72999</t>
+          <t>2.01</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>1.6062</t>
+          <t>1.3213</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -7355,7 +7343,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
       <c r="H64" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -7378,7 +7370,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -7408,7 +7400,7 @@
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>1785569792</t>
+          <t>1785570690</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
@@ -7418,7 +7410,7 @@
       </c>
       <c r="T64" t="inlineStr">
         <is>
-          <t>32.544313</t>
+          <t>6.256809</t>
         </is>
       </c>
       <c r="U64" t="inlineStr">
@@ -7435,7 +7427,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
+          <t>0x9ccefc1515ec9e1257b3d0f9f65f808fe1446d77cbc2f9cc0c37554c268e0067</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -7450,7 +7442,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -7520,7 +7512,7 @@
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>1785569076</t>
+          <t>1785570471</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
@@ -7530,7 +7522,7 @@
       </c>
       <c r="T65" t="inlineStr">
         <is>
-          <t>6.59375</t>
+          <t>31.25</t>
         </is>
       </c>
       <c r="U65" t="inlineStr">
@@ -7547,27 +7539,23 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
+          <t>0x764a423b844385f70317e68d948d8de418ed16c80adb98bd7be4b9175056d7fc</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>19.72999</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>1.605</t>
+          <t>1.6062</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -7575,11 +7563,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>York City</t>
-        </is>
-      </c>
+      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
           <t>EFL Cup</t>
@@ -7587,27 +7571,27 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>York City vs Crawley Town</t>
+          <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>L19299060</t>
+          <t>L19298738</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -7632,17 +7616,17 @@
       </c>
       <c r="R66" t="inlineStr">
         <is>
-          <t>1785512959</t>
+          <t>1785569792</t>
         </is>
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1785592800</t>
         </is>
       </c>
       <c r="T66" t="inlineStr">
         <is>
-          <t>1.652893</t>
+          <t>32.544313</t>
         </is>
       </c>
       <c r="U66" t="inlineStr">
@@ -7659,12 +7643,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+          <t>0x44f29cf57c20021e7e7e449174763be6f207e0b02c6b89ddb4920a9bf1321c08</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -7674,12 +7658,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2.51</t>
+          <t>2.11</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -7689,32 +7673,32 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>EFL Cup</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers vs Rochdale</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>Tranmere Rovers</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0xf04eea9a70094c51c5cc3b38ae8e3db134e1352a6837fa48aa53ad083cb80ca6</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -7744,7 +7728,7 @@
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>1785497246</t>
+          <t>1785569076</t>
         </is>
       </c>
       <c r="S67" t="inlineStr">
@@ -7754,7 +7738,7 @@
       </c>
       <c r="T67" t="inlineStr">
         <is>
-          <t>5.97619</t>
+          <t>6.59375</t>
         </is>
       </c>
       <c r="U67" t="inlineStr">
@@ -7771,7 +7755,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+          <t>0x36cf5688604a3ba39fe6b9529067d54c13bfa7ec1b63236e0ec4f1937b6af02c</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -7791,7 +7775,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>1.605</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -7801,7 +7785,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -7811,27 +7795,27 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Tranmere Rovers vs Rochdale</t>
+          <t>York City vs Crawley Town</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+          <t>0x04308ca0f25865eb56bfd580b4513136555071038315ffd87972a7b7d616ec8e</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>L19298738</t>
+          <t>L19299060</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -7856,17 +7840,17 @@
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>1785346230</t>
+          <t>1785512959</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>1785592800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T68" t="inlineStr">
         <is>
-          <t>2.173913</t>
+          <t>1.652893</t>
         </is>
       </c>
       <c r="U68" t="inlineStr">
@@ -7883,110 +7867,334 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
+          <t>0xafadd85041692a6469e14a73163edbf74e19a88c38f0b34d41d3e5d623337052</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>1785497246</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>5.97619</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>0xdfeaf7b051b9d7063f363dd72618d2c0d985c49ee94fdf3ce82ffcac6c9652f3</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>EFL Cup</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers vs Rochdale</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Rochdale</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>L19298738</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>1785346230</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>1785592800</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>2.173913</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
           <t>0xea48d5fe72de69b25067fdb4fdaf1d08ce7262ad75f6855864d3a656da39b313</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B71" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
         <is>
           <t>1.46</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F71" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
+      <c r="G71" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr">
+      <c r="H71" t="inlineStr">
         <is>
           <t>EFL Cup</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr">
+      <c r="I71" t="inlineStr">
         <is>
           <t>Tranmere Rovers vs Rochdale</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr">
+      <c r="J71" t="inlineStr">
         <is>
           <t>Tranmere Rovers</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr">
+      <c r="K71" t="inlineStr">
         <is>
           <t>Rochdale</t>
         </is>
       </c>
-      <c r="L69" t="inlineStr">
+      <c r="L71" t="inlineStr">
         <is>
           <t>0x43a39ce33d7418b38c509663bbe3c399611d27aadbb9e7bc6d02f052fce4d587</t>
         </is>
       </c>
-      <c r="M69" t="inlineStr">
+      <c r="M71" t="inlineStr">
         <is>
           <t>L19298738</t>
         </is>
       </c>
-      <c r="N69" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O69" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P69" t="inlineStr">
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q69" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R69" t="inlineStr">
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
         <is>
           <t>1785345250</t>
         </is>
       </c>
-      <c r="S69" t="inlineStr">
+      <c r="S71" t="inlineStr">
         <is>
           <t>1785592800</t>
         </is>
       </c>
-      <c r="T69" t="inlineStr">
+      <c r="T71" t="inlineStr">
         <is>
           <t>2.173913</t>
         </is>
       </c>
-      <c r="U69" t="inlineStr">
+      <c r="U71" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V69" t="inlineStr">
+      <c r="V71" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-09 00:03:09 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/EFL Cup/trades.xlsx
+++ b/data/sxbet/ligas/EFL Cup/trades.xlsx
@@ -56761,7 +56761,7 @@
       </c>
       <c r="O523" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="P523" t="inlineStr">
@@ -56865,7 +56865,7 @@
       </c>
       <c r="O524" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="P524" t="inlineStr">

</xml_diff>